<commit_message>
refactor: update effective capacity factor to 0.96 (17.28T for Cont 40ft, 4.80T for Xe 5T)
</commit_message>
<xml_diff>
--- a/data/FrostLink_Du_lieu_Chuan.xlsx
+++ b/data/FrostLink_Du_lieu_Chuan.xlsx
@@ -736,7 +736,7 @@
       </c>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>Thực tế - Cont 40ft (18T*0.95)</t>
+          <t>Thực tế - Cont 40ft (18T*0.96)</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>Thực tế - Xe 5T (5T*0.95)</t>
+          <t>Thực tế - Xe 5T (5T*0.96)</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="R2" s="9" t="inlineStr">
         <is>
-          <t>Dự báo - Cont 40ft (18T*0.95)</t>
+          <t>Dự báo - Cont 40ft (18T*0.96)</t>
         </is>
       </c>
       <c r="S2" s="9" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="T2" s="9" t="inlineStr">
         <is>
-          <t>Dự báo - Xe 5T (5T*0.95)</t>
+          <t>Dự báo - Xe 5T (5T*0.96)</t>
         </is>
       </c>
       <c r="U2" s="10" t="inlineStr">
@@ -939,15 +939,15 @@
         </is>
       </c>
       <c r="J3" s="18">
-        <f>INT(H3/(18*0.95))</f>
+        <f>INT(H3/(18*0.96))</f>
         <v/>
       </c>
       <c r="K3" s="18">
-        <f>ROUND(MOD(H3, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H3, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L3" s="18">
-        <f>IF(K3&gt;0, ROUNDUP(K3/(5*0.95), 0), 0)</f>
+        <f>IF(K3&gt;0, ROUNDUP(K3/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M3" s="18">
@@ -971,15 +971,15 @@
         <v/>
       </c>
       <c r="R3" s="18">
-        <f>INT(Q3/(18*0.95))</f>
+        <f>INT(Q3/(18*0.96))</f>
         <v/>
       </c>
       <c r="S3" s="18">
-        <f>ROUND(MOD(Q3, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q3, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T3" s="18">
-        <f>IF(S3&gt;0, ROUNDUP(S3/(5*0.95), 0), 0)</f>
+        <f>IF(S3&gt;0, ROUNDUP(S3/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U3" s="18">
@@ -1101,15 +1101,15 @@
         </is>
       </c>
       <c r="J4" s="18">
-        <f>INT(H4/(18*0.95))</f>
+        <f>INT(H4/(18*0.96))</f>
         <v/>
       </c>
       <c r="K4" s="18">
-        <f>ROUND(MOD(H4, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H4, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L4" s="18">
-        <f>IF(K4&gt;0, ROUNDUP(K4/(5*0.95), 0), 0)</f>
+        <f>IF(K4&gt;0, ROUNDUP(K4/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M4" s="18">
@@ -1133,15 +1133,15 @@
         <v/>
       </c>
       <c r="R4" s="18">
-        <f>INT(Q4/(18*0.95))</f>
+        <f>INT(Q4/(18*0.96))</f>
         <v/>
       </c>
       <c r="S4" s="18">
-        <f>ROUND(MOD(Q4, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q4, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T4" s="18">
-        <f>IF(S4&gt;0, ROUNDUP(S4/(5*0.95), 0), 0)</f>
+        <f>IF(S4&gt;0, ROUNDUP(S4/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U4" s="18">
@@ -1263,15 +1263,15 @@
         </is>
       </c>
       <c r="J5" s="18">
-        <f>INT(H5/(18*0.95))</f>
+        <f>INT(H5/(18*0.96))</f>
         <v/>
       </c>
       <c r="K5" s="18">
-        <f>ROUND(MOD(H5, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H5, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L5" s="18">
-        <f>IF(K5&gt;0, ROUNDUP(K5/(5*0.95), 0), 0)</f>
+        <f>IF(K5&gt;0, ROUNDUP(K5/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M5" s="18">
@@ -1295,15 +1295,15 @@
         <v/>
       </c>
       <c r="R5" s="18">
-        <f>INT(Q5/(18*0.95))</f>
+        <f>INT(Q5/(18*0.96))</f>
         <v/>
       </c>
       <c r="S5" s="18">
-        <f>ROUND(MOD(Q5, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q5, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T5" s="18">
-        <f>IF(S5&gt;0, ROUNDUP(S5/(5*0.95), 0), 0)</f>
+        <f>IF(S5&gt;0, ROUNDUP(S5/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U5" s="18">
@@ -1425,15 +1425,15 @@
         </is>
       </c>
       <c r="J6" s="18">
-        <f>INT(H6/(18*0.95))</f>
+        <f>INT(H6/(18*0.96))</f>
         <v/>
       </c>
       <c r="K6" s="18">
-        <f>ROUND(MOD(H6, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H6, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L6" s="18">
-        <f>IF(K6&gt;0, ROUNDUP(K6/(5*0.95), 0), 0)</f>
+        <f>IF(K6&gt;0, ROUNDUP(K6/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M6" s="18">
@@ -1457,15 +1457,15 @@
         <v/>
       </c>
       <c r="R6" s="18">
-        <f>INT(Q6/(18*0.95))</f>
+        <f>INT(Q6/(18*0.96))</f>
         <v/>
       </c>
       <c r="S6" s="18">
-        <f>ROUND(MOD(Q6, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q6, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T6" s="18">
-        <f>IF(S6&gt;0, ROUNDUP(S6/(5*0.95), 0), 0)</f>
+        <f>IF(S6&gt;0, ROUNDUP(S6/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U6" s="18">
@@ -1593,15 +1593,15 @@
         </is>
       </c>
       <c r="J7" s="18">
-        <f>INT(H7/(18*0.95))</f>
+        <f>INT(H7/(18*0.96))</f>
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>ROUND(MOD(H7, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H7, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>IF(K7&gt;0, ROUNDUP(K7/(5*0.95), 0), 0)</f>
+        <f>IF(K7&gt;0, ROUNDUP(K7/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M7" s="18">
@@ -1625,15 +1625,15 @@
         <v/>
       </c>
       <c r="R7" s="18">
-        <f>INT(Q7/(18*0.95))</f>
+        <f>INT(Q7/(18*0.96))</f>
         <v/>
       </c>
       <c r="S7" s="18">
-        <f>ROUND(MOD(Q7, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q7, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T7" s="18">
-        <f>IF(S7&gt;0, ROUNDUP(S7/(5*0.95), 0), 0)</f>
+        <f>IF(S7&gt;0, ROUNDUP(S7/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U7" s="18">
@@ -1761,15 +1761,15 @@
         </is>
       </c>
       <c r="J8" s="18">
-        <f>INT(H8/(18*0.95))</f>
+        <f>INT(H8/(18*0.96))</f>
         <v/>
       </c>
       <c r="K8" s="18">
-        <f>ROUND(MOD(H8, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H8, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L8" s="18">
-        <f>IF(K8&gt;0, ROUNDUP(K8/(5*0.95), 0), 0)</f>
+        <f>IF(K8&gt;0, ROUNDUP(K8/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M8" s="18">
@@ -1793,15 +1793,15 @@
         <v/>
       </c>
       <c r="R8" s="18">
-        <f>INT(Q8/(18*0.95))</f>
+        <f>INT(Q8/(18*0.96))</f>
         <v/>
       </c>
       <c r="S8" s="18">
-        <f>ROUND(MOD(Q8, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q8, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T8" s="18">
-        <f>IF(S8&gt;0, ROUNDUP(S8/(5*0.95), 0), 0)</f>
+        <f>IF(S8&gt;0, ROUNDUP(S8/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U8" s="18">
@@ -1929,15 +1929,15 @@
         </is>
       </c>
       <c r="J9" s="18">
-        <f>INT(H9/(18*0.95))</f>
+        <f>INT(H9/(18*0.96))</f>
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>ROUND(MOD(H9, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H9, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>IF(K9&gt;0, ROUNDUP(K9/(5*0.95), 0), 0)</f>
+        <f>IF(K9&gt;0, ROUNDUP(K9/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M9" s="18">
@@ -1961,15 +1961,15 @@
         <v/>
       </c>
       <c r="R9" s="18">
-        <f>INT(Q9/(18*0.95))</f>
+        <f>INT(Q9/(18*0.96))</f>
         <v/>
       </c>
       <c r="S9" s="18">
-        <f>ROUND(MOD(Q9, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q9, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T9" s="18">
-        <f>IF(S9&gt;0, ROUNDUP(S9/(5*0.95), 0), 0)</f>
+        <f>IF(S9&gt;0, ROUNDUP(S9/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U9" s="18">
@@ -2097,15 +2097,15 @@
         </is>
       </c>
       <c r="J10" s="18">
-        <f>INT(H10/(18*0.95))</f>
+        <f>INT(H10/(18*0.96))</f>
         <v/>
       </c>
       <c r="K10" s="18">
-        <f>ROUND(MOD(H10, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H10, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L10" s="18">
-        <f>IF(K10&gt;0, ROUNDUP(K10/(5*0.95), 0), 0)</f>
+        <f>IF(K10&gt;0, ROUNDUP(K10/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M10" s="18">
@@ -2129,15 +2129,15 @@
         <v/>
       </c>
       <c r="R10" s="18">
-        <f>INT(Q10/(18*0.95))</f>
+        <f>INT(Q10/(18*0.96))</f>
         <v/>
       </c>
       <c r="S10" s="18">
-        <f>ROUND(MOD(Q10, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q10, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T10" s="18">
-        <f>IF(S10&gt;0, ROUNDUP(S10/(5*0.95), 0), 0)</f>
+        <f>IF(S10&gt;0, ROUNDUP(S10/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U10" s="18">
@@ -2265,15 +2265,15 @@
         </is>
       </c>
       <c r="J11" s="18">
-        <f>INT(H11/(18*0.95))</f>
+        <f>INT(H11/(18*0.96))</f>
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>ROUND(MOD(H11, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H11, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>IF(K11&gt;0, ROUNDUP(K11/(5*0.95), 0), 0)</f>
+        <f>IF(K11&gt;0, ROUNDUP(K11/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M11" s="18">
@@ -2297,15 +2297,15 @@
         <v/>
       </c>
       <c r="R11" s="18">
-        <f>INT(Q11/(18*0.95))</f>
+        <f>INT(Q11/(18*0.96))</f>
         <v/>
       </c>
       <c r="S11" s="18">
-        <f>ROUND(MOD(Q11, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q11, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T11" s="18">
-        <f>IF(S11&gt;0, ROUNDUP(S11/(5*0.95), 0), 0)</f>
+        <f>IF(S11&gt;0, ROUNDUP(S11/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U11" s="18">
@@ -2433,15 +2433,15 @@
         </is>
       </c>
       <c r="J12" s="18">
-        <f>INT(H12/(18*0.95))</f>
+        <f>INT(H12/(18*0.96))</f>
         <v/>
       </c>
       <c r="K12" s="18">
-        <f>ROUND(MOD(H12, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H12, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L12" s="18">
-        <f>IF(K12&gt;0, ROUNDUP(K12/(5*0.95), 0), 0)</f>
+        <f>IF(K12&gt;0, ROUNDUP(K12/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M12" s="18">
@@ -2465,15 +2465,15 @@
         <v/>
       </c>
       <c r="R12" s="18">
-        <f>INT(Q12/(18*0.95))</f>
+        <f>INT(Q12/(18*0.96))</f>
         <v/>
       </c>
       <c r="S12" s="18">
-        <f>ROUND(MOD(Q12, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q12, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T12" s="18">
-        <f>IF(S12&gt;0, ROUNDUP(S12/(5*0.95), 0), 0)</f>
+        <f>IF(S12&gt;0, ROUNDUP(S12/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U12" s="18">
@@ -2601,15 +2601,15 @@
         </is>
       </c>
       <c r="J13" s="18">
-        <f>INT(H13/(18*0.95))</f>
+        <f>INT(H13/(18*0.96))</f>
         <v/>
       </c>
       <c r="K13" s="18">
-        <f>ROUND(MOD(H13, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H13, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>IF(K13&gt;0, ROUNDUP(K13/(5*0.95), 0), 0)</f>
+        <f>IF(K13&gt;0, ROUNDUP(K13/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M13" s="18">
@@ -2633,15 +2633,15 @@
         <v/>
       </c>
       <c r="R13" s="18">
-        <f>INT(Q13/(18*0.95))</f>
+        <f>INT(Q13/(18*0.96))</f>
         <v/>
       </c>
       <c r="S13" s="18">
-        <f>ROUND(MOD(Q13, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q13, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T13" s="18">
-        <f>IF(S13&gt;0, ROUNDUP(S13/(5*0.95), 0), 0)</f>
+        <f>IF(S13&gt;0, ROUNDUP(S13/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U13" s="18">
@@ -2769,15 +2769,15 @@
         </is>
       </c>
       <c r="J14" s="18">
-        <f>INT(H14/(18*0.95))</f>
+        <f>INT(H14/(18*0.96))</f>
         <v/>
       </c>
       <c r="K14" s="18">
-        <f>ROUND(MOD(H14, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H14, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L14" s="18">
-        <f>IF(K14&gt;0, ROUNDUP(K14/(5*0.95), 0), 0)</f>
+        <f>IF(K14&gt;0, ROUNDUP(K14/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M14" s="18">
@@ -2801,15 +2801,15 @@
         <v/>
       </c>
       <c r="R14" s="18">
-        <f>INT(Q14/(18*0.95))</f>
+        <f>INT(Q14/(18*0.96))</f>
         <v/>
       </c>
       <c r="S14" s="18">
-        <f>ROUND(MOD(Q14, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q14, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T14" s="18">
-        <f>IF(S14&gt;0, ROUNDUP(S14/(5*0.95), 0), 0)</f>
+        <f>IF(S14&gt;0, ROUNDUP(S14/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U14" s="18">
@@ -2937,15 +2937,15 @@
         </is>
       </c>
       <c r="J15" s="18">
-        <f>INT(H15/(18*0.95))</f>
+        <f>INT(H15/(18*0.96))</f>
         <v/>
       </c>
       <c r="K15" s="18">
-        <f>ROUND(MOD(H15, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H15, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>IF(K15&gt;0, ROUNDUP(K15/(5*0.95), 0), 0)</f>
+        <f>IF(K15&gt;0, ROUNDUP(K15/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M15" s="18">
@@ -2969,15 +2969,15 @@
         <v/>
       </c>
       <c r="R15" s="18">
-        <f>INT(Q15/(18*0.95))</f>
+        <f>INT(Q15/(18*0.96))</f>
         <v/>
       </c>
       <c r="S15" s="18">
-        <f>ROUND(MOD(Q15, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q15, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T15" s="18">
-        <f>IF(S15&gt;0, ROUNDUP(S15/(5*0.95), 0), 0)</f>
+        <f>IF(S15&gt;0, ROUNDUP(S15/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U15" s="18">
@@ -3105,15 +3105,15 @@
         </is>
       </c>
       <c r="J16" s="18">
-        <f>INT(H16/(18*0.95))</f>
+        <f>INT(H16/(18*0.96))</f>
         <v/>
       </c>
       <c r="K16" s="18">
-        <f>ROUND(MOD(H16, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H16, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L16" s="18">
-        <f>IF(K16&gt;0, ROUNDUP(K16/(5*0.95), 0), 0)</f>
+        <f>IF(K16&gt;0, ROUNDUP(K16/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M16" s="18">
@@ -3137,15 +3137,15 @@
         <v/>
       </c>
       <c r="R16" s="18">
-        <f>INT(Q16/(18*0.95))</f>
+        <f>INT(Q16/(18*0.96))</f>
         <v/>
       </c>
       <c r="S16" s="18">
-        <f>ROUND(MOD(Q16, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q16, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T16" s="18">
-        <f>IF(S16&gt;0, ROUNDUP(S16/(5*0.95), 0), 0)</f>
+        <f>IF(S16&gt;0, ROUNDUP(S16/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U16" s="18">
@@ -3273,15 +3273,15 @@
         </is>
       </c>
       <c r="J17" s="18">
-        <f>INT(H17/(18*0.95))</f>
+        <f>INT(H17/(18*0.96))</f>
         <v/>
       </c>
       <c r="K17" s="18">
-        <f>ROUND(MOD(H17, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H17, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>IF(K17&gt;0, ROUNDUP(K17/(5*0.95), 0), 0)</f>
+        <f>IF(K17&gt;0, ROUNDUP(K17/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M17" s="18">
@@ -3305,15 +3305,15 @@
         <v/>
       </c>
       <c r="R17" s="18">
-        <f>INT(Q17/(18*0.95))</f>
+        <f>INT(Q17/(18*0.96))</f>
         <v/>
       </c>
       <c r="S17" s="18">
-        <f>ROUND(MOD(Q17, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q17, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T17" s="18">
-        <f>IF(S17&gt;0, ROUNDUP(S17/(5*0.95), 0), 0)</f>
+        <f>IF(S17&gt;0, ROUNDUP(S17/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U17" s="18">
@@ -3441,15 +3441,15 @@
         </is>
       </c>
       <c r="J18" s="18">
-        <f>INT(H18/(18*0.95))</f>
+        <f>INT(H18/(18*0.96))</f>
         <v/>
       </c>
       <c r="K18" s="18">
-        <f>ROUND(MOD(H18, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H18, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L18" s="18">
-        <f>IF(K18&gt;0, ROUNDUP(K18/(5*0.95), 0), 0)</f>
+        <f>IF(K18&gt;0, ROUNDUP(K18/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M18" s="18">
@@ -3473,15 +3473,15 @@
         <v/>
       </c>
       <c r="R18" s="18">
-        <f>INT(Q18/(18*0.95))</f>
+        <f>INT(Q18/(18*0.96))</f>
         <v/>
       </c>
       <c r="S18" s="18">
-        <f>ROUND(MOD(Q18, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q18, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T18" s="18">
-        <f>IF(S18&gt;0, ROUNDUP(S18/(5*0.95), 0), 0)</f>
+        <f>IF(S18&gt;0, ROUNDUP(S18/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U18" s="18">
@@ -3609,15 +3609,15 @@
         </is>
       </c>
       <c r="J19" s="18">
-        <f>INT(H19/(18*0.95))</f>
+        <f>INT(H19/(18*0.96))</f>
         <v/>
       </c>
       <c r="K19" s="18">
-        <f>ROUND(MOD(H19, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H19, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>IF(K19&gt;0, ROUNDUP(K19/(5*0.95), 0), 0)</f>
+        <f>IF(K19&gt;0, ROUNDUP(K19/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M19" s="18">
@@ -3641,15 +3641,15 @@
         <v/>
       </c>
       <c r="R19" s="18">
-        <f>INT(Q19/(18*0.95))</f>
+        <f>INT(Q19/(18*0.96))</f>
         <v/>
       </c>
       <c r="S19" s="18">
-        <f>ROUND(MOD(Q19, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q19, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T19" s="18">
-        <f>IF(S19&gt;0, ROUNDUP(S19/(5*0.95), 0), 0)</f>
+        <f>IF(S19&gt;0, ROUNDUP(S19/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U19" s="18">
@@ -3777,15 +3777,15 @@
         </is>
       </c>
       <c r="J20" s="18">
-        <f>INT(H20/(18*0.95))</f>
+        <f>INT(H20/(18*0.96))</f>
         <v/>
       </c>
       <c r="K20" s="18">
-        <f>ROUND(MOD(H20, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H20, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L20" s="18">
-        <f>IF(K20&gt;0, ROUNDUP(K20/(5*0.95), 0), 0)</f>
+        <f>IF(K20&gt;0, ROUNDUP(K20/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M20" s="18">
@@ -3809,15 +3809,15 @@
         <v/>
       </c>
       <c r="R20" s="18">
-        <f>INT(Q20/(18*0.95))</f>
+        <f>INT(Q20/(18*0.96))</f>
         <v/>
       </c>
       <c r="S20" s="18">
-        <f>ROUND(MOD(Q20, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q20, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T20" s="18">
-        <f>IF(S20&gt;0, ROUNDUP(S20/(5*0.95), 0), 0)</f>
+        <f>IF(S20&gt;0, ROUNDUP(S20/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U20" s="18">
@@ -3945,15 +3945,15 @@
         </is>
       </c>
       <c r="J21" s="18">
-        <f>INT(H21/(18*0.95))</f>
+        <f>INT(H21/(18*0.96))</f>
         <v/>
       </c>
       <c r="K21" s="18">
-        <f>ROUND(MOD(H21, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H21, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L21" s="18">
-        <f>IF(K21&gt;0, ROUNDUP(K21/(5*0.95), 0), 0)</f>
+        <f>IF(K21&gt;0, ROUNDUP(K21/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M21" s="18">
@@ -3977,15 +3977,15 @@
         <v/>
       </c>
       <c r="R21" s="18">
-        <f>INT(Q21/(18*0.95))</f>
+        <f>INT(Q21/(18*0.96))</f>
         <v/>
       </c>
       <c r="S21" s="18">
-        <f>ROUND(MOD(Q21, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q21, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T21" s="18">
-        <f>IF(S21&gt;0, ROUNDUP(S21/(5*0.95), 0), 0)</f>
+        <f>IF(S21&gt;0, ROUNDUP(S21/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U21" s="18">
@@ -4113,15 +4113,15 @@
         </is>
       </c>
       <c r="J22" s="18">
-        <f>INT(H22/(18*0.95))</f>
+        <f>INT(H22/(18*0.96))</f>
         <v/>
       </c>
       <c r="K22" s="18">
-        <f>ROUND(MOD(H22, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H22, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L22" s="18">
-        <f>IF(K22&gt;0, ROUNDUP(K22/(5*0.95), 0), 0)</f>
+        <f>IF(K22&gt;0, ROUNDUP(K22/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M22" s="18">
@@ -4145,15 +4145,15 @@
         <v/>
       </c>
       <c r="R22" s="18">
-        <f>INT(Q22/(18*0.95))</f>
+        <f>INT(Q22/(18*0.96))</f>
         <v/>
       </c>
       <c r="S22" s="18">
-        <f>ROUND(MOD(Q22, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q22, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T22" s="18">
-        <f>IF(S22&gt;0, ROUNDUP(S22/(5*0.95), 0), 0)</f>
+        <f>IF(S22&gt;0, ROUNDUP(S22/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U22" s="18">
@@ -4281,15 +4281,15 @@
         </is>
       </c>
       <c r="J23" s="18">
-        <f>INT(H23/(18*0.95))</f>
+        <f>INT(H23/(18*0.96))</f>
         <v/>
       </c>
       <c r="K23" s="18">
-        <f>ROUND(MOD(H23, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H23, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L23" s="18">
-        <f>IF(K23&gt;0, ROUNDUP(K23/(5*0.95), 0), 0)</f>
+        <f>IF(K23&gt;0, ROUNDUP(K23/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M23" s="18">
@@ -4313,15 +4313,15 @@
         <v/>
       </c>
       <c r="R23" s="18">
-        <f>INT(Q23/(18*0.95))</f>
+        <f>INT(Q23/(18*0.96))</f>
         <v/>
       </c>
       <c r="S23" s="18">
-        <f>ROUND(MOD(Q23, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q23, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T23" s="18">
-        <f>IF(S23&gt;0, ROUNDUP(S23/(5*0.95), 0), 0)</f>
+        <f>IF(S23&gt;0, ROUNDUP(S23/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U23" s="18">
@@ -4449,15 +4449,15 @@
         </is>
       </c>
       <c r="J24" s="18">
-        <f>INT(H24/(18*0.95))</f>
+        <f>INT(H24/(18*0.96))</f>
         <v/>
       </c>
       <c r="K24" s="18">
-        <f>ROUND(MOD(H24, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H24, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L24" s="18">
-        <f>IF(K24&gt;0, ROUNDUP(K24/(5*0.95), 0), 0)</f>
+        <f>IF(K24&gt;0, ROUNDUP(K24/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M24" s="18">
@@ -4481,15 +4481,15 @@
         <v/>
       </c>
       <c r="R24" s="18">
-        <f>INT(Q24/(18*0.95))</f>
+        <f>INT(Q24/(18*0.96))</f>
         <v/>
       </c>
       <c r="S24" s="18">
-        <f>ROUND(MOD(Q24, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q24, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T24" s="18">
-        <f>IF(S24&gt;0, ROUNDUP(S24/(5*0.95), 0), 0)</f>
+        <f>IF(S24&gt;0, ROUNDUP(S24/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U24" s="18">
@@ -4617,15 +4617,15 @@
         </is>
       </c>
       <c r="J25" s="18">
-        <f>INT(H25/(18*0.95))</f>
+        <f>INT(H25/(18*0.96))</f>
         <v/>
       </c>
       <c r="K25" s="18">
-        <f>ROUND(MOD(H25, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H25, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L25" s="18">
-        <f>IF(K25&gt;0, ROUNDUP(K25/(5*0.95), 0), 0)</f>
+        <f>IF(K25&gt;0, ROUNDUP(K25/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M25" s="18">
@@ -4649,15 +4649,15 @@
         <v/>
       </c>
       <c r="R25" s="18">
-        <f>INT(Q25/(18*0.95))</f>
+        <f>INT(Q25/(18*0.96))</f>
         <v/>
       </c>
       <c r="S25" s="18">
-        <f>ROUND(MOD(Q25, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q25, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T25" s="18">
-        <f>IF(S25&gt;0, ROUNDUP(S25/(5*0.95), 0), 0)</f>
+        <f>IF(S25&gt;0, ROUNDUP(S25/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U25" s="18">
@@ -4785,15 +4785,15 @@
         </is>
       </c>
       <c r="J26" s="18">
-        <f>INT(H26/(18*0.95))</f>
+        <f>INT(H26/(18*0.96))</f>
         <v/>
       </c>
       <c r="K26" s="18">
-        <f>ROUND(MOD(H26, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H26, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L26" s="18">
-        <f>IF(K26&gt;0, ROUNDUP(K26/(5*0.95), 0), 0)</f>
+        <f>IF(K26&gt;0, ROUNDUP(K26/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M26" s="18">
@@ -4817,15 +4817,15 @@
         <v/>
       </c>
       <c r="R26" s="18">
-        <f>INT(Q26/(18*0.95))</f>
+        <f>INT(Q26/(18*0.96))</f>
         <v/>
       </c>
       <c r="S26" s="18">
-        <f>ROUND(MOD(Q26, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q26, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T26" s="18">
-        <f>IF(S26&gt;0, ROUNDUP(S26/(5*0.95), 0), 0)</f>
+        <f>IF(S26&gt;0, ROUNDUP(S26/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U26" s="18">
@@ -4953,15 +4953,15 @@
         </is>
       </c>
       <c r="J27" s="18">
-        <f>INT(H27/(18*0.95))</f>
+        <f>INT(H27/(18*0.96))</f>
         <v/>
       </c>
       <c r="K27" s="18">
-        <f>ROUND(MOD(H27, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H27, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L27" s="18">
-        <f>IF(K27&gt;0, ROUNDUP(K27/(5*0.95), 0), 0)</f>
+        <f>IF(K27&gt;0, ROUNDUP(K27/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M27" s="18">
@@ -4985,15 +4985,15 @@
         <v/>
       </c>
       <c r="R27" s="18">
-        <f>INT(Q27/(18*0.95))</f>
+        <f>INT(Q27/(18*0.96))</f>
         <v/>
       </c>
       <c r="S27" s="18">
-        <f>ROUND(MOD(Q27, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q27, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T27" s="18">
-        <f>IF(S27&gt;0, ROUNDUP(S27/(5*0.95), 0), 0)</f>
+        <f>IF(S27&gt;0, ROUNDUP(S27/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U27" s="18">
@@ -5121,15 +5121,15 @@
         </is>
       </c>
       <c r="J28" s="18">
-        <f>INT(H28/(18*0.95))</f>
+        <f>INT(H28/(18*0.96))</f>
         <v/>
       </c>
       <c r="K28" s="18">
-        <f>ROUND(MOD(H28, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H28, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L28" s="18">
-        <f>IF(K28&gt;0, ROUNDUP(K28/(5*0.95), 0), 0)</f>
+        <f>IF(K28&gt;0, ROUNDUP(K28/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M28" s="18">
@@ -5153,15 +5153,15 @@
         <v/>
       </c>
       <c r="R28" s="18">
-        <f>INT(Q28/(18*0.95))</f>
+        <f>INT(Q28/(18*0.96))</f>
         <v/>
       </c>
       <c r="S28" s="18">
-        <f>ROUND(MOD(Q28, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q28, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T28" s="18">
-        <f>IF(S28&gt;0, ROUNDUP(S28/(5*0.95), 0), 0)</f>
+        <f>IF(S28&gt;0, ROUNDUP(S28/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U28" s="18">
@@ -5289,15 +5289,15 @@
         </is>
       </c>
       <c r="J29" s="18">
-        <f>INT(H29/(18*0.95))</f>
+        <f>INT(H29/(18*0.96))</f>
         <v/>
       </c>
       <c r="K29" s="18">
-        <f>ROUND(MOD(H29, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H29, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L29" s="18">
-        <f>IF(K29&gt;0, ROUNDUP(K29/(5*0.95), 0), 0)</f>
+        <f>IF(K29&gt;0, ROUNDUP(K29/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M29" s="18">
@@ -5321,15 +5321,15 @@
         <v/>
       </c>
       <c r="R29" s="18">
-        <f>INT(Q29/(18*0.95))</f>
+        <f>INT(Q29/(18*0.96))</f>
         <v/>
       </c>
       <c r="S29" s="18">
-        <f>ROUND(MOD(Q29, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q29, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T29" s="18">
-        <f>IF(S29&gt;0, ROUNDUP(S29/(5*0.95), 0), 0)</f>
+        <f>IF(S29&gt;0, ROUNDUP(S29/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U29" s="18">
@@ -5457,15 +5457,15 @@
         </is>
       </c>
       <c r="J30" s="18">
-        <f>INT(H30/(18*0.95))</f>
+        <f>INT(H30/(18*0.96))</f>
         <v/>
       </c>
       <c r="K30" s="18">
-        <f>ROUND(MOD(H30, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H30, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L30" s="18">
-        <f>IF(K30&gt;0, ROUNDUP(K30/(5*0.95), 0), 0)</f>
+        <f>IF(K30&gt;0, ROUNDUP(K30/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M30" s="18">
@@ -5489,15 +5489,15 @@
         <v/>
       </c>
       <c r="R30" s="18">
-        <f>INT(Q30/(18*0.95))</f>
+        <f>INT(Q30/(18*0.96))</f>
         <v/>
       </c>
       <c r="S30" s="18">
-        <f>ROUND(MOD(Q30, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q30, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T30" s="18">
-        <f>IF(S30&gt;0, ROUNDUP(S30/(5*0.95), 0), 0)</f>
+        <f>IF(S30&gt;0, ROUNDUP(S30/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U30" s="18">
@@ -5625,15 +5625,15 @@
         </is>
       </c>
       <c r="J31" s="18">
-        <f>INT(H31/(18*0.95))</f>
+        <f>INT(H31/(18*0.96))</f>
         <v/>
       </c>
       <c r="K31" s="18">
-        <f>ROUND(MOD(H31, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H31, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L31" s="18">
-        <f>IF(K31&gt;0, ROUNDUP(K31/(5*0.95), 0), 0)</f>
+        <f>IF(K31&gt;0, ROUNDUP(K31/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M31" s="18">
@@ -5657,15 +5657,15 @@
         <v/>
       </c>
       <c r="R31" s="18">
-        <f>INT(Q31/(18*0.95))</f>
+        <f>INT(Q31/(18*0.96))</f>
         <v/>
       </c>
       <c r="S31" s="18">
-        <f>ROUND(MOD(Q31, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q31, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T31" s="18">
-        <f>IF(S31&gt;0, ROUNDUP(S31/(5*0.95), 0), 0)</f>
+        <f>IF(S31&gt;0, ROUNDUP(S31/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U31" s="18">
@@ -5793,15 +5793,15 @@
         </is>
       </c>
       <c r="J32" s="18">
-        <f>INT(H32/(18*0.95))</f>
+        <f>INT(H32/(18*0.96))</f>
         <v/>
       </c>
       <c r="K32" s="18">
-        <f>ROUND(MOD(H32, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H32, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L32" s="18">
-        <f>IF(K32&gt;0, ROUNDUP(K32/(5*0.95), 0), 0)</f>
+        <f>IF(K32&gt;0, ROUNDUP(K32/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M32" s="18">
@@ -5825,15 +5825,15 @@
         <v/>
       </c>
       <c r="R32" s="18">
-        <f>INT(Q32/(18*0.95))</f>
+        <f>INT(Q32/(18*0.96))</f>
         <v/>
       </c>
       <c r="S32" s="18">
-        <f>ROUND(MOD(Q32, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q32, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T32" s="18">
-        <f>IF(S32&gt;0, ROUNDUP(S32/(5*0.95), 0), 0)</f>
+        <f>IF(S32&gt;0, ROUNDUP(S32/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U32" s="18">
@@ -5961,15 +5961,15 @@
         </is>
       </c>
       <c r="J33" s="18">
-        <f>INT(H33/(18*0.95))</f>
+        <f>INT(H33/(18*0.96))</f>
         <v/>
       </c>
       <c r="K33" s="18">
-        <f>ROUND(MOD(H33, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H33, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L33" s="18">
-        <f>IF(K33&gt;0, ROUNDUP(K33/(5*0.95), 0), 0)</f>
+        <f>IF(K33&gt;0, ROUNDUP(K33/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M33" s="18">
@@ -5993,15 +5993,15 @@
         <v/>
       </c>
       <c r="R33" s="18">
-        <f>INT(Q33/(18*0.95))</f>
+        <f>INT(Q33/(18*0.96))</f>
         <v/>
       </c>
       <c r="S33" s="18">
-        <f>ROUND(MOD(Q33, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q33, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T33" s="18">
-        <f>IF(S33&gt;0, ROUNDUP(S33/(5*0.95), 0), 0)</f>
+        <f>IF(S33&gt;0, ROUNDUP(S33/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U33" s="18">
@@ -6129,15 +6129,15 @@
         </is>
       </c>
       <c r="J34" s="18">
-        <f>INT(H34/(18*0.95))</f>
+        <f>INT(H34/(18*0.96))</f>
         <v/>
       </c>
       <c r="K34" s="18">
-        <f>ROUND(MOD(H34, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H34, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L34" s="18">
-        <f>IF(K34&gt;0, ROUNDUP(K34/(5*0.95), 0), 0)</f>
+        <f>IF(K34&gt;0, ROUNDUP(K34/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M34" s="18">
@@ -6161,15 +6161,15 @@
         <v/>
       </c>
       <c r="R34" s="18">
-        <f>INT(Q34/(18*0.95))</f>
+        <f>INT(Q34/(18*0.96))</f>
         <v/>
       </c>
       <c r="S34" s="18">
-        <f>ROUND(MOD(Q34, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q34, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T34" s="18">
-        <f>IF(S34&gt;0, ROUNDUP(S34/(5*0.95), 0), 0)</f>
+        <f>IF(S34&gt;0, ROUNDUP(S34/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U34" s="18">
@@ -6297,15 +6297,15 @@
         </is>
       </c>
       <c r="J35" s="18">
-        <f>INT(H35/(18*0.95))</f>
+        <f>INT(H35/(18*0.96))</f>
         <v/>
       </c>
       <c r="K35" s="18">
-        <f>ROUND(MOD(H35, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H35, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L35" s="18">
-        <f>IF(K35&gt;0, ROUNDUP(K35/(5*0.95), 0), 0)</f>
+        <f>IF(K35&gt;0, ROUNDUP(K35/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M35" s="18">
@@ -6329,15 +6329,15 @@
         <v/>
       </c>
       <c r="R35" s="18">
-        <f>INT(Q35/(18*0.95))</f>
+        <f>INT(Q35/(18*0.96))</f>
         <v/>
       </c>
       <c r="S35" s="18">
-        <f>ROUND(MOD(Q35, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q35, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T35" s="18">
-        <f>IF(S35&gt;0, ROUNDUP(S35/(5*0.95), 0), 0)</f>
+        <f>IF(S35&gt;0, ROUNDUP(S35/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U35" s="18">
@@ -6465,15 +6465,15 @@
         </is>
       </c>
       <c r="J36" s="18">
-        <f>INT(H36/(18*0.95))</f>
+        <f>INT(H36/(18*0.96))</f>
         <v/>
       </c>
       <c r="K36" s="18">
-        <f>ROUND(MOD(H36, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H36, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L36" s="18">
-        <f>IF(K36&gt;0, ROUNDUP(K36/(5*0.95), 0), 0)</f>
+        <f>IF(K36&gt;0, ROUNDUP(K36/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M36" s="18">
@@ -6497,15 +6497,15 @@
         <v/>
       </c>
       <c r="R36" s="18">
-        <f>INT(Q36/(18*0.95))</f>
+        <f>INT(Q36/(18*0.96))</f>
         <v/>
       </c>
       <c r="S36" s="18">
-        <f>ROUND(MOD(Q36, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q36, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T36" s="18">
-        <f>IF(S36&gt;0, ROUNDUP(S36/(5*0.95), 0), 0)</f>
+        <f>IF(S36&gt;0, ROUNDUP(S36/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U36" s="18">
@@ -6633,15 +6633,15 @@
         </is>
       </c>
       <c r="J37" s="18">
-        <f>INT(H37/(18*0.95))</f>
+        <f>INT(H37/(18*0.96))</f>
         <v/>
       </c>
       <c r="K37" s="18">
-        <f>ROUND(MOD(H37, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H37, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L37" s="18">
-        <f>IF(K37&gt;0, ROUNDUP(K37/(5*0.95), 0), 0)</f>
+        <f>IF(K37&gt;0, ROUNDUP(K37/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M37" s="18">
@@ -6665,15 +6665,15 @@
         <v/>
       </c>
       <c r="R37" s="18">
-        <f>INT(Q37/(18*0.95))</f>
+        <f>INT(Q37/(18*0.96))</f>
         <v/>
       </c>
       <c r="S37" s="18">
-        <f>ROUND(MOD(Q37, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q37, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T37" s="18">
-        <f>IF(S37&gt;0, ROUNDUP(S37/(5*0.95), 0), 0)</f>
+        <f>IF(S37&gt;0, ROUNDUP(S37/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U37" s="18">
@@ -6801,15 +6801,15 @@
         </is>
       </c>
       <c r="J38" s="18">
-        <f>INT(H38/(18*0.95))</f>
+        <f>INT(H38/(18*0.96))</f>
         <v/>
       </c>
       <c r="K38" s="18">
-        <f>ROUND(MOD(H38, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H38, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L38" s="18">
-        <f>IF(K38&gt;0, ROUNDUP(K38/(5*0.95), 0), 0)</f>
+        <f>IF(K38&gt;0, ROUNDUP(K38/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M38" s="18">
@@ -6833,15 +6833,15 @@
         <v/>
       </c>
       <c r="R38" s="18">
-        <f>INT(Q38/(18*0.95))</f>
+        <f>INT(Q38/(18*0.96))</f>
         <v/>
       </c>
       <c r="S38" s="18">
-        <f>ROUND(MOD(Q38, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q38, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T38" s="18">
-        <f>IF(S38&gt;0, ROUNDUP(S38/(5*0.95), 0), 0)</f>
+        <f>IF(S38&gt;0, ROUNDUP(S38/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U38" s="18">
@@ -6969,15 +6969,15 @@
         </is>
       </c>
       <c r="J39" s="18">
-        <f>INT(H39/(18*0.95))</f>
+        <f>INT(H39/(18*0.96))</f>
         <v/>
       </c>
       <c r="K39" s="18">
-        <f>ROUND(MOD(H39, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H39, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L39" s="18">
-        <f>IF(K39&gt;0, ROUNDUP(K39/(5*0.95), 0), 0)</f>
+        <f>IF(K39&gt;0, ROUNDUP(K39/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M39" s="18">
@@ -7001,15 +7001,15 @@
         <v/>
       </c>
       <c r="R39" s="18">
-        <f>INT(Q39/(18*0.95))</f>
+        <f>INT(Q39/(18*0.96))</f>
         <v/>
       </c>
       <c r="S39" s="18">
-        <f>ROUND(MOD(Q39, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q39, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T39" s="18">
-        <f>IF(S39&gt;0, ROUNDUP(S39/(5*0.95), 0), 0)</f>
+        <f>IF(S39&gt;0, ROUNDUP(S39/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U39" s="18">
@@ -7137,15 +7137,15 @@
         </is>
       </c>
       <c r="J40" s="18">
-        <f>INT(H40/(18*0.95))</f>
+        <f>INT(H40/(18*0.96))</f>
         <v/>
       </c>
       <c r="K40" s="18">
-        <f>ROUND(MOD(H40, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H40, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L40" s="18">
-        <f>IF(K40&gt;0, ROUNDUP(K40/(5*0.95), 0), 0)</f>
+        <f>IF(K40&gt;0, ROUNDUP(K40/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M40" s="18">
@@ -7169,15 +7169,15 @@
         <v/>
       </c>
       <c r="R40" s="18">
-        <f>INT(Q40/(18*0.95))</f>
+        <f>INT(Q40/(18*0.96))</f>
         <v/>
       </c>
       <c r="S40" s="18">
-        <f>ROUND(MOD(Q40, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q40, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T40" s="18">
-        <f>IF(S40&gt;0, ROUNDUP(S40/(5*0.95), 0), 0)</f>
+        <f>IF(S40&gt;0, ROUNDUP(S40/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U40" s="18">
@@ -7305,15 +7305,15 @@
         </is>
       </c>
       <c r="J41" s="18">
-        <f>INT(H41/(18*0.95))</f>
+        <f>INT(H41/(18*0.96))</f>
         <v/>
       </c>
       <c r="K41" s="18">
-        <f>ROUND(MOD(H41, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H41, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L41" s="18">
-        <f>IF(K41&gt;0, ROUNDUP(K41/(5*0.95), 0), 0)</f>
+        <f>IF(K41&gt;0, ROUNDUP(K41/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M41" s="18">
@@ -7337,15 +7337,15 @@
         <v/>
       </c>
       <c r="R41" s="18">
-        <f>INT(Q41/(18*0.95))</f>
+        <f>INT(Q41/(18*0.96))</f>
         <v/>
       </c>
       <c r="S41" s="18">
-        <f>ROUND(MOD(Q41, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q41, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T41" s="18">
-        <f>IF(S41&gt;0, ROUNDUP(S41/(5*0.95), 0), 0)</f>
+        <f>IF(S41&gt;0, ROUNDUP(S41/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U41" s="18">
@@ -7473,15 +7473,15 @@
         </is>
       </c>
       <c r="J42" s="18">
-        <f>INT(H42/(18*0.95))</f>
+        <f>INT(H42/(18*0.96))</f>
         <v/>
       </c>
       <c r="K42" s="18">
-        <f>ROUND(MOD(H42, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H42, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L42" s="18">
-        <f>IF(K42&gt;0, ROUNDUP(K42/(5*0.95), 0), 0)</f>
+        <f>IF(K42&gt;0, ROUNDUP(K42/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M42" s="18">
@@ -7505,15 +7505,15 @@
         <v/>
       </c>
       <c r="R42" s="18">
-        <f>INT(Q42/(18*0.95))</f>
+        <f>INT(Q42/(18*0.96))</f>
         <v/>
       </c>
       <c r="S42" s="18">
-        <f>ROUND(MOD(Q42, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q42, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T42" s="18">
-        <f>IF(S42&gt;0, ROUNDUP(S42/(5*0.95), 0), 0)</f>
+        <f>IF(S42&gt;0, ROUNDUP(S42/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U42" s="18">
@@ -7641,15 +7641,15 @@
         </is>
       </c>
       <c r="J43" s="18">
-        <f>INT(H43/(18*0.95))</f>
+        <f>INT(H43/(18*0.96))</f>
         <v/>
       </c>
       <c r="K43" s="18">
-        <f>ROUND(MOD(H43, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H43, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L43" s="18">
-        <f>IF(K43&gt;0, ROUNDUP(K43/(5*0.95), 0), 0)</f>
+        <f>IF(K43&gt;0, ROUNDUP(K43/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M43" s="18">
@@ -7673,15 +7673,15 @@
         <v/>
       </c>
       <c r="R43" s="18">
-        <f>INT(Q43/(18*0.95))</f>
+        <f>INT(Q43/(18*0.96))</f>
         <v/>
       </c>
       <c r="S43" s="18">
-        <f>ROUND(MOD(Q43, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q43, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T43" s="18">
-        <f>IF(S43&gt;0, ROUNDUP(S43/(5*0.95), 0), 0)</f>
+        <f>IF(S43&gt;0, ROUNDUP(S43/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U43" s="18">
@@ -7809,15 +7809,15 @@
         </is>
       </c>
       <c r="J44" s="18">
-        <f>INT(H44/(18*0.95))</f>
+        <f>INT(H44/(18*0.96))</f>
         <v/>
       </c>
       <c r="K44" s="18">
-        <f>ROUND(MOD(H44, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H44, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L44" s="18">
-        <f>IF(K44&gt;0, ROUNDUP(K44/(5*0.95), 0), 0)</f>
+        <f>IF(K44&gt;0, ROUNDUP(K44/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M44" s="18">
@@ -7841,15 +7841,15 @@
         <v/>
       </c>
       <c r="R44" s="18">
-        <f>INT(Q44/(18*0.95))</f>
+        <f>INT(Q44/(18*0.96))</f>
         <v/>
       </c>
       <c r="S44" s="18">
-        <f>ROUND(MOD(Q44, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q44, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T44" s="18">
-        <f>IF(S44&gt;0, ROUNDUP(S44/(5*0.95), 0), 0)</f>
+        <f>IF(S44&gt;0, ROUNDUP(S44/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U44" s="18">
@@ -7977,15 +7977,15 @@
         </is>
       </c>
       <c r="J45" s="18">
-        <f>INT(H45/(18*0.95))</f>
+        <f>INT(H45/(18*0.96))</f>
         <v/>
       </c>
       <c r="K45" s="18">
-        <f>ROUND(MOD(H45, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H45, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L45" s="18">
-        <f>IF(K45&gt;0, ROUNDUP(K45/(5*0.95), 0), 0)</f>
+        <f>IF(K45&gt;0, ROUNDUP(K45/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M45" s="18">
@@ -8009,15 +8009,15 @@
         <v/>
       </c>
       <c r="R45" s="18">
-        <f>INT(Q45/(18*0.95))</f>
+        <f>INT(Q45/(18*0.96))</f>
         <v/>
       </c>
       <c r="S45" s="18">
-        <f>ROUND(MOD(Q45, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q45, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T45" s="18">
-        <f>IF(S45&gt;0, ROUNDUP(S45/(5*0.95), 0), 0)</f>
+        <f>IF(S45&gt;0, ROUNDUP(S45/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U45" s="18">
@@ -8145,15 +8145,15 @@
         </is>
       </c>
       <c r="J46" s="18">
-        <f>INT(H46/(18*0.95))</f>
+        <f>INT(H46/(18*0.96))</f>
         <v/>
       </c>
       <c r="K46" s="18">
-        <f>ROUND(MOD(H46, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H46, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L46" s="18">
-        <f>IF(K46&gt;0, ROUNDUP(K46/(5*0.95), 0), 0)</f>
+        <f>IF(K46&gt;0, ROUNDUP(K46/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M46" s="18">
@@ -8177,15 +8177,15 @@
         <v/>
       </c>
       <c r="R46" s="18">
-        <f>INT(Q46/(18*0.95))</f>
+        <f>INT(Q46/(18*0.96))</f>
         <v/>
       </c>
       <c r="S46" s="18">
-        <f>ROUND(MOD(Q46, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q46, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T46" s="18">
-        <f>IF(S46&gt;0, ROUNDUP(S46/(5*0.95), 0), 0)</f>
+        <f>IF(S46&gt;0, ROUNDUP(S46/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U46" s="18">
@@ -8313,15 +8313,15 @@
         </is>
       </c>
       <c r="J47" s="18">
-        <f>INT(H47/(18*0.95))</f>
+        <f>INT(H47/(18*0.96))</f>
         <v/>
       </c>
       <c r="K47" s="18">
-        <f>ROUND(MOD(H47, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H47, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L47" s="18">
-        <f>IF(K47&gt;0, ROUNDUP(K47/(5*0.95), 0), 0)</f>
+        <f>IF(K47&gt;0, ROUNDUP(K47/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M47" s="18">
@@ -8345,15 +8345,15 @@
         <v/>
       </c>
       <c r="R47" s="18">
-        <f>INT(Q47/(18*0.95))</f>
+        <f>INT(Q47/(18*0.96))</f>
         <v/>
       </c>
       <c r="S47" s="18">
-        <f>ROUND(MOD(Q47, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q47, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T47" s="18">
-        <f>IF(S47&gt;0, ROUNDUP(S47/(5*0.95), 0), 0)</f>
+        <f>IF(S47&gt;0, ROUNDUP(S47/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U47" s="18">
@@ -8481,15 +8481,15 @@
         </is>
       </c>
       <c r="J48" s="18">
-        <f>INT(H48/(18*0.95))</f>
+        <f>INT(H48/(18*0.96))</f>
         <v/>
       </c>
       <c r="K48" s="18">
-        <f>ROUND(MOD(H48, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H48, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L48" s="18">
-        <f>IF(K48&gt;0, ROUNDUP(K48/(5*0.95), 0), 0)</f>
+        <f>IF(K48&gt;0, ROUNDUP(K48/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M48" s="18">
@@ -8513,15 +8513,15 @@
         <v/>
       </c>
       <c r="R48" s="18">
-        <f>INT(Q48/(18*0.95))</f>
+        <f>INT(Q48/(18*0.96))</f>
         <v/>
       </c>
       <c r="S48" s="18">
-        <f>ROUND(MOD(Q48, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q48, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T48" s="18">
-        <f>IF(S48&gt;0, ROUNDUP(S48/(5*0.95), 0), 0)</f>
+        <f>IF(S48&gt;0, ROUNDUP(S48/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U48" s="18">
@@ -8649,15 +8649,15 @@
         </is>
       </c>
       <c r="J49" s="18">
-        <f>INT(H49/(18*0.95))</f>
+        <f>INT(H49/(18*0.96))</f>
         <v/>
       </c>
       <c r="K49" s="18">
-        <f>ROUND(MOD(H49, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H49, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L49" s="18">
-        <f>IF(K49&gt;0, ROUNDUP(K49/(5*0.95), 0), 0)</f>
+        <f>IF(K49&gt;0, ROUNDUP(K49/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M49" s="18">
@@ -8681,15 +8681,15 @@
         <v/>
       </c>
       <c r="R49" s="18">
-        <f>INT(Q49/(18*0.95))</f>
+        <f>INT(Q49/(18*0.96))</f>
         <v/>
       </c>
       <c r="S49" s="18">
-        <f>ROUND(MOD(Q49, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q49, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T49" s="18">
-        <f>IF(S49&gt;0, ROUNDUP(S49/(5*0.95), 0), 0)</f>
+        <f>IF(S49&gt;0, ROUNDUP(S49/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U49" s="18">
@@ -8817,15 +8817,15 @@
         </is>
       </c>
       <c r="J50" s="18">
-        <f>INT(H50/(18*0.95))</f>
+        <f>INT(H50/(18*0.96))</f>
         <v/>
       </c>
       <c r="K50" s="18">
-        <f>ROUND(MOD(H50, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H50, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L50" s="18">
-        <f>IF(K50&gt;0, ROUNDUP(K50/(5*0.95), 0), 0)</f>
+        <f>IF(K50&gt;0, ROUNDUP(K50/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M50" s="18">
@@ -8849,15 +8849,15 @@
         <v/>
       </c>
       <c r="R50" s="18">
-        <f>INT(Q50/(18*0.95))</f>
+        <f>INT(Q50/(18*0.96))</f>
         <v/>
       </c>
       <c r="S50" s="18">
-        <f>ROUND(MOD(Q50, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q50, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T50" s="18">
-        <f>IF(S50&gt;0, ROUNDUP(S50/(5*0.95), 0), 0)</f>
+        <f>IF(S50&gt;0, ROUNDUP(S50/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U50" s="18">
@@ -8985,15 +8985,15 @@
         </is>
       </c>
       <c r="J51" s="18">
-        <f>INT(H51/(18*0.95))</f>
+        <f>INT(H51/(18*0.96))</f>
         <v/>
       </c>
       <c r="K51" s="18">
-        <f>ROUND(MOD(H51, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H51, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L51" s="18">
-        <f>IF(K51&gt;0, ROUNDUP(K51/(5*0.95), 0), 0)</f>
+        <f>IF(K51&gt;0, ROUNDUP(K51/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M51" s="18">
@@ -9017,15 +9017,15 @@
         <v/>
       </c>
       <c r="R51" s="18">
-        <f>INT(Q51/(18*0.95))</f>
+        <f>INT(Q51/(18*0.96))</f>
         <v/>
       </c>
       <c r="S51" s="18">
-        <f>ROUND(MOD(Q51, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q51, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T51" s="18">
-        <f>IF(S51&gt;0, ROUNDUP(S51/(5*0.95), 0), 0)</f>
+        <f>IF(S51&gt;0, ROUNDUP(S51/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U51" s="18">
@@ -9153,15 +9153,15 @@
         </is>
       </c>
       <c r="J52" s="18">
-        <f>INT(H52/(18*0.95))</f>
+        <f>INT(H52/(18*0.96))</f>
         <v/>
       </c>
       <c r="K52" s="18">
-        <f>ROUND(MOD(H52, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H52, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L52" s="18">
-        <f>IF(K52&gt;0, ROUNDUP(K52/(5*0.95), 0), 0)</f>
+        <f>IF(K52&gt;0, ROUNDUP(K52/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M52" s="18">
@@ -9185,15 +9185,15 @@
         <v/>
       </c>
       <c r="R52" s="18">
-        <f>INT(Q52/(18*0.95))</f>
+        <f>INT(Q52/(18*0.96))</f>
         <v/>
       </c>
       <c r="S52" s="18">
-        <f>ROUND(MOD(Q52, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q52, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T52" s="18">
-        <f>IF(S52&gt;0, ROUNDUP(S52/(5*0.95), 0), 0)</f>
+        <f>IF(S52&gt;0, ROUNDUP(S52/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U52" s="18">
@@ -9321,15 +9321,15 @@
         </is>
       </c>
       <c r="J53" s="18">
-        <f>INT(H53/(18*0.95))</f>
+        <f>INT(H53/(18*0.96))</f>
         <v/>
       </c>
       <c r="K53" s="18">
-        <f>ROUND(MOD(H53, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H53, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L53" s="18">
-        <f>IF(K53&gt;0, ROUNDUP(K53/(5*0.95), 0), 0)</f>
+        <f>IF(K53&gt;0, ROUNDUP(K53/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M53" s="18">
@@ -9353,15 +9353,15 @@
         <v/>
       </c>
       <c r="R53" s="18">
-        <f>INT(Q53/(18*0.95))</f>
+        <f>INT(Q53/(18*0.96))</f>
         <v/>
       </c>
       <c r="S53" s="18">
-        <f>ROUND(MOD(Q53, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q53, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T53" s="18">
-        <f>IF(S53&gt;0, ROUNDUP(S53/(5*0.95), 0), 0)</f>
+        <f>IF(S53&gt;0, ROUNDUP(S53/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U53" s="18">
@@ -9489,15 +9489,15 @@
         </is>
       </c>
       <c r="J54" s="18">
-        <f>INT(H54/(18*0.95))</f>
+        <f>INT(H54/(18*0.96))</f>
         <v/>
       </c>
       <c r="K54" s="18">
-        <f>ROUND(MOD(H54, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H54, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L54" s="18">
-        <f>IF(K54&gt;0, ROUNDUP(K54/(5*0.95), 0), 0)</f>
+        <f>IF(K54&gt;0, ROUNDUP(K54/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M54" s="18">
@@ -9521,15 +9521,15 @@
         <v/>
       </c>
       <c r="R54" s="18">
-        <f>INT(Q54/(18*0.95))</f>
+        <f>INT(Q54/(18*0.96))</f>
         <v/>
       </c>
       <c r="S54" s="18">
-        <f>ROUND(MOD(Q54, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q54, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T54" s="18">
-        <f>IF(S54&gt;0, ROUNDUP(S54/(5*0.95), 0), 0)</f>
+        <f>IF(S54&gt;0, ROUNDUP(S54/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U54" s="18">
@@ -9657,15 +9657,15 @@
         </is>
       </c>
       <c r="J55" s="18">
-        <f>INT(H55/(18*0.95))</f>
+        <f>INT(H55/(18*0.96))</f>
         <v/>
       </c>
       <c r="K55" s="18">
-        <f>ROUND(MOD(H55, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H55, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L55" s="18">
-        <f>IF(K55&gt;0, ROUNDUP(K55/(5*0.95), 0), 0)</f>
+        <f>IF(K55&gt;0, ROUNDUP(K55/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M55" s="18">
@@ -9689,15 +9689,15 @@
         <v/>
       </c>
       <c r="R55" s="18">
-        <f>INT(Q55/(18*0.95))</f>
+        <f>INT(Q55/(18*0.96))</f>
         <v/>
       </c>
       <c r="S55" s="18">
-        <f>ROUND(MOD(Q55, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q55, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T55" s="18">
-        <f>IF(S55&gt;0, ROUNDUP(S55/(5*0.95), 0), 0)</f>
+        <f>IF(S55&gt;0, ROUNDUP(S55/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U55" s="18">
@@ -9825,15 +9825,15 @@
         </is>
       </c>
       <c r="J56" s="18">
-        <f>INT(H56/(18*0.95))</f>
+        <f>INT(H56/(18*0.96))</f>
         <v/>
       </c>
       <c r="K56" s="18">
-        <f>ROUND(MOD(H56, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H56, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L56" s="18">
-        <f>IF(K56&gt;0, ROUNDUP(K56/(5*0.95), 0), 0)</f>
+        <f>IF(K56&gt;0, ROUNDUP(K56/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M56" s="18">
@@ -9857,15 +9857,15 @@
         <v/>
       </c>
       <c r="R56" s="18">
-        <f>INT(Q56/(18*0.95))</f>
+        <f>INT(Q56/(18*0.96))</f>
         <v/>
       </c>
       <c r="S56" s="18">
-        <f>ROUND(MOD(Q56, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q56, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T56" s="18">
-        <f>IF(S56&gt;0, ROUNDUP(S56/(5*0.95), 0), 0)</f>
+        <f>IF(S56&gt;0, ROUNDUP(S56/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U56" s="18">
@@ -9993,15 +9993,15 @@
         </is>
       </c>
       <c r="J57" s="18">
-        <f>INT(H57/(18*0.95))</f>
+        <f>INT(H57/(18*0.96))</f>
         <v/>
       </c>
       <c r="K57" s="18">
-        <f>ROUND(MOD(H57, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H57, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L57" s="18">
-        <f>IF(K57&gt;0, ROUNDUP(K57/(5*0.95), 0), 0)</f>
+        <f>IF(K57&gt;0, ROUNDUP(K57/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M57" s="18">
@@ -10025,15 +10025,15 @@
         <v/>
       </c>
       <c r="R57" s="18">
-        <f>INT(Q57/(18*0.95))</f>
+        <f>INT(Q57/(18*0.96))</f>
         <v/>
       </c>
       <c r="S57" s="18">
-        <f>ROUND(MOD(Q57, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q57, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T57" s="18">
-        <f>IF(S57&gt;0, ROUNDUP(S57/(5*0.95), 0), 0)</f>
+        <f>IF(S57&gt;0, ROUNDUP(S57/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U57" s="18">
@@ -10161,15 +10161,15 @@
         </is>
       </c>
       <c r="J58" s="18">
-        <f>INT(H58/(18*0.95))</f>
+        <f>INT(H58/(18*0.96))</f>
         <v/>
       </c>
       <c r="K58" s="18">
-        <f>ROUND(MOD(H58, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H58, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L58" s="18">
-        <f>IF(K58&gt;0, ROUNDUP(K58/(5*0.95), 0), 0)</f>
+        <f>IF(K58&gt;0, ROUNDUP(K58/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M58" s="18">
@@ -10193,15 +10193,15 @@
         <v/>
       </c>
       <c r="R58" s="18">
-        <f>INT(Q58/(18*0.95))</f>
+        <f>INT(Q58/(18*0.96))</f>
         <v/>
       </c>
       <c r="S58" s="18">
-        <f>ROUND(MOD(Q58, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q58, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T58" s="18">
-        <f>IF(S58&gt;0, ROUNDUP(S58/(5*0.95), 0), 0)</f>
+        <f>IF(S58&gt;0, ROUNDUP(S58/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U58" s="18">
@@ -10329,15 +10329,15 @@
         </is>
       </c>
       <c r="J59" s="18">
-        <f>INT(H59/(18*0.95))</f>
+        <f>INT(H59/(18*0.96))</f>
         <v/>
       </c>
       <c r="K59" s="18">
-        <f>ROUND(MOD(H59, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H59, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L59" s="18">
-        <f>IF(K59&gt;0, ROUNDUP(K59/(5*0.95), 0), 0)</f>
+        <f>IF(K59&gt;0, ROUNDUP(K59/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M59" s="18">
@@ -10361,15 +10361,15 @@
         <v/>
       </c>
       <c r="R59" s="18">
-        <f>INT(Q59/(18*0.95))</f>
+        <f>INT(Q59/(18*0.96))</f>
         <v/>
       </c>
       <c r="S59" s="18">
-        <f>ROUND(MOD(Q59, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q59, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T59" s="18">
-        <f>IF(S59&gt;0, ROUNDUP(S59/(5*0.95), 0), 0)</f>
+        <f>IF(S59&gt;0, ROUNDUP(S59/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U59" s="18">
@@ -10497,15 +10497,15 @@
         </is>
       </c>
       <c r="J60" s="18">
-        <f>INT(H60/(18*0.95))</f>
+        <f>INT(H60/(18*0.96))</f>
         <v/>
       </c>
       <c r="K60" s="18">
-        <f>ROUND(MOD(H60, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H60, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L60" s="18">
-        <f>IF(K60&gt;0, ROUNDUP(K60/(5*0.95), 0), 0)</f>
+        <f>IF(K60&gt;0, ROUNDUP(K60/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M60" s="18">
@@ -10529,15 +10529,15 @@
         <v/>
       </c>
       <c r="R60" s="18">
-        <f>INT(Q60/(18*0.95))</f>
+        <f>INT(Q60/(18*0.96))</f>
         <v/>
       </c>
       <c r="S60" s="18">
-        <f>ROUND(MOD(Q60, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q60, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T60" s="18">
-        <f>IF(S60&gt;0, ROUNDUP(S60/(5*0.95), 0), 0)</f>
+        <f>IF(S60&gt;0, ROUNDUP(S60/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U60" s="18">
@@ -10665,15 +10665,15 @@
         </is>
       </c>
       <c r="J61" s="18">
-        <f>INT(H61/(18*0.95))</f>
+        <f>INT(H61/(18*0.96))</f>
         <v/>
       </c>
       <c r="K61" s="18">
-        <f>ROUND(MOD(H61, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H61, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L61" s="18">
-        <f>IF(K61&gt;0, ROUNDUP(K61/(5*0.95), 0), 0)</f>
+        <f>IF(K61&gt;0, ROUNDUP(K61/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M61" s="18">
@@ -10697,15 +10697,15 @@
         <v/>
       </c>
       <c r="R61" s="18">
-        <f>INT(Q61/(18*0.95))</f>
+        <f>INT(Q61/(18*0.96))</f>
         <v/>
       </c>
       <c r="S61" s="18">
-        <f>ROUND(MOD(Q61, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q61, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T61" s="18">
-        <f>IF(S61&gt;0, ROUNDUP(S61/(5*0.95), 0), 0)</f>
+        <f>IF(S61&gt;0, ROUNDUP(S61/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U61" s="18">
@@ -10833,15 +10833,15 @@
         </is>
       </c>
       <c r="J62" s="18">
-        <f>INT(H62/(18*0.95))</f>
+        <f>INT(H62/(18*0.96))</f>
         <v/>
       </c>
       <c r="K62" s="18">
-        <f>ROUND(MOD(H62, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H62, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L62" s="18">
-        <f>IF(K62&gt;0, ROUNDUP(K62/(5*0.95), 0), 0)</f>
+        <f>IF(K62&gt;0, ROUNDUP(K62/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M62" s="18">
@@ -10865,15 +10865,15 @@
         <v/>
       </c>
       <c r="R62" s="18">
-        <f>INT(Q62/(18*0.95))</f>
+        <f>INT(Q62/(18*0.96))</f>
         <v/>
       </c>
       <c r="S62" s="18">
-        <f>ROUND(MOD(Q62, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q62, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T62" s="18">
-        <f>IF(S62&gt;0, ROUNDUP(S62/(5*0.95), 0), 0)</f>
+        <f>IF(S62&gt;0, ROUNDUP(S62/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U62" s="18">
@@ -11001,15 +11001,15 @@
         </is>
       </c>
       <c r="J63" s="18">
-        <f>INT(H63/(18*0.95))</f>
+        <f>INT(H63/(18*0.96))</f>
         <v/>
       </c>
       <c r="K63" s="18">
-        <f>ROUND(MOD(H63, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H63, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L63" s="18">
-        <f>IF(K63&gt;0, ROUNDUP(K63/(5*0.95), 0), 0)</f>
+        <f>IF(K63&gt;0, ROUNDUP(K63/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M63" s="18">
@@ -11033,15 +11033,15 @@
         <v/>
       </c>
       <c r="R63" s="18">
-        <f>INT(Q63/(18*0.95))</f>
+        <f>INT(Q63/(18*0.96))</f>
         <v/>
       </c>
       <c r="S63" s="18">
-        <f>ROUND(MOD(Q63, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q63, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T63" s="18">
-        <f>IF(S63&gt;0, ROUNDUP(S63/(5*0.95), 0), 0)</f>
+        <f>IF(S63&gt;0, ROUNDUP(S63/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U63" s="18">
@@ -11169,15 +11169,15 @@
         </is>
       </c>
       <c r="J64" s="18">
-        <f>INT(H64/(18*0.95))</f>
+        <f>INT(H64/(18*0.96))</f>
         <v/>
       </c>
       <c r="K64" s="18">
-        <f>ROUND(MOD(H64, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H64, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L64" s="18">
-        <f>IF(K64&gt;0, ROUNDUP(K64/(5*0.95), 0), 0)</f>
+        <f>IF(K64&gt;0, ROUNDUP(K64/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M64" s="18">
@@ -11201,15 +11201,15 @@
         <v/>
       </c>
       <c r="R64" s="18">
-        <f>INT(Q64/(18*0.95))</f>
+        <f>INT(Q64/(18*0.96))</f>
         <v/>
       </c>
       <c r="S64" s="18">
-        <f>ROUND(MOD(Q64, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q64, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T64" s="18">
-        <f>IF(S64&gt;0, ROUNDUP(S64/(5*0.95), 0), 0)</f>
+        <f>IF(S64&gt;0, ROUNDUP(S64/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U64" s="18">
@@ -11337,15 +11337,15 @@
         </is>
       </c>
       <c r="J65" s="18">
-        <f>INT(H65/(18*0.95))</f>
+        <f>INT(H65/(18*0.96))</f>
         <v/>
       </c>
       <c r="K65" s="18">
-        <f>ROUND(MOD(H65, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H65, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L65" s="18">
-        <f>IF(K65&gt;0, ROUNDUP(K65/(5*0.95), 0), 0)</f>
+        <f>IF(K65&gt;0, ROUNDUP(K65/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M65" s="18">
@@ -11369,15 +11369,15 @@
         <v/>
       </c>
       <c r="R65" s="18">
-        <f>INT(Q65/(18*0.95))</f>
+        <f>INT(Q65/(18*0.96))</f>
         <v/>
       </c>
       <c r="S65" s="18">
-        <f>ROUND(MOD(Q65, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q65, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T65" s="18">
-        <f>IF(S65&gt;0, ROUNDUP(S65/(5*0.95), 0), 0)</f>
+        <f>IF(S65&gt;0, ROUNDUP(S65/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U65" s="18">
@@ -11505,15 +11505,15 @@
         </is>
       </c>
       <c r="J66" s="18">
-        <f>INT(H66/(18*0.95))</f>
+        <f>INT(H66/(18*0.96))</f>
         <v/>
       </c>
       <c r="K66" s="18">
-        <f>ROUND(MOD(H66, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H66, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L66" s="18">
-        <f>IF(K66&gt;0, ROUNDUP(K66/(5*0.95), 0), 0)</f>
+        <f>IF(K66&gt;0, ROUNDUP(K66/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M66" s="18">
@@ -11537,15 +11537,15 @@
         <v/>
       </c>
       <c r="R66" s="18">
-        <f>INT(Q66/(18*0.95))</f>
+        <f>INT(Q66/(18*0.96))</f>
         <v/>
       </c>
       <c r="S66" s="18">
-        <f>ROUND(MOD(Q66, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q66, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T66" s="18">
-        <f>IF(S66&gt;0, ROUNDUP(S66/(5*0.95), 0), 0)</f>
+        <f>IF(S66&gt;0, ROUNDUP(S66/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U66" s="18">
@@ -11673,15 +11673,15 @@
         </is>
       </c>
       <c r="J67" s="18">
-        <f>INT(H67/(18*0.95))</f>
+        <f>INT(H67/(18*0.96))</f>
         <v/>
       </c>
       <c r="K67" s="18">
-        <f>ROUND(MOD(H67, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H67, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L67" s="18">
-        <f>IF(K67&gt;0, ROUNDUP(K67/(5*0.95), 0), 0)</f>
+        <f>IF(K67&gt;0, ROUNDUP(K67/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M67" s="18">
@@ -11705,15 +11705,15 @@
         <v/>
       </c>
       <c r="R67" s="18">
-        <f>INT(Q67/(18*0.95))</f>
+        <f>INT(Q67/(18*0.96))</f>
         <v/>
       </c>
       <c r="S67" s="18">
-        <f>ROUND(MOD(Q67, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q67, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T67" s="18">
-        <f>IF(S67&gt;0, ROUNDUP(S67/(5*0.95), 0), 0)</f>
+        <f>IF(S67&gt;0, ROUNDUP(S67/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U67" s="18">
@@ -11841,15 +11841,15 @@
         </is>
       </c>
       <c r="J68" s="18">
-        <f>INT(H68/(18*0.95))</f>
+        <f>INT(H68/(18*0.96))</f>
         <v/>
       </c>
       <c r="K68" s="18">
-        <f>ROUND(MOD(H68, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H68, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L68" s="18">
-        <f>IF(K68&gt;0, ROUNDUP(K68/(5*0.95), 0), 0)</f>
+        <f>IF(K68&gt;0, ROUNDUP(K68/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M68" s="18">
@@ -11873,15 +11873,15 @@
         <v/>
       </c>
       <c r="R68" s="18">
-        <f>INT(Q68/(18*0.95))</f>
+        <f>INT(Q68/(18*0.96))</f>
         <v/>
       </c>
       <c r="S68" s="18">
-        <f>ROUND(MOD(Q68, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q68, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T68" s="18">
-        <f>IF(S68&gt;0, ROUNDUP(S68/(5*0.95), 0), 0)</f>
+        <f>IF(S68&gt;0, ROUNDUP(S68/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U68" s="18">
@@ -12009,15 +12009,15 @@
         </is>
       </c>
       <c r="J69" s="18">
-        <f>INT(H69/(18*0.95))</f>
+        <f>INT(H69/(18*0.96))</f>
         <v/>
       </c>
       <c r="K69" s="18">
-        <f>ROUND(MOD(H69, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H69, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L69" s="18">
-        <f>IF(K69&gt;0, ROUNDUP(K69/(5*0.95), 0), 0)</f>
+        <f>IF(K69&gt;0, ROUNDUP(K69/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M69" s="18">
@@ -12041,15 +12041,15 @@
         <v/>
       </c>
       <c r="R69" s="18">
-        <f>INT(Q69/(18*0.95))</f>
+        <f>INT(Q69/(18*0.96))</f>
         <v/>
       </c>
       <c r="S69" s="18">
-        <f>ROUND(MOD(Q69, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q69, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T69" s="18">
-        <f>IF(S69&gt;0, ROUNDUP(S69/(5*0.95), 0), 0)</f>
+        <f>IF(S69&gt;0, ROUNDUP(S69/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U69" s="18">
@@ -12177,15 +12177,15 @@
         </is>
       </c>
       <c r="J70" s="18">
-        <f>INT(H70/(18*0.95))</f>
+        <f>INT(H70/(18*0.96))</f>
         <v/>
       </c>
       <c r="K70" s="18">
-        <f>ROUND(MOD(H70, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H70, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L70" s="18">
-        <f>IF(K70&gt;0, ROUNDUP(K70/(5*0.95), 0), 0)</f>
+        <f>IF(K70&gt;0, ROUNDUP(K70/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M70" s="18">
@@ -12209,15 +12209,15 @@
         <v/>
       </c>
       <c r="R70" s="18">
-        <f>INT(Q70/(18*0.95))</f>
+        <f>INT(Q70/(18*0.96))</f>
         <v/>
       </c>
       <c r="S70" s="18">
-        <f>ROUND(MOD(Q70, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q70, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T70" s="18">
-        <f>IF(S70&gt;0, ROUNDUP(S70/(5*0.95), 0), 0)</f>
+        <f>IF(S70&gt;0, ROUNDUP(S70/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U70" s="18">
@@ -12345,15 +12345,15 @@
         </is>
       </c>
       <c r="J71" s="18">
-        <f>INT(H71/(18*0.95))</f>
+        <f>INT(H71/(18*0.96))</f>
         <v/>
       </c>
       <c r="K71" s="18">
-        <f>ROUND(MOD(H71, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H71, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L71" s="18">
-        <f>IF(K71&gt;0, ROUNDUP(K71/(5*0.95), 0), 0)</f>
+        <f>IF(K71&gt;0, ROUNDUP(K71/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M71" s="18">
@@ -12377,15 +12377,15 @@
         <v/>
       </c>
       <c r="R71" s="18">
-        <f>INT(Q71/(18*0.95))</f>
+        <f>INT(Q71/(18*0.96))</f>
         <v/>
       </c>
       <c r="S71" s="18">
-        <f>ROUND(MOD(Q71, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q71, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T71" s="18">
-        <f>IF(S71&gt;0, ROUNDUP(S71/(5*0.95), 0), 0)</f>
+        <f>IF(S71&gt;0, ROUNDUP(S71/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U71" s="18">
@@ -12513,15 +12513,15 @@
         </is>
       </c>
       <c r="J72" s="18">
-        <f>INT(H72/(18*0.95))</f>
+        <f>INT(H72/(18*0.96))</f>
         <v/>
       </c>
       <c r="K72" s="18">
-        <f>ROUND(MOD(H72, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H72, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L72" s="18">
-        <f>IF(K72&gt;0, ROUNDUP(K72/(5*0.95), 0), 0)</f>
+        <f>IF(K72&gt;0, ROUNDUP(K72/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M72" s="18">
@@ -12545,15 +12545,15 @@
         <v/>
       </c>
       <c r="R72" s="18">
-        <f>INT(Q72/(18*0.95))</f>
+        <f>INT(Q72/(18*0.96))</f>
         <v/>
       </c>
       <c r="S72" s="18">
-        <f>ROUND(MOD(Q72, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q72, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T72" s="18">
-        <f>IF(S72&gt;0, ROUNDUP(S72/(5*0.95), 0), 0)</f>
+        <f>IF(S72&gt;0, ROUNDUP(S72/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U72" s="18">
@@ -12681,15 +12681,15 @@
         </is>
       </c>
       <c r="J73" s="18">
-        <f>INT(H73/(18*0.95))</f>
+        <f>INT(H73/(18*0.96))</f>
         <v/>
       </c>
       <c r="K73" s="18">
-        <f>ROUND(MOD(H73, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H73, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L73" s="18">
-        <f>IF(K73&gt;0, ROUNDUP(K73/(5*0.95), 0), 0)</f>
+        <f>IF(K73&gt;0, ROUNDUP(K73/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M73" s="18">
@@ -12713,15 +12713,15 @@
         <v/>
       </c>
       <c r="R73" s="18">
-        <f>INT(Q73/(18*0.95))</f>
+        <f>INT(Q73/(18*0.96))</f>
         <v/>
       </c>
       <c r="S73" s="18">
-        <f>ROUND(MOD(Q73, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q73, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T73" s="18">
-        <f>IF(S73&gt;0, ROUNDUP(S73/(5*0.95), 0), 0)</f>
+        <f>IF(S73&gt;0, ROUNDUP(S73/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U73" s="18">
@@ -12849,15 +12849,15 @@
         </is>
       </c>
       <c r="J74" s="18">
-        <f>INT(H74/(18*0.95))</f>
+        <f>INT(H74/(18*0.96))</f>
         <v/>
       </c>
       <c r="K74" s="18">
-        <f>ROUND(MOD(H74, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H74, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L74" s="18">
-        <f>IF(K74&gt;0, ROUNDUP(K74/(5*0.95), 0), 0)</f>
+        <f>IF(K74&gt;0, ROUNDUP(K74/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M74" s="18">
@@ -12881,15 +12881,15 @@
         <v/>
       </c>
       <c r="R74" s="18">
-        <f>INT(Q74/(18*0.95))</f>
+        <f>INT(Q74/(18*0.96))</f>
         <v/>
       </c>
       <c r="S74" s="18">
-        <f>ROUND(MOD(Q74, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q74, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T74" s="18">
-        <f>IF(S74&gt;0, ROUNDUP(S74/(5*0.95), 0), 0)</f>
+        <f>IF(S74&gt;0, ROUNDUP(S74/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U74" s="18">
@@ -13017,15 +13017,15 @@
         </is>
       </c>
       <c r="J75" s="18">
-        <f>INT(H75/(18*0.95))</f>
+        <f>INT(H75/(18*0.96))</f>
         <v/>
       </c>
       <c r="K75" s="18">
-        <f>ROUND(MOD(H75, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H75, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L75" s="18">
-        <f>IF(K75&gt;0, ROUNDUP(K75/(5*0.95), 0), 0)</f>
+        <f>IF(K75&gt;0, ROUNDUP(K75/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M75" s="18">
@@ -13049,15 +13049,15 @@
         <v/>
       </c>
       <c r="R75" s="18">
-        <f>INT(Q75/(18*0.95))</f>
+        <f>INT(Q75/(18*0.96))</f>
         <v/>
       </c>
       <c r="S75" s="18">
-        <f>ROUND(MOD(Q75, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q75, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T75" s="18">
-        <f>IF(S75&gt;0, ROUNDUP(S75/(5*0.95), 0), 0)</f>
+        <f>IF(S75&gt;0, ROUNDUP(S75/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U75" s="18">
@@ -13185,15 +13185,15 @@
         </is>
       </c>
       <c r="J76" s="18">
-        <f>INT(H76/(18*0.95))</f>
+        <f>INT(H76/(18*0.96))</f>
         <v/>
       </c>
       <c r="K76" s="18">
-        <f>ROUND(MOD(H76, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H76, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L76" s="18">
-        <f>IF(K76&gt;0, ROUNDUP(K76/(5*0.95), 0), 0)</f>
+        <f>IF(K76&gt;0, ROUNDUP(K76/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M76" s="18">
@@ -13217,15 +13217,15 @@
         <v/>
       </c>
       <c r="R76" s="18">
-        <f>INT(Q76/(18*0.95))</f>
+        <f>INT(Q76/(18*0.96))</f>
         <v/>
       </c>
       <c r="S76" s="18">
-        <f>ROUND(MOD(Q76, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q76, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T76" s="18">
-        <f>IF(S76&gt;0, ROUNDUP(S76/(5*0.95), 0), 0)</f>
+        <f>IF(S76&gt;0, ROUNDUP(S76/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U76" s="18">
@@ -13353,15 +13353,15 @@
         </is>
       </c>
       <c r="J77" s="18">
-        <f>INT(H77/(18*0.95))</f>
+        <f>INT(H77/(18*0.96))</f>
         <v/>
       </c>
       <c r="K77" s="18">
-        <f>ROUND(MOD(H77, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H77, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L77" s="18">
-        <f>IF(K77&gt;0, ROUNDUP(K77/(5*0.95), 0), 0)</f>
+        <f>IF(K77&gt;0, ROUNDUP(K77/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M77" s="18">
@@ -13385,15 +13385,15 @@
         <v/>
       </c>
       <c r="R77" s="18">
-        <f>INT(Q77/(18*0.95))</f>
+        <f>INT(Q77/(18*0.96))</f>
         <v/>
       </c>
       <c r="S77" s="18">
-        <f>ROUND(MOD(Q77, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q77, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T77" s="18">
-        <f>IF(S77&gt;0, ROUNDUP(S77/(5*0.95), 0), 0)</f>
+        <f>IF(S77&gt;0, ROUNDUP(S77/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U77" s="18">
@@ -13521,15 +13521,15 @@
         </is>
       </c>
       <c r="J78" s="18">
-        <f>INT(H78/(18*0.95))</f>
+        <f>INT(H78/(18*0.96))</f>
         <v/>
       </c>
       <c r="K78" s="18">
-        <f>ROUND(MOD(H78, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H78, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L78" s="18">
-        <f>IF(K78&gt;0, ROUNDUP(K78/(5*0.95), 0), 0)</f>
+        <f>IF(K78&gt;0, ROUNDUP(K78/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M78" s="18">
@@ -13553,15 +13553,15 @@
         <v/>
       </c>
       <c r="R78" s="18">
-        <f>INT(Q78/(18*0.95))</f>
+        <f>INT(Q78/(18*0.96))</f>
         <v/>
       </c>
       <c r="S78" s="18">
-        <f>ROUND(MOD(Q78, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q78, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T78" s="18">
-        <f>IF(S78&gt;0, ROUNDUP(S78/(5*0.95), 0), 0)</f>
+        <f>IF(S78&gt;0, ROUNDUP(S78/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U78" s="18">
@@ -13689,15 +13689,15 @@
         </is>
       </c>
       <c r="J79" s="18">
-        <f>INT(H79/(18*0.95))</f>
+        <f>INT(H79/(18*0.96))</f>
         <v/>
       </c>
       <c r="K79" s="18">
-        <f>ROUND(MOD(H79, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H79, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L79" s="18">
-        <f>IF(K79&gt;0, ROUNDUP(K79/(5*0.95), 0), 0)</f>
+        <f>IF(K79&gt;0, ROUNDUP(K79/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M79" s="18">
@@ -13721,15 +13721,15 @@
         <v/>
       </c>
       <c r="R79" s="18">
-        <f>INT(Q79/(18*0.95))</f>
+        <f>INT(Q79/(18*0.96))</f>
         <v/>
       </c>
       <c r="S79" s="18">
-        <f>ROUND(MOD(Q79, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q79, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T79" s="18">
-        <f>IF(S79&gt;0, ROUNDUP(S79/(5*0.95), 0), 0)</f>
+        <f>IF(S79&gt;0, ROUNDUP(S79/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U79" s="18">
@@ -13857,15 +13857,15 @@
         </is>
       </c>
       <c r="J80" s="18">
-        <f>INT(H80/(18*0.95))</f>
+        <f>INT(H80/(18*0.96))</f>
         <v/>
       </c>
       <c r="K80" s="18">
-        <f>ROUND(MOD(H80, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H80, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L80" s="18">
-        <f>IF(K80&gt;0, ROUNDUP(K80/(5*0.95), 0), 0)</f>
+        <f>IF(K80&gt;0, ROUNDUP(K80/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M80" s="18">
@@ -13889,15 +13889,15 @@
         <v/>
       </c>
       <c r="R80" s="18">
-        <f>INT(Q80/(18*0.95))</f>
+        <f>INT(Q80/(18*0.96))</f>
         <v/>
       </c>
       <c r="S80" s="18">
-        <f>ROUND(MOD(Q80, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q80, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T80" s="18">
-        <f>IF(S80&gt;0, ROUNDUP(S80/(5*0.95), 0), 0)</f>
+        <f>IF(S80&gt;0, ROUNDUP(S80/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U80" s="18">
@@ -14025,15 +14025,15 @@
         </is>
       </c>
       <c r="J81" s="18">
-        <f>INT(H81/(18*0.95))</f>
+        <f>INT(H81/(18*0.96))</f>
         <v/>
       </c>
       <c r="K81" s="18">
-        <f>ROUND(MOD(H81, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H81, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L81" s="18">
-        <f>IF(K81&gt;0, ROUNDUP(K81/(5*0.95), 0), 0)</f>
+        <f>IF(K81&gt;0, ROUNDUP(K81/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M81" s="18">
@@ -14057,15 +14057,15 @@
         <v/>
       </c>
       <c r="R81" s="18">
-        <f>INT(Q81/(18*0.95))</f>
+        <f>INT(Q81/(18*0.96))</f>
         <v/>
       </c>
       <c r="S81" s="18">
-        <f>ROUND(MOD(Q81, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q81, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T81" s="18">
-        <f>IF(S81&gt;0, ROUNDUP(S81/(5*0.95), 0), 0)</f>
+        <f>IF(S81&gt;0, ROUNDUP(S81/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U81" s="18">
@@ -14193,15 +14193,15 @@
         </is>
       </c>
       <c r="J82" s="18">
-        <f>INT(H82/(18*0.95))</f>
+        <f>INT(H82/(18*0.96))</f>
         <v/>
       </c>
       <c r="K82" s="18">
-        <f>ROUND(MOD(H82, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H82, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L82" s="18">
-        <f>IF(K82&gt;0, ROUNDUP(K82/(5*0.95), 0), 0)</f>
+        <f>IF(K82&gt;0, ROUNDUP(K82/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M82" s="18">
@@ -14225,15 +14225,15 @@
         <v/>
       </c>
       <c r="R82" s="18">
-        <f>INT(Q82/(18*0.95))</f>
+        <f>INT(Q82/(18*0.96))</f>
         <v/>
       </c>
       <c r="S82" s="18">
-        <f>ROUND(MOD(Q82, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q82, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T82" s="18">
-        <f>IF(S82&gt;0, ROUNDUP(S82/(5*0.95), 0), 0)</f>
+        <f>IF(S82&gt;0, ROUNDUP(S82/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U82" s="18">
@@ -14361,15 +14361,15 @@
         </is>
       </c>
       <c r="J83" s="18">
-        <f>INT(H83/(18*0.95))</f>
+        <f>INT(H83/(18*0.96))</f>
         <v/>
       </c>
       <c r="K83" s="18">
-        <f>ROUND(MOD(H83, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H83, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L83" s="18">
-        <f>IF(K83&gt;0, ROUNDUP(K83/(5*0.95), 0), 0)</f>
+        <f>IF(K83&gt;0, ROUNDUP(K83/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M83" s="18">
@@ -14393,15 +14393,15 @@
         <v/>
       </c>
       <c r="R83" s="18">
-        <f>INT(Q83/(18*0.95))</f>
+        <f>INT(Q83/(18*0.96))</f>
         <v/>
       </c>
       <c r="S83" s="18">
-        <f>ROUND(MOD(Q83, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q83, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T83" s="18">
-        <f>IF(S83&gt;0, ROUNDUP(S83/(5*0.95), 0), 0)</f>
+        <f>IF(S83&gt;0, ROUNDUP(S83/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U83" s="18">
@@ -14529,15 +14529,15 @@
         </is>
       </c>
       <c r="J84" s="18">
-        <f>INT(H84/(18*0.95))</f>
+        <f>INT(H84/(18*0.96))</f>
         <v/>
       </c>
       <c r="K84" s="18">
-        <f>ROUND(MOD(H84, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H84, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L84" s="18">
-        <f>IF(K84&gt;0, ROUNDUP(K84/(5*0.95), 0), 0)</f>
+        <f>IF(K84&gt;0, ROUNDUP(K84/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M84" s="18">
@@ -14561,15 +14561,15 @@
         <v/>
       </c>
       <c r="R84" s="18">
-        <f>INT(Q84/(18*0.95))</f>
+        <f>INT(Q84/(18*0.96))</f>
         <v/>
       </c>
       <c r="S84" s="18">
-        <f>ROUND(MOD(Q84, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q84, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T84" s="18">
-        <f>IF(S84&gt;0, ROUNDUP(S84/(5*0.95), 0), 0)</f>
+        <f>IF(S84&gt;0, ROUNDUP(S84/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U84" s="18">
@@ -14697,15 +14697,15 @@
         </is>
       </c>
       <c r="J85" s="18">
-        <f>INT(H85/(18*0.95))</f>
+        <f>INT(H85/(18*0.96))</f>
         <v/>
       </c>
       <c r="K85" s="18">
-        <f>ROUND(MOD(H85, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H85, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L85" s="18">
-        <f>IF(K85&gt;0, ROUNDUP(K85/(5*0.95), 0), 0)</f>
+        <f>IF(K85&gt;0, ROUNDUP(K85/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M85" s="18">
@@ -14729,15 +14729,15 @@
         <v/>
       </c>
       <c r="R85" s="18">
-        <f>INT(Q85/(18*0.95))</f>
+        <f>INT(Q85/(18*0.96))</f>
         <v/>
       </c>
       <c r="S85" s="18">
-        <f>ROUND(MOD(Q85, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q85, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T85" s="18">
-        <f>IF(S85&gt;0, ROUNDUP(S85/(5*0.95), 0), 0)</f>
+        <f>IF(S85&gt;0, ROUNDUP(S85/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U85" s="18">
@@ -14865,15 +14865,15 @@
         </is>
       </c>
       <c r="J86" s="18">
-        <f>INT(H86/(18*0.95))</f>
+        <f>INT(H86/(18*0.96))</f>
         <v/>
       </c>
       <c r="K86" s="18">
-        <f>ROUND(MOD(H86, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H86, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L86" s="18">
-        <f>IF(K86&gt;0, ROUNDUP(K86/(5*0.95), 0), 0)</f>
+        <f>IF(K86&gt;0, ROUNDUP(K86/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M86" s="18">
@@ -14897,15 +14897,15 @@
         <v/>
       </c>
       <c r="R86" s="18">
-        <f>INT(Q86/(18*0.95))</f>
+        <f>INT(Q86/(18*0.96))</f>
         <v/>
       </c>
       <c r="S86" s="18">
-        <f>ROUND(MOD(Q86, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q86, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T86" s="18">
-        <f>IF(S86&gt;0, ROUNDUP(S86/(5*0.95), 0), 0)</f>
+        <f>IF(S86&gt;0, ROUNDUP(S86/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U86" s="18">
@@ -15033,15 +15033,15 @@
         </is>
       </c>
       <c r="J87" s="18">
-        <f>INT(H87/(18*0.95))</f>
+        <f>INT(H87/(18*0.96))</f>
         <v/>
       </c>
       <c r="K87" s="18">
-        <f>ROUND(MOD(H87, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H87, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L87" s="18">
-        <f>IF(K87&gt;0, ROUNDUP(K87/(5*0.95), 0), 0)</f>
+        <f>IF(K87&gt;0, ROUNDUP(K87/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M87" s="18">
@@ -15065,15 +15065,15 @@
         <v/>
       </c>
       <c r="R87" s="18">
-        <f>INT(Q87/(18*0.95))</f>
+        <f>INT(Q87/(18*0.96))</f>
         <v/>
       </c>
       <c r="S87" s="18">
-        <f>ROUND(MOD(Q87, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q87, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T87" s="18">
-        <f>IF(S87&gt;0, ROUNDUP(S87/(5*0.95), 0), 0)</f>
+        <f>IF(S87&gt;0, ROUNDUP(S87/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U87" s="18">
@@ -15201,15 +15201,15 @@
         </is>
       </c>
       <c r="J88" s="18">
-        <f>INT(H88/(18*0.95))</f>
+        <f>INT(H88/(18*0.96))</f>
         <v/>
       </c>
       <c r="K88" s="18">
-        <f>ROUND(MOD(H88, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H88, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L88" s="18">
-        <f>IF(K88&gt;0, ROUNDUP(K88/(5*0.95), 0), 0)</f>
+        <f>IF(K88&gt;0, ROUNDUP(K88/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M88" s="18">
@@ -15233,15 +15233,15 @@
         <v/>
       </c>
       <c r="R88" s="18">
-        <f>INT(Q88/(18*0.95))</f>
+        <f>INT(Q88/(18*0.96))</f>
         <v/>
       </c>
       <c r="S88" s="18">
-        <f>ROUND(MOD(Q88, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q88, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T88" s="18">
-        <f>IF(S88&gt;0, ROUNDUP(S88/(5*0.95), 0), 0)</f>
+        <f>IF(S88&gt;0, ROUNDUP(S88/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U88" s="18">
@@ -15369,15 +15369,15 @@
         </is>
       </c>
       <c r="J89" s="18">
-        <f>INT(H89/(18*0.95))</f>
+        <f>INT(H89/(18*0.96))</f>
         <v/>
       </c>
       <c r="K89" s="18">
-        <f>ROUND(MOD(H89, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H89, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L89" s="18">
-        <f>IF(K89&gt;0, ROUNDUP(K89/(5*0.95), 0), 0)</f>
+        <f>IF(K89&gt;0, ROUNDUP(K89/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M89" s="18">
@@ -15401,15 +15401,15 @@
         <v/>
       </c>
       <c r="R89" s="18">
-        <f>INT(Q89/(18*0.95))</f>
+        <f>INT(Q89/(18*0.96))</f>
         <v/>
       </c>
       <c r="S89" s="18">
-        <f>ROUND(MOD(Q89, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q89, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T89" s="18">
-        <f>IF(S89&gt;0, ROUNDUP(S89/(5*0.95), 0), 0)</f>
+        <f>IF(S89&gt;0, ROUNDUP(S89/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U89" s="18">
@@ -15537,15 +15537,15 @@
         </is>
       </c>
       <c r="J90" s="18">
-        <f>INT(H90/(18*0.95))</f>
+        <f>INT(H90/(18*0.96))</f>
         <v/>
       </c>
       <c r="K90" s="18">
-        <f>ROUND(MOD(H90, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H90, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L90" s="18">
-        <f>IF(K90&gt;0, ROUNDUP(K90/(5*0.95), 0), 0)</f>
+        <f>IF(K90&gt;0, ROUNDUP(K90/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M90" s="18">
@@ -15569,15 +15569,15 @@
         <v/>
       </c>
       <c r="R90" s="18">
-        <f>INT(Q90/(18*0.95))</f>
+        <f>INT(Q90/(18*0.96))</f>
         <v/>
       </c>
       <c r="S90" s="18">
-        <f>ROUND(MOD(Q90, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q90, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T90" s="18">
-        <f>IF(S90&gt;0, ROUNDUP(S90/(5*0.95), 0), 0)</f>
+        <f>IF(S90&gt;0, ROUNDUP(S90/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U90" s="18">
@@ -15705,15 +15705,15 @@
         </is>
       </c>
       <c r="J91" s="18">
-        <f>INT(H91/(18*0.95))</f>
+        <f>INT(H91/(18*0.96))</f>
         <v/>
       </c>
       <c r="K91" s="18">
-        <f>ROUND(MOD(H91, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H91, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L91" s="18">
-        <f>IF(K91&gt;0, ROUNDUP(K91/(5*0.95), 0), 0)</f>
+        <f>IF(K91&gt;0, ROUNDUP(K91/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M91" s="18">
@@ -15737,15 +15737,15 @@
         <v/>
       </c>
       <c r="R91" s="18">
-        <f>INT(Q91/(18*0.95))</f>
+        <f>INT(Q91/(18*0.96))</f>
         <v/>
       </c>
       <c r="S91" s="18">
-        <f>ROUND(MOD(Q91, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q91, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T91" s="18">
-        <f>IF(S91&gt;0, ROUNDUP(S91/(5*0.95), 0), 0)</f>
+        <f>IF(S91&gt;0, ROUNDUP(S91/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U91" s="18">
@@ -15873,15 +15873,15 @@
         </is>
       </c>
       <c r="J92" s="18">
-        <f>INT(H92/(18*0.95))</f>
+        <f>INT(H92/(18*0.96))</f>
         <v/>
       </c>
       <c r="K92" s="18">
-        <f>ROUND(MOD(H92, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H92, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L92" s="18">
-        <f>IF(K92&gt;0, ROUNDUP(K92/(5*0.95), 0), 0)</f>
+        <f>IF(K92&gt;0, ROUNDUP(K92/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M92" s="18">
@@ -15905,15 +15905,15 @@
         <v/>
       </c>
       <c r="R92" s="18">
-        <f>INT(Q92/(18*0.95))</f>
+        <f>INT(Q92/(18*0.96))</f>
         <v/>
       </c>
       <c r="S92" s="18">
-        <f>ROUND(MOD(Q92, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q92, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T92" s="18">
-        <f>IF(S92&gt;0, ROUNDUP(S92/(5*0.95), 0), 0)</f>
+        <f>IF(S92&gt;0, ROUNDUP(S92/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U92" s="18">
@@ -16041,15 +16041,15 @@
         </is>
       </c>
       <c r="J93" s="18">
-        <f>INT(H93/(18*0.95))</f>
+        <f>INT(H93/(18*0.96))</f>
         <v/>
       </c>
       <c r="K93" s="18">
-        <f>ROUND(MOD(H93, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H93, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L93" s="18">
-        <f>IF(K93&gt;0, ROUNDUP(K93/(5*0.95), 0), 0)</f>
+        <f>IF(K93&gt;0, ROUNDUP(K93/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M93" s="18">
@@ -16073,15 +16073,15 @@
         <v/>
       </c>
       <c r="R93" s="18">
-        <f>INT(Q93/(18*0.95))</f>
+        <f>INT(Q93/(18*0.96))</f>
         <v/>
       </c>
       <c r="S93" s="18">
-        <f>ROUND(MOD(Q93, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q93, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T93" s="18">
-        <f>IF(S93&gt;0, ROUNDUP(S93/(5*0.95), 0), 0)</f>
+        <f>IF(S93&gt;0, ROUNDUP(S93/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U93" s="18">
@@ -16209,15 +16209,15 @@
         </is>
       </c>
       <c r="J94" s="18">
-        <f>INT(H94/(18*0.95))</f>
+        <f>INT(H94/(18*0.96))</f>
         <v/>
       </c>
       <c r="K94" s="18">
-        <f>ROUND(MOD(H94, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(H94, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="L94" s="18">
-        <f>IF(K94&gt;0, ROUNDUP(K94/(5*0.95), 0), 0)</f>
+        <f>IF(K94&gt;0, ROUNDUP(K94/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="M94" s="18">
@@ -16241,15 +16241,15 @@
         <v/>
       </c>
       <c r="R94" s="18">
-        <f>INT(Q94/(18*0.95))</f>
+        <f>INT(Q94/(18*0.96))</f>
         <v/>
       </c>
       <c r="S94" s="18">
-        <f>ROUND(MOD(Q94, (18*0.95)), 2)</f>
+        <f>ROUND(MOD(Q94, (18*0.96)), 2)</f>
         <v/>
       </c>
       <c r="T94" s="18">
-        <f>IF(S94&gt;0, ROUNDUP(S94/(5*0.95), 0), 0)</f>
+        <f>IF(S94&gt;0, ROUNDUP(S94/(5*0.96), 0), 0)</f>
         <v/>
       </c>
       <c r="U94" s="18">
@@ -16431,11 +16431,11 @@
         </is>
       </c>
       <c r="C100" s="22">
-        <f>AVERAGE(AJ6:AJ94)*(18*0.95)</f>
+        <f>AVERAGE(AJ6:AJ94)*(18*0.96)</f>
         <v/>
       </c>
       <c r="D100" s="22">
-        <f>D98*(18*0.95)</f>
+        <f>D98*(18*0.96)</f>
         <v/>
       </c>
       <c r="E100" s="22">

</xml_diff>

<commit_message>
fix(eda): resolve title clipping in eda_01 and eliminate negative dispatch bar in eda_02
</commit_message>
<xml_diff>
--- a/data/FrostLink_Du_lieu_Chuan.xlsx
+++ b/data/FrostLink_Du_lieu_Chuan.xlsx
@@ -665,16 +665,16 @@
     <col width="33" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="23" customWidth="1" min="13" max="13"/>
-    <col width="44" customWidth="1" min="14" max="14"/>
-    <col width="48" customWidth="1" min="15" max="15"/>
-    <col width="48" customWidth="1" min="16" max="16"/>
+    <col width="53" customWidth="1" min="14" max="14"/>
+    <col width="57" customWidth="1" min="15" max="15"/>
+    <col width="57" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
     <col width="32" customWidth="1" min="18" max="18"/>
     <col width="33" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="39" customWidth="1" min="22" max="22"/>
-    <col width="47" customWidth="1" min="23" max="23"/>
+    <col width="55" customWidth="1" min="23" max="23"/>
     <col width="52" customWidth="1" min="24" max="24"/>
     <col width="30" customWidth="1" min="25" max="25"/>
     <col width="31" customWidth="1" min="26" max="26"/>
@@ -971,15 +971,15 @@
         <v/>
       </c>
       <c r="N3" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E3), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E3), 1))</f>
         <v/>
       </c>
       <c r="O3" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B3:E3), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B3:E3), 1))</f>
         <v/>
       </c>
       <c r="P3" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B3:F3), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B3:F3), 1))</f>
         <v/>
       </c>
       <c r="Q3" s="22">
@@ -987,7 +987,7 @@
         <v/>
       </c>
       <c r="R3" s="21">
-        <f>INT(Q3/(18*0.96))</f>
+        <f>MAX(0, INT(Q3/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S3" s="22">
@@ -1003,11 +1003,11 @@
         <v/>
       </c>
       <c r="V3" s="21">
-        <f>ROUND(R3*70%, 0)</f>
+        <f>MAX(0, ROUND(R3*70%, 0))</f>
         <v/>
       </c>
       <c r="W3" s="21">
-        <f>MIN(ROUNDUP(R3*0.2, 0), MAX(0, R3 - V3))</f>
+        <f>MAX(0, MIN(ROUNDUP(R3*0.2, 0), MAX(0, R3 - V3)))</f>
         <v/>
       </c>
       <c r="X3" s="17">
@@ -1133,15 +1133,15 @@
         <v/>
       </c>
       <c r="N4" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E4), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E4), 1))</f>
         <v/>
       </c>
       <c r="O4" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B4:E4), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B4:E4), 1))</f>
         <v/>
       </c>
       <c r="P4" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B4:F4), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B4:F4), 1))</f>
         <v/>
       </c>
       <c r="Q4" s="22">
@@ -1149,7 +1149,7 @@
         <v/>
       </c>
       <c r="R4" s="21">
-        <f>INT(Q4/(18*0.96))</f>
+        <f>MAX(0, INT(Q4/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S4" s="22">
@@ -1165,11 +1165,11 @@
         <v/>
       </c>
       <c r="V4" s="21">
-        <f>ROUND(R4*70%, 0)</f>
+        <f>MAX(0, ROUND(R4*70%, 0))</f>
         <v/>
       </c>
       <c r="W4" s="21">
-        <f>MIN(ROUNDUP(R4*0.2, 0), MAX(0, R4 - V4))</f>
+        <f>MAX(0, MIN(ROUNDUP(R4*0.2, 0), MAX(0, R4 - V4)))</f>
         <v/>
       </c>
       <c r="X4" s="17">
@@ -1295,15 +1295,15 @@
         <v/>
       </c>
       <c r="N5" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E5), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E5), 1))</f>
         <v/>
       </c>
       <c r="O5" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B5:E5), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B5:E5), 1))</f>
         <v/>
       </c>
       <c r="P5" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B5:F5), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B5:F5), 1))</f>
         <v/>
       </c>
       <c r="Q5" s="22">
@@ -1311,7 +1311,7 @@
         <v/>
       </c>
       <c r="R5" s="21">
-        <f>INT(Q5/(18*0.96))</f>
+        <f>MAX(0, INT(Q5/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S5" s="22">
@@ -1327,11 +1327,11 @@
         <v/>
       </c>
       <c r="V5" s="21">
-        <f>ROUND(R5*70%, 0)</f>
+        <f>MAX(0, ROUND(R5*70%, 0))</f>
         <v/>
       </c>
       <c r="W5" s="21">
-        <f>MIN(ROUNDUP(R5*0.2, 0), MAX(0, R5 - V5))</f>
+        <f>MAX(0, MIN(ROUNDUP(R5*0.2, 0), MAX(0, R5 - V5)))</f>
         <v/>
       </c>
       <c r="X5" s="17">
@@ -1457,15 +1457,15 @@
         <v/>
       </c>
       <c r="N6" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E6), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E6), 1))</f>
         <v/>
       </c>
       <c r="O6" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B6:E6), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B6:E6), 1))</f>
         <v/>
       </c>
       <c r="P6" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B6:F6), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B6:F6), 1))</f>
         <v/>
       </c>
       <c r="Q6" s="22">
@@ -1473,7 +1473,7 @@
         <v/>
       </c>
       <c r="R6" s="21">
-        <f>INT(Q6/(18*0.96))</f>
+        <f>MAX(0, INT(Q6/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S6" s="22">
@@ -1489,11 +1489,11 @@
         <v/>
       </c>
       <c r="V6" s="21">
-        <f>ROUND(R6*70%, 0)</f>
+        <f>MAX(0, ROUND(R6*70%, 0))</f>
         <v/>
       </c>
       <c r="W6" s="21">
-        <f>MIN(ROUNDUP(R6*0.2, 0), MAX(0, R6 - V6))</f>
+        <f>MAX(0, MIN(ROUNDUP(R6*0.2, 0), MAX(0, R6 - V6)))</f>
         <v/>
       </c>
       <c r="X6" s="17">
@@ -1625,15 +1625,15 @@
         <v/>
       </c>
       <c r="N7" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E7), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E7), 1))</f>
         <v/>
       </c>
       <c r="O7" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B7:E7), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B7:E7), 1))</f>
         <v/>
       </c>
       <c r="P7" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B7:F7), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B7:F7), 1))</f>
         <v/>
       </c>
       <c r="Q7" s="22">
@@ -1641,7 +1641,7 @@
         <v/>
       </c>
       <c r="R7" s="21">
-        <f>INT(Q7/(18*0.96))</f>
+        <f>MAX(0, INT(Q7/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S7" s="22">
@@ -1657,11 +1657,11 @@
         <v/>
       </c>
       <c r="V7" s="21">
-        <f>ROUND(R7*70%, 0)</f>
+        <f>MAX(0, ROUND(R7*70%, 0))</f>
         <v/>
       </c>
       <c r="W7" s="21">
-        <f>MIN(ROUNDUP(R7*0.2, 0), MAX(0, R7 - V7))</f>
+        <f>MAX(0, MIN(ROUNDUP(R7*0.2, 0), MAX(0, R7 - V7)))</f>
         <v/>
       </c>
       <c r="X7" s="17">
@@ -1793,15 +1793,15 @@
         <v/>
       </c>
       <c r="N8" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E8), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E8), 1))</f>
         <v/>
       </c>
       <c r="O8" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B8:E8), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B8:E8), 1))</f>
         <v/>
       </c>
       <c r="P8" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B8:F8), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B8:F8), 1))</f>
         <v/>
       </c>
       <c r="Q8" s="22">
@@ -1809,7 +1809,7 @@
         <v/>
       </c>
       <c r="R8" s="21">
-        <f>INT(Q8/(18*0.96))</f>
+        <f>MAX(0, INT(Q8/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S8" s="22">
@@ -1825,11 +1825,11 @@
         <v/>
       </c>
       <c r="V8" s="21">
-        <f>ROUND(R8*70%, 0)</f>
+        <f>MAX(0, ROUND(R8*70%, 0))</f>
         <v/>
       </c>
       <c r="W8" s="21">
-        <f>MIN(ROUNDUP(R8*0.2, 0), MAX(0, R8 - V8))</f>
+        <f>MAX(0, MIN(ROUNDUP(R8*0.2, 0), MAX(0, R8 - V8)))</f>
         <v/>
       </c>
       <c r="X8" s="17">
@@ -1961,15 +1961,15 @@
         <v/>
       </c>
       <c r="N9" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E9), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E9), 1))</f>
         <v/>
       </c>
       <c r="O9" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B9:E9), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B9:E9), 1))</f>
         <v/>
       </c>
       <c r="P9" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B9:F9), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B9:F9), 1))</f>
         <v/>
       </c>
       <c r="Q9" s="22">
@@ -1977,7 +1977,7 @@
         <v/>
       </c>
       <c r="R9" s="21">
-        <f>INT(Q9/(18*0.96))</f>
+        <f>MAX(0, INT(Q9/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S9" s="22">
@@ -1993,11 +1993,11 @@
         <v/>
       </c>
       <c r="V9" s="21">
-        <f>ROUND(R9*70%, 0)</f>
+        <f>MAX(0, ROUND(R9*70%, 0))</f>
         <v/>
       </c>
       <c r="W9" s="21">
-        <f>MIN(ROUNDUP(R9*0.2, 0), MAX(0, R9 - V9))</f>
+        <f>MAX(0, MIN(ROUNDUP(R9*0.2, 0), MAX(0, R9 - V9)))</f>
         <v/>
       </c>
       <c r="X9" s="17">
@@ -2129,15 +2129,15 @@
         <v/>
       </c>
       <c r="N10" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E10), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E10), 1))</f>
         <v/>
       </c>
       <c r="O10" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B10:E10), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B10:E10), 1))</f>
         <v/>
       </c>
       <c r="P10" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B10:F10), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B10:F10), 1))</f>
         <v/>
       </c>
       <c r="Q10" s="22">
@@ -2145,7 +2145,7 @@
         <v/>
       </c>
       <c r="R10" s="21">
-        <f>INT(Q10/(18*0.96))</f>
+        <f>MAX(0, INT(Q10/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S10" s="22">
@@ -2161,11 +2161,11 @@
         <v/>
       </c>
       <c r="V10" s="21">
-        <f>ROUND(R10*70%, 0)</f>
+        <f>MAX(0, ROUND(R10*70%, 0))</f>
         <v/>
       </c>
       <c r="W10" s="21">
-        <f>MIN(ROUNDUP(R10*0.2, 0), MAX(0, R10 - V10))</f>
+        <f>MAX(0, MIN(ROUNDUP(R10*0.2, 0), MAX(0, R10 - V10)))</f>
         <v/>
       </c>
       <c r="X10" s="17">
@@ -2297,15 +2297,15 @@
         <v/>
       </c>
       <c r="N11" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E11), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E11), 1))</f>
         <v/>
       </c>
       <c r="O11" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B11:E11), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B11:E11), 1))</f>
         <v/>
       </c>
       <c r="P11" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B11:F11), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B11:F11), 1))</f>
         <v/>
       </c>
       <c r="Q11" s="22">
@@ -2313,7 +2313,7 @@
         <v/>
       </c>
       <c r="R11" s="21">
-        <f>INT(Q11/(18*0.96))</f>
+        <f>MAX(0, INT(Q11/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S11" s="22">
@@ -2329,11 +2329,11 @@
         <v/>
       </c>
       <c r="V11" s="21">
-        <f>ROUND(R11*70%, 0)</f>
+        <f>MAX(0, ROUND(R11*70%, 0))</f>
         <v/>
       </c>
       <c r="W11" s="21">
-        <f>MIN(ROUNDUP(R11*0.2, 0), MAX(0, R11 - V11))</f>
+        <f>MAX(0, MIN(ROUNDUP(R11*0.2, 0), MAX(0, R11 - V11)))</f>
         <v/>
       </c>
       <c r="X11" s="17">
@@ -2465,15 +2465,15 @@
         <v/>
       </c>
       <c r="N12" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E12), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E12), 1))</f>
         <v/>
       </c>
       <c r="O12" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B12:E12), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B12:E12), 1))</f>
         <v/>
       </c>
       <c r="P12" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B12:F12), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B12:F12), 1))</f>
         <v/>
       </c>
       <c r="Q12" s="22">
@@ -2481,7 +2481,7 @@
         <v/>
       </c>
       <c r="R12" s="21">
-        <f>INT(Q12/(18*0.96))</f>
+        <f>MAX(0, INT(Q12/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S12" s="22">
@@ -2497,11 +2497,11 @@
         <v/>
       </c>
       <c r="V12" s="21">
-        <f>ROUND(R12*70%, 0)</f>
+        <f>MAX(0, ROUND(R12*70%, 0))</f>
         <v/>
       </c>
       <c r="W12" s="21">
-        <f>MIN(ROUNDUP(R12*0.2, 0), MAX(0, R12 - V12))</f>
+        <f>MAX(0, MIN(ROUNDUP(R12*0.2, 0), MAX(0, R12 - V12)))</f>
         <v/>
       </c>
       <c r="X12" s="17">
@@ -2633,15 +2633,15 @@
         <v/>
       </c>
       <c r="N13" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E13), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E13), 1))</f>
         <v/>
       </c>
       <c r="O13" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B13:E13), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B13:E13), 1))</f>
         <v/>
       </c>
       <c r="P13" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B13:F13), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B13:F13), 1))</f>
         <v/>
       </c>
       <c r="Q13" s="22">
@@ -2649,7 +2649,7 @@
         <v/>
       </c>
       <c r="R13" s="21">
-        <f>INT(Q13/(18*0.96))</f>
+        <f>MAX(0, INT(Q13/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S13" s="22">
@@ -2665,11 +2665,11 @@
         <v/>
       </c>
       <c r="V13" s="21">
-        <f>ROUND(R13*70%, 0)</f>
+        <f>MAX(0, ROUND(R13*70%, 0))</f>
         <v/>
       </c>
       <c r="W13" s="21">
-        <f>MIN(ROUNDUP(R13*0.2, 0), MAX(0, R13 - V13))</f>
+        <f>MAX(0, MIN(ROUNDUP(R13*0.2, 0), MAX(0, R13 - V13)))</f>
         <v/>
       </c>
       <c r="X13" s="17">
@@ -2801,15 +2801,15 @@
         <v/>
       </c>
       <c r="N14" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E14), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E14), 1))</f>
         <v/>
       </c>
       <c r="O14" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B14:E14), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B14:E14), 1))</f>
         <v/>
       </c>
       <c r="P14" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B14:F14), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B14:F14), 1))</f>
         <v/>
       </c>
       <c r="Q14" s="22">
@@ -2817,7 +2817,7 @@
         <v/>
       </c>
       <c r="R14" s="21">
-        <f>INT(Q14/(18*0.96))</f>
+        <f>MAX(0, INT(Q14/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S14" s="22">
@@ -2833,11 +2833,11 @@
         <v/>
       </c>
       <c r="V14" s="21">
-        <f>ROUND(R14*70%, 0)</f>
+        <f>MAX(0, ROUND(R14*70%, 0))</f>
         <v/>
       </c>
       <c r="W14" s="21">
-        <f>MIN(ROUNDUP(R14*0.2, 0), MAX(0, R14 - V14))</f>
+        <f>MAX(0, MIN(ROUNDUP(R14*0.2, 0), MAX(0, R14 - V14)))</f>
         <v/>
       </c>
       <c r="X14" s="17">
@@ -2969,15 +2969,15 @@
         <v/>
       </c>
       <c r="N15" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E15), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E15), 1))</f>
         <v/>
       </c>
       <c r="O15" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B15:E15), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B15:E15), 1))</f>
         <v/>
       </c>
       <c r="P15" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B15:F15), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B15:F15), 1))</f>
         <v/>
       </c>
       <c r="Q15" s="22">
@@ -2985,7 +2985,7 @@
         <v/>
       </c>
       <c r="R15" s="21">
-        <f>INT(Q15/(18*0.96))</f>
+        <f>MAX(0, INT(Q15/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S15" s="22">
@@ -3001,11 +3001,11 @@
         <v/>
       </c>
       <c r="V15" s="21">
-        <f>ROUND(R15*70%, 0)</f>
+        <f>MAX(0, ROUND(R15*70%, 0))</f>
         <v/>
       </c>
       <c r="W15" s="21">
-        <f>MIN(ROUNDUP(R15*0.2, 0), MAX(0, R15 - V15))</f>
+        <f>MAX(0, MIN(ROUNDUP(R15*0.2, 0), MAX(0, R15 - V15)))</f>
         <v/>
       </c>
       <c r="X15" s="17">
@@ -3137,15 +3137,15 @@
         <v/>
       </c>
       <c r="N16" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E16), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E16), 1))</f>
         <v/>
       </c>
       <c r="O16" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B16:E16), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B16:E16), 1))</f>
         <v/>
       </c>
       <c r="P16" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B16:F16), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B16:F16), 1))</f>
         <v/>
       </c>
       <c r="Q16" s="22">
@@ -3153,7 +3153,7 @@
         <v/>
       </c>
       <c r="R16" s="21">
-        <f>INT(Q16/(18*0.96))</f>
+        <f>MAX(0, INT(Q16/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S16" s="22">
@@ -3169,11 +3169,11 @@
         <v/>
       </c>
       <c r="V16" s="21">
-        <f>ROUND(R16*70%, 0)</f>
+        <f>MAX(0, ROUND(R16*70%, 0))</f>
         <v/>
       </c>
       <c r="W16" s="21">
-        <f>MIN(ROUNDUP(R16*0.2, 0), MAX(0, R16 - V16))</f>
+        <f>MAX(0, MIN(ROUNDUP(R16*0.2, 0), MAX(0, R16 - V16)))</f>
         <v/>
       </c>
       <c r="X16" s="17">
@@ -3305,15 +3305,15 @@
         <v/>
       </c>
       <c r="N17" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E17), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E17), 1))</f>
         <v/>
       </c>
       <c r="O17" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B17:E17), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B17:E17), 1))</f>
         <v/>
       </c>
       <c r="P17" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B17:F17), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B17:F17), 1))</f>
         <v/>
       </c>
       <c r="Q17" s="22">
@@ -3321,7 +3321,7 @@
         <v/>
       </c>
       <c r="R17" s="21">
-        <f>INT(Q17/(18*0.96))</f>
+        <f>MAX(0, INT(Q17/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S17" s="22">
@@ -3337,11 +3337,11 @@
         <v/>
       </c>
       <c r="V17" s="21">
-        <f>ROUND(R17*70%, 0)</f>
+        <f>MAX(0, ROUND(R17*70%, 0))</f>
         <v/>
       </c>
       <c r="W17" s="21">
-        <f>MIN(ROUNDUP(R17*0.2, 0), MAX(0, R17 - V17))</f>
+        <f>MAX(0, MIN(ROUNDUP(R17*0.2, 0), MAX(0, R17 - V17)))</f>
         <v/>
       </c>
       <c r="X17" s="17">
@@ -3473,15 +3473,15 @@
         <v/>
       </c>
       <c r="N18" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E18), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E18), 1))</f>
         <v/>
       </c>
       <c r="O18" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B18:E18), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B18:E18), 1))</f>
         <v/>
       </c>
       <c r="P18" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B18:F18), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B18:F18), 1))</f>
         <v/>
       </c>
       <c r="Q18" s="22">
@@ -3489,7 +3489,7 @@
         <v/>
       </c>
       <c r="R18" s="21">
-        <f>INT(Q18/(18*0.96))</f>
+        <f>MAX(0, INT(Q18/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S18" s="22">
@@ -3505,11 +3505,11 @@
         <v/>
       </c>
       <c r="V18" s="21">
-        <f>ROUND(R18*70%, 0)</f>
+        <f>MAX(0, ROUND(R18*70%, 0))</f>
         <v/>
       </c>
       <c r="W18" s="21">
-        <f>MIN(ROUNDUP(R18*0.2, 0), MAX(0, R18 - V18))</f>
+        <f>MAX(0, MIN(ROUNDUP(R18*0.2, 0), MAX(0, R18 - V18)))</f>
         <v/>
       </c>
       <c r="X18" s="17">
@@ -3641,15 +3641,15 @@
         <v/>
       </c>
       <c r="N19" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E19), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E19), 1))</f>
         <v/>
       </c>
       <c r="O19" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B19:E19), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B19:E19), 1))</f>
         <v/>
       </c>
       <c r="P19" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B19:F19), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B19:F19), 1))</f>
         <v/>
       </c>
       <c r="Q19" s="22">
@@ -3657,7 +3657,7 @@
         <v/>
       </c>
       <c r="R19" s="21">
-        <f>INT(Q19/(18*0.96))</f>
+        <f>MAX(0, INT(Q19/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S19" s="22">
@@ -3673,11 +3673,11 @@
         <v/>
       </c>
       <c r="V19" s="21">
-        <f>ROUND(R19*70%, 0)</f>
+        <f>MAX(0, ROUND(R19*70%, 0))</f>
         <v/>
       </c>
       <c r="W19" s="21">
-        <f>MIN(ROUNDUP(R19*0.2, 0), MAX(0, R19 - V19))</f>
+        <f>MAX(0, MIN(ROUNDUP(R19*0.2, 0), MAX(0, R19 - V19)))</f>
         <v/>
       </c>
       <c r="X19" s="17">
@@ -3809,15 +3809,15 @@
         <v/>
       </c>
       <c r="N20" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E20), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E20), 1))</f>
         <v/>
       </c>
       <c r="O20" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B20:E20), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B20:E20), 1))</f>
         <v/>
       </c>
       <c r="P20" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B20:F20), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B20:F20), 1))</f>
         <v/>
       </c>
       <c r="Q20" s="22">
@@ -3825,7 +3825,7 @@
         <v/>
       </c>
       <c r="R20" s="21">
-        <f>INT(Q20/(18*0.96))</f>
+        <f>MAX(0, INT(Q20/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S20" s="22">
@@ -3841,11 +3841,11 @@
         <v/>
       </c>
       <c r="V20" s="21">
-        <f>ROUND(R20*70%, 0)</f>
+        <f>MAX(0, ROUND(R20*70%, 0))</f>
         <v/>
       </c>
       <c r="W20" s="21">
-        <f>MIN(ROUNDUP(R20*0.2, 0), MAX(0, R20 - V20))</f>
+        <f>MAX(0, MIN(ROUNDUP(R20*0.2, 0), MAX(0, R20 - V20)))</f>
         <v/>
       </c>
       <c r="X20" s="17">
@@ -3977,15 +3977,15 @@
         <v/>
       </c>
       <c r="N21" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E21), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E21), 1))</f>
         <v/>
       </c>
       <c r="O21" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B21:E21), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B21:E21), 1))</f>
         <v/>
       </c>
       <c r="P21" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B21:F21), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B21:F21), 1))</f>
         <v/>
       </c>
       <c r="Q21" s="22">
@@ -3993,7 +3993,7 @@
         <v/>
       </c>
       <c r="R21" s="21">
-        <f>INT(Q21/(18*0.96))</f>
+        <f>MAX(0, INT(Q21/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S21" s="22">
@@ -4009,11 +4009,11 @@
         <v/>
       </c>
       <c r="V21" s="21">
-        <f>ROUND(R21*70%, 0)</f>
+        <f>MAX(0, ROUND(R21*70%, 0))</f>
         <v/>
       </c>
       <c r="W21" s="21">
-        <f>MIN(ROUNDUP(R21*0.2, 0), MAX(0, R21 - V21))</f>
+        <f>MAX(0, MIN(ROUNDUP(R21*0.2, 0), MAX(0, R21 - V21)))</f>
         <v/>
       </c>
       <c r="X21" s="17">
@@ -4145,15 +4145,15 @@
         <v/>
       </c>
       <c r="N22" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E22), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E22), 1))</f>
         <v/>
       </c>
       <c r="O22" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B22:E22), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B22:E22), 1))</f>
         <v/>
       </c>
       <c r="P22" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B22:F22), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B22:F22), 1))</f>
         <v/>
       </c>
       <c r="Q22" s="22">
@@ -4161,7 +4161,7 @@
         <v/>
       </c>
       <c r="R22" s="21">
-        <f>INT(Q22/(18*0.96))</f>
+        <f>MAX(0, INT(Q22/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S22" s="22">
@@ -4177,11 +4177,11 @@
         <v/>
       </c>
       <c r="V22" s="21">
-        <f>ROUND(R22*70%, 0)</f>
+        <f>MAX(0, ROUND(R22*70%, 0))</f>
         <v/>
       </c>
       <c r="W22" s="21">
-        <f>MIN(ROUNDUP(R22*0.2, 0), MAX(0, R22 - V22))</f>
+        <f>MAX(0, MIN(ROUNDUP(R22*0.2, 0), MAX(0, R22 - V22)))</f>
         <v/>
       </c>
       <c r="X22" s="17">
@@ -4313,15 +4313,15 @@
         <v/>
       </c>
       <c r="N23" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E23), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E23), 1))</f>
         <v/>
       </c>
       <c r="O23" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B23:E23), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B23:E23), 1))</f>
         <v/>
       </c>
       <c r="P23" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B23:F23), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B23:F23), 1))</f>
         <v/>
       </c>
       <c r="Q23" s="22">
@@ -4329,7 +4329,7 @@
         <v/>
       </c>
       <c r="R23" s="21">
-        <f>INT(Q23/(18*0.96))</f>
+        <f>MAX(0, INT(Q23/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S23" s="22">
@@ -4345,11 +4345,11 @@
         <v/>
       </c>
       <c r="V23" s="21">
-        <f>ROUND(R23*70%, 0)</f>
+        <f>MAX(0, ROUND(R23*70%, 0))</f>
         <v/>
       </c>
       <c r="W23" s="21">
-        <f>MIN(ROUNDUP(R23*0.2, 0), MAX(0, R23 - V23))</f>
+        <f>MAX(0, MIN(ROUNDUP(R23*0.2, 0), MAX(0, R23 - V23)))</f>
         <v/>
       </c>
       <c r="X23" s="17">
@@ -4481,15 +4481,15 @@
         <v/>
       </c>
       <c r="N24" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E24), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E24), 1))</f>
         <v/>
       </c>
       <c r="O24" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B24:E24), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B24:E24), 1))</f>
         <v/>
       </c>
       <c r="P24" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B24:F24), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B24:F24), 1))</f>
         <v/>
       </c>
       <c r="Q24" s="22">
@@ -4497,7 +4497,7 @@
         <v/>
       </c>
       <c r="R24" s="21">
-        <f>INT(Q24/(18*0.96))</f>
+        <f>MAX(0, INT(Q24/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S24" s="22">
@@ -4513,11 +4513,11 @@
         <v/>
       </c>
       <c r="V24" s="21">
-        <f>ROUND(R24*70%, 0)</f>
+        <f>MAX(0, ROUND(R24*70%, 0))</f>
         <v/>
       </c>
       <c r="W24" s="21">
-        <f>MIN(ROUNDUP(R24*0.2, 0), MAX(0, R24 - V24))</f>
+        <f>MAX(0, MIN(ROUNDUP(R24*0.2, 0), MAX(0, R24 - V24)))</f>
         <v/>
       </c>
       <c r="X24" s="17">
@@ -4649,15 +4649,15 @@
         <v/>
       </c>
       <c r="N25" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E25), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E25), 1))</f>
         <v/>
       </c>
       <c r="O25" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B25:E25), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B25:E25), 1))</f>
         <v/>
       </c>
       <c r="P25" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B25:F25), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B25:F25), 1))</f>
         <v/>
       </c>
       <c r="Q25" s="22">
@@ -4665,7 +4665,7 @@
         <v/>
       </c>
       <c r="R25" s="21">
-        <f>INT(Q25/(18*0.96))</f>
+        <f>MAX(0, INT(Q25/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S25" s="22">
@@ -4681,11 +4681,11 @@
         <v/>
       </c>
       <c r="V25" s="21">
-        <f>ROUND(R25*70%, 0)</f>
+        <f>MAX(0, ROUND(R25*70%, 0))</f>
         <v/>
       </c>
       <c r="W25" s="21">
-        <f>MIN(ROUNDUP(R25*0.2, 0), MAX(0, R25 - V25))</f>
+        <f>MAX(0, MIN(ROUNDUP(R25*0.2, 0), MAX(0, R25 - V25)))</f>
         <v/>
       </c>
       <c r="X25" s="17">
@@ -4817,15 +4817,15 @@
         <v/>
       </c>
       <c r="N26" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E26), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E26), 1))</f>
         <v/>
       </c>
       <c r="O26" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B26:E26), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B26:E26), 1))</f>
         <v/>
       </c>
       <c r="P26" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B26:F26), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B26:F26), 1))</f>
         <v/>
       </c>
       <c r="Q26" s="22">
@@ -4833,7 +4833,7 @@
         <v/>
       </c>
       <c r="R26" s="21">
-        <f>INT(Q26/(18*0.96))</f>
+        <f>MAX(0, INT(Q26/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S26" s="22">
@@ -4849,11 +4849,11 @@
         <v/>
       </c>
       <c r="V26" s="21">
-        <f>ROUND(R26*70%, 0)</f>
+        <f>MAX(0, ROUND(R26*70%, 0))</f>
         <v/>
       </c>
       <c r="W26" s="21">
-        <f>MIN(ROUNDUP(R26*0.2, 0), MAX(0, R26 - V26))</f>
+        <f>MAX(0, MIN(ROUNDUP(R26*0.2, 0), MAX(0, R26 - V26)))</f>
         <v/>
       </c>
       <c r="X26" s="17">
@@ -4985,15 +4985,15 @@
         <v/>
       </c>
       <c r="N27" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E27), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E27), 1))</f>
         <v/>
       </c>
       <c r="O27" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B27:E27), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B27:E27), 1))</f>
         <v/>
       </c>
       <c r="P27" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B27:F27), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B27:F27), 1))</f>
         <v/>
       </c>
       <c r="Q27" s="22">
@@ -5001,7 +5001,7 @@
         <v/>
       </c>
       <c r="R27" s="21">
-        <f>INT(Q27/(18*0.96))</f>
+        <f>MAX(0, INT(Q27/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S27" s="22">
@@ -5017,11 +5017,11 @@
         <v/>
       </c>
       <c r="V27" s="21">
-        <f>ROUND(R27*70%, 0)</f>
+        <f>MAX(0, ROUND(R27*70%, 0))</f>
         <v/>
       </c>
       <c r="W27" s="21">
-        <f>MIN(ROUNDUP(R27*0.2, 0), MAX(0, R27 - V27))</f>
+        <f>MAX(0, MIN(ROUNDUP(R27*0.2, 0), MAX(0, R27 - V27)))</f>
         <v/>
       </c>
       <c r="X27" s="17">
@@ -5153,15 +5153,15 @@
         <v/>
       </c>
       <c r="N28" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E28), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E28), 1))</f>
         <v/>
       </c>
       <c r="O28" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B28:E28), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B28:E28), 1))</f>
         <v/>
       </c>
       <c r="P28" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B28:F28), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B28:F28), 1))</f>
         <v/>
       </c>
       <c r="Q28" s="22">
@@ -5169,7 +5169,7 @@
         <v/>
       </c>
       <c r="R28" s="21">
-        <f>INT(Q28/(18*0.96))</f>
+        <f>MAX(0, INT(Q28/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S28" s="22">
@@ -5185,11 +5185,11 @@
         <v/>
       </c>
       <c r="V28" s="21">
-        <f>ROUND(R28*70%, 0)</f>
+        <f>MAX(0, ROUND(R28*70%, 0))</f>
         <v/>
       </c>
       <c r="W28" s="21">
-        <f>MIN(ROUNDUP(R28*0.2, 0), MAX(0, R28 - V28))</f>
+        <f>MAX(0, MIN(ROUNDUP(R28*0.2, 0), MAX(0, R28 - V28)))</f>
         <v/>
       </c>
       <c r="X28" s="17">
@@ -5321,15 +5321,15 @@
         <v/>
       </c>
       <c r="N29" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E29), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E29), 1))</f>
         <v/>
       </c>
       <c r="O29" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B29:E29), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B29:E29), 1))</f>
         <v/>
       </c>
       <c r="P29" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B29:F29), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B29:F29), 1))</f>
         <v/>
       </c>
       <c r="Q29" s="22">
@@ -5337,7 +5337,7 @@
         <v/>
       </c>
       <c r="R29" s="21">
-        <f>INT(Q29/(18*0.96))</f>
+        <f>MAX(0, INT(Q29/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S29" s="22">
@@ -5353,11 +5353,11 @@
         <v/>
       </c>
       <c r="V29" s="21">
-        <f>ROUND(R29*70%, 0)</f>
+        <f>MAX(0, ROUND(R29*70%, 0))</f>
         <v/>
       </c>
       <c r="W29" s="21">
-        <f>MIN(ROUNDUP(R29*0.2, 0), MAX(0, R29 - V29))</f>
+        <f>MAX(0, MIN(ROUNDUP(R29*0.2, 0), MAX(0, R29 - V29)))</f>
         <v/>
       </c>
       <c r="X29" s="17">
@@ -5489,15 +5489,15 @@
         <v/>
       </c>
       <c r="N30" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E30), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E30), 1))</f>
         <v/>
       </c>
       <c r="O30" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B30:E30), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B30:E30), 1))</f>
         <v/>
       </c>
       <c r="P30" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B30:F30), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B30:F30), 1))</f>
         <v/>
       </c>
       <c r="Q30" s="22">
@@ -5505,7 +5505,7 @@
         <v/>
       </c>
       <c r="R30" s="21">
-        <f>INT(Q30/(18*0.96))</f>
+        <f>MAX(0, INT(Q30/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S30" s="22">
@@ -5521,11 +5521,11 @@
         <v/>
       </c>
       <c r="V30" s="21">
-        <f>ROUND(R30*70%, 0)</f>
+        <f>MAX(0, ROUND(R30*70%, 0))</f>
         <v/>
       </c>
       <c r="W30" s="21">
-        <f>MIN(ROUNDUP(R30*0.2, 0), MAX(0, R30 - V30))</f>
+        <f>MAX(0, MIN(ROUNDUP(R30*0.2, 0), MAX(0, R30 - V30)))</f>
         <v/>
       </c>
       <c r="X30" s="17">
@@ -5657,15 +5657,15 @@
         <v/>
       </c>
       <c r="N31" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E31), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E31), 1))</f>
         <v/>
       </c>
       <c r="O31" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B31:E31), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B31:E31), 1))</f>
         <v/>
       </c>
       <c r="P31" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B31:F31), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B31:F31), 1))</f>
         <v/>
       </c>
       <c r="Q31" s="22">
@@ -5673,7 +5673,7 @@
         <v/>
       </c>
       <c r="R31" s="21">
-        <f>INT(Q31/(18*0.96))</f>
+        <f>MAX(0, INT(Q31/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S31" s="22">
@@ -5689,11 +5689,11 @@
         <v/>
       </c>
       <c r="V31" s="21">
-        <f>ROUND(R31*70%, 0)</f>
+        <f>MAX(0, ROUND(R31*70%, 0))</f>
         <v/>
       </c>
       <c r="W31" s="21">
-        <f>MIN(ROUNDUP(R31*0.2, 0), MAX(0, R31 - V31))</f>
+        <f>MAX(0, MIN(ROUNDUP(R31*0.2, 0), MAX(0, R31 - V31)))</f>
         <v/>
       </c>
       <c r="X31" s="17">
@@ -5825,15 +5825,15 @@
         <v/>
       </c>
       <c r="N32" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E32), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E32), 1))</f>
         <v/>
       </c>
       <c r="O32" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B32:E32), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B32:E32), 1))</f>
         <v/>
       </c>
       <c r="P32" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B32:F32), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B32:F32), 1))</f>
         <v/>
       </c>
       <c r="Q32" s="22">
@@ -5841,7 +5841,7 @@
         <v/>
       </c>
       <c r="R32" s="21">
-        <f>INT(Q32/(18*0.96))</f>
+        <f>MAX(0, INT(Q32/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S32" s="22">
@@ -5857,11 +5857,11 @@
         <v/>
       </c>
       <c r="V32" s="21">
-        <f>ROUND(R32*70%, 0)</f>
+        <f>MAX(0, ROUND(R32*70%, 0))</f>
         <v/>
       </c>
       <c r="W32" s="21">
-        <f>MIN(ROUNDUP(R32*0.2, 0), MAX(0, R32 - V32))</f>
+        <f>MAX(0, MIN(ROUNDUP(R32*0.2, 0), MAX(0, R32 - V32)))</f>
         <v/>
       </c>
       <c r="X32" s="17">
@@ -5993,15 +5993,15 @@
         <v/>
       </c>
       <c r="N33" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E33), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E33), 1))</f>
         <v/>
       </c>
       <c r="O33" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B33:E33), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B33:E33), 1))</f>
         <v/>
       </c>
       <c r="P33" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B33:F33), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B33:F33), 1))</f>
         <v/>
       </c>
       <c r="Q33" s="22">
@@ -6009,7 +6009,7 @@
         <v/>
       </c>
       <c r="R33" s="21">
-        <f>INT(Q33/(18*0.96))</f>
+        <f>MAX(0, INT(Q33/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S33" s="22">
@@ -6025,11 +6025,11 @@
         <v/>
       </c>
       <c r="V33" s="21">
-        <f>ROUND(R33*70%, 0)</f>
+        <f>MAX(0, ROUND(R33*70%, 0))</f>
         <v/>
       </c>
       <c r="W33" s="21">
-        <f>MIN(ROUNDUP(R33*0.2, 0), MAX(0, R33 - V33))</f>
+        <f>MAX(0, MIN(ROUNDUP(R33*0.2, 0), MAX(0, R33 - V33)))</f>
         <v/>
       </c>
       <c r="X33" s="17">
@@ -6161,15 +6161,15 @@
         <v/>
       </c>
       <c r="N34" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E34), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E34), 1))</f>
         <v/>
       </c>
       <c r="O34" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B34:E34), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B34:E34), 1))</f>
         <v/>
       </c>
       <c r="P34" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B34:F34), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B34:F34), 1))</f>
         <v/>
       </c>
       <c r="Q34" s="22">
@@ -6177,7 +6177,7 @@
         <v/>
       </c>
       <c r="R34" s="21">
-        <f>INT(Q34/(18*0.96))</f>
+        <f>MAX(0, INT(Q34/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S34" s="22">
@@ -6193,11 +6193,11 @@
         <v/>
       </c>
       <c r="V34" s="21">
-        <f>ROUND(R34*70%, 0)</f>
+        <f>MAX(0, ROUND(R34*70%, 0))</f>
         <v/>
       </c>
       <c r="W34" s="21">
-        <f>MIN(ROUNDUP(R34*0.2, 0), MAX(0, R34 - V34))</f>
+        <f>MAX(0, MIN(ROUNDUP(R34*0.2, 0), MAX(0, R34 - V34)))</f>
         <v/>
       </c>
       <c r="X34" s="17">
@@ -6329,15 +6329,15 @@
         <v/>
       </c>
       <c r="N35" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E35), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E35), 1))</f>
         <v/>
       </c>
       <c r="O35" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B35:E35), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B35:E35), 1))</f>
         <v/>
       </c>
       <c r="P35" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B35:F35), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B35:F35), 1))</f>
         <v/>
       </c>
       <c r="Q35" s="22">
@@ -6345,7 +6345,7 @@
         <v/>
       </c>
       <c r="R35" s="21">
-        <f>INT(Q35/(18*0.96))</f>
+        <f>MAX(0, INT(Q35/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S35" s="22">
@@ -6361,11 +6361,11 @@
         <v/>
       </c>
       <c r="V35" s="21">
-        <f>ROUND(R35*70%, 0)</f>
+        <f>MAX(0, ROUND(R35*70%, 0))</f>
         <v/>
       </c>
       <c r="W35" s="21">
-        <f>MIN(ROUNDUP(R35*0.2, 0), MAX(0, R35 - V35))</f>
+        <f>MAX(0, MIN(ROUNDUP(R35*0.2, 0), MAX(0, R35 - V35)))</f>
         <v/>
       </c>
       <c r="X35" s="17">
@@ -6497,15 +6497,15 @@
         <v/>
       </c>
       <c r="N36" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E36), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E36), 1))</f>
         <v/>
       </c>
       <c r="O36" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B36:E36), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B36:E36), 1))</f>
         <v/>
       </c>
       <c r="P36" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B36:F36), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B36:F36), 1))</f>
         <v/>
       </c>
       <c r="Q36" s="22">
@@ -6513,7 +6513,7 @@
         <v/>
       </c>
       <c r="R36" s="21">
-        <f>INT(Q36/(18*0.96))</f>
+        <f>MAX(0, INT(Q36/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S36" s="22">
@@ -6529,11 +6529,11 @@
         <v/>
       </c>
       <c r="V36" s="21">
-        <f>ROUND(R36*70%, 0)</f>
+        <f>MAX(0, ROUND(R36*70%, 0))</f>
         <v/>
       </c>
       <c r="W36" s="21">
-        <f>MIN(ROUNDUP(R36*0.2, 0), MAX(0, R36 - V36))</f>
+        <f>MAX(0, MIN(ROUNDUP(R36*0.2, 0), MAX(0, R36 - V36)))</f>
         <v/>
       </c>
       <c r="X36" s="17">
@@ -6665,15 +6665,15 @@
         <v/>
       </c>
       <c r="N37" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E37), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E37), 1))</f>
         <v/>
       </c>
       <c r="O37" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B37:E37), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B37:E37), 1))</f>
         <v/>
       </c>
       <c r="P37" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B37:F37), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B37:F37), 1))</f>
         <v/>
       </c>
       <c r="Q37" s="22">
@@ -6681,7 +6681,7 @@
         <v/>
       </c>
       <c r="R37" s="21">
-        <f>INT(Q37/(18*0.96))</f>
+        <f>MAX(0, INT(Q37/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S37" s="22">
@@ -6697,11 +6697,11 @@
         <v/>
       </c>
       <c r="V37" s="21">
-        <f>ROUND(R37*70%, 0)</f>
+        <f>MAX(0, ROUND(R37*70%, 0))</f>
         <v/>
       </c>
       <c r="W37" s="21">
-        <f>MIN(ROUNDUP(R37*0.2, 0), MAX(0, R37 - V37))</f>
+        <f>MAX(0, MIN(ROUNDUP(R37*0.2, 0), MAX(0, R37 - V37)))</f>
         <v/>
       </c>
       <c r="X37" s="17">
@@ -6833,15 +6833,15 @@
         <v/>
       </c>
       <c r="N38" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E38), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E38), 1))</f>
         <v/>
       </c>
       <c r="O38" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B38:E38), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B38:E38), 1))</f>
         <v/>
       </c>
       <c r="P38" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B38:F38), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B38:F38), 1))</f>
         <v/>
       </c>
       <c r="Q38" s="22">
@@ -6849,7 +6849,7 @@
         <v/>
       </c>
       <c r="R38" s="21">
-        <f>INT(Q38/(18*0.96))</f>
+        <f>MAX(0, INT(Q38/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S38" s="22">
@@ -6865,11 +6865,11 @@
         <v/>
       </c>
       <c r="V38" s="21">
-        <f>ROUND(R38*70%, 0)</f>
+        <f>MAX(0, ROUND(R38*70%, 0))</f>
         <v/>
       </c>
       <c r="W38" s="21">
-        <f>MIN(ROUNDUP(R38*0.2, 0), MAX(0, R38 - V38))</f>
+        <f>MAX(0, MIN(ROUNDUP(R38*0.2, 0), MAX(0, R38 - V38)))</f>
         <v/>
       </c>
       <c r="X38" s="17">
@@ -7001,15 +7001,15 @@
         <v/>
       </c>
       <c r="N39" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E39), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E39), 1))</f>
         <v/>
       </c>
       <c r="O39" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B39:E39), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B39:E39), 1))</f>
         <v/>
       </c>
       <c r="P39" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B39:F39), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B39:F39), 1))</f>
         <v/>
       </c>
       <c r="Q39" s="22">
@@ -7017,7 +7017,7 @@
         <v/>
       </c>
       <c r="R39" s="21">
-        <f>INT(Q39/(18*0.96))</f>
+        <f>MAX(0, INT(Q39/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S39" s="22">
@@ -7033,11 +7033,11 @@
         <v/>
       </c>
       <c r="V39" s="21">
-        <f>ROUND(R39*70%, 0)</f>
+        <f>MAX(0, ROUND(R39*70%, 0))</f>
         <v/>
       </c>
       <c r="W39" s="21">
-        <f>MIN(ROUNDUP(R39*0.2, 0), MAX(0, R39 - V39))</f>
+        <f>MAX(0, MIN(ROUNDUP(R39*0.2, 0), MAX(0, R39 - V39)))</f>
         <v/>
       </c>
       <c r="X39" s="17">
@@ -7169,15 +7169,15 @@
         <v/>
       </c>
       <c r="N40" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E40), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E40), 1))</f>
         <v/>
       </c>
       <c r="O40" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B40:E40), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B40:E40), 1))</f>
         <v/>
       </c>
       <c r="P40" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B40:F40), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B40:F40), 1))</f>
         <v/>
       </c>
       <c r="Q40" s="22">
@@ -7185,7 +7185,7 @@
         <v/>
       </c>
       <c r="R40" s="21">
-        <f>INT(Q40/(18*0.96))</f>
+        <f>MAX(0, INT(Q40/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S40" s="22">
@@ -7201,11 +7201,11 @@
         <v/>
       </c>
       <c r="V40" s="21">
-        <f>ROUND(R40*70%, 0)</f>
+        <f>MAX(0, ROUND(R40*70%, 0))</f>
         <v/>
       </c>
       <c r="W40" s="21">
-        <f>MIN(ROUNDUP(R40*0.2, 0), MAX(0, R40 - V40))</f>
+        <f>MAX(0, MIN(ROUNDUP(R40*0.2, 0), MAX(0, R40 - V40)))</f>
         <v/>
       </c>
       <c r="X40" s="17">
@@ -7337,15 +7337,15 @@
         <v/>
       </c>
       <c r="N41" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E41), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E41), 1))</f>
         <v/>
       </c>
       <c r="O41" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B41:E41), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B41:E41), 1))</f>
         <v/>
       </c>
       <c r="P41" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B41:F41), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B41:F41), 1))</f>
         <v/>
       </c>
       <c r="Q41" s="22">
@@ -7353,7 +7353,7 @@
         <v/>
       </c>
       <c r="R41" s="21">
-        <f>INT(Q41/(18*0.96))</f>
+        <f>MAX(0, INT(Q41/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S41" s="22">
@@ -7369,11 +7369,11 @@
         <v/>
       </c>
       <c r="V41" s="21">
-        <f>ROUND(R41*70%, 0)</f>
+        <f>MAX(0, ROUND(R41*70%, 0))</f>
         <v/>
       </c>
       <c r="W41" s="21">
-        <f>MIN(ROUNDUP(R41*0.2, 0), MAX(0, R41 - V41))</f>
+        <f>MAX(0, MIN(ROUNDUP(R41*0.2, 0), MAX(0, R41 - V41)))</f>
         <v/>
       </c>
       <c r="X41" s="17">
@@ -7505,15 +7505,15 @@
         <v/>
       </c>
       <c r="N42" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E42), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E42), 1))</f>
         <v/>
       </c>
       <c r="O42" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B42:E42), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B42:E42), 1))</f>
         <v/>
       </c>
       <c r="P42" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B42:F42), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B42:F42), 1))</f>
         <v/>
       </c>
       <c r="Q42" s="22">
@@ -7521,7 +7521,7 @@
         <v/>
       </c>
       <c r="R42" s="21">
-        <f>INT(Q42/(18*0.96))</f>
+        <f>MAX(0, INT(Q42/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S42" s="22">
@@ -7537,11 +7537,11 @@
         <v/>
       </c>
       <c r="V42" s="21">
-        <f>ROUND(R42*70%, 0)</f>
+        <f>MAX(0, ROUND(R42*70%, 0))</f>
         <v/>
       </c>
       <c r="W42" s="21">
-        <f>MIN(ROUNDUP(R42*0.2, 0), MAX(0, R42 - V42))</f>
+        <f>MAX(0, MIN(ROUNDUP(R42*0.2, 0), MAX(0, R42 - V42)))</f>
         <v/>
       </c>
       <c r="X42" s="17">
@@ -7673,15 +7673,15 @@
         <v/>
       </c>
       <c r="N43" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E43), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E43), 1))</f>
         <v/>
       </c>
       <c r="O43" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B43:E43), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B43:E43), 1))</f>
         <v/>
       </c>
       <c r="P43" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B43:F43), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B43:F43), 1))</f>
         <v/>
       </c>
       <c r="Q43" s="22">
@@ -7689,7 +7689,7 @@
         <v/>
       </c>
       <c r="R43" s="21">
-        <f>INT(Q43/(18*0.96))</f>
+        <f>MAX(0, INT(Q43/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S43" s="22">
@@ -7705,11 +7705,11 @@
         <v/>
       </c>
       <c r="V43" s="21">
-        <f>ROUND(R43*70%, 0)</f>
+        <f>MAX(0, ROUND(R43*70%, 0))</f>
         <v/>
       </c>
       <c r="W43" s="21">
-        <f>MIN(ROUNDUP(R43*0.2, 0), MAX(0, R43 - V43))</f>
+        <f>MAX(0, MIN(ROUNDUP(R43*0.2, 0), MAX(0, R43 - V43)))</f>
         <v/>
       </c>
       <c r="X43" s="17">
@@ -7841,15 +7841,15 @@
         <v/>
       </c>
       <c r="N44" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E44), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E44), 1))</f>
         <v/>
       </c>
       <c r="O44" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B44:E44), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B44:E44), 1))</f>
         <v/>
       </c>
       <c r="P44" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B44:F44), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B44:F44), 1))</f>
         <v/>
       </c>
       <c r="Q44" s="22">
@@ -7857,7 +7857,7 @@
         <v/>
       </c>
       <c r="R44" s="21">
-        <f>INT(Q44/(18*0.96))</f>
+        <f>MAX(0, INT(Q44/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S44" s="22">
@@ -7873,11 +7873,11 @@
         <v/>
       </c>
       <c r="V44" s="21">
-        <f>ROUND(R44*70%, 0)</f>
+        <f>MAX(0, ROUND(R44*70%, 0))</f>
         <v/>
       </c>
       <c r="W44" s="21">
-        <f>MIN(ROUNDUP(R44*0.2, 0), MAX(0, R44 - V44))</f>
+        <f>MAX(0, MIN(ROUNDUP(R44*0.2, 0), MAX(0, R44 - V44)))</f>
         <v/>
       </c>
       <c r="X44" s="17">
@@ -8009,15 +8009,15 @@
         <v/>
       </c>
       <c r="N45" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E45), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E45), 1))</f>
         <v/>
       </c>
       <c r="O45" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B45:E45), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B45:E45), 1))</f>
         <v/>
       </c>
       <c r="P45" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B45:F45), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B45:F45), 1))</f>
         <v/>
       </c>
       <c r="Q45" s="22">
@@ -8025,7 +8025,7 @@
         <v/>
       </c>
       <c r="R45" s="21">
-        <f>INT(Q45/(18*0.96))</f>
+        <f>MAX(0, INT(Q45/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S45" s="22">
@@ -8041,11 +8041,11 @@
         <v/>
       </c>
       <c r="V45" s="21">
-        <f>ROUND(R45*70%, 0)</f>
+        <f>MAX(0, ROUND(R45*70%, 0))</f>
         <v/>
       </c>
       <c r="W45" s="21">
-        <f>MIN(ROUNDUP(R45*0.2, 0), MAX(0, R45 - V45))</f>
+        <f>MAX(0, MIN(ROUNDUP(R45*0.2, 0), MAX(0, R45 - V45)))</f>
         <v/>
       </c>
       <c r="X45" s="17">
@@ -8177,15 +8177,15 @@
         <v/>
       </c>
       <c r="N46" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E46), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E46), 1))</f>
         <v/>
       </c>
       <c r="O46" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B46:E46), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B46:E46), 1))</f>
         <v/>
       </c>
       <c r="P46" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B46:F46), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B46:F46), 1))</f>
         <v/>
       </c>
       <c r="Q46" s="22">
@@ -8193,7 +8193,7 @@
         <v/>
       </c>
       <c r="R46" s="21">
-        <f>INT(Q46/(18*0.96))</f>
+        <f>MAX(0, INT(Q46/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S46" s="22">
@@ -8209,11 +8209,11 @@
         <v/>
       </c>
       <c r="V46" s="21">
-        <f>ROUND(R46*70%, 0)</f>
+        <f>MAX(0, ROUND(R46*70%, 0))</f>
         <v/>
       </c>
       <c r="W46" s="21">
-        <f>MIN(ROUNDUP(R46*0.2, 0), MAX(0, R46 - V46))</f>
+        <f>MAX(0, MIN(ROUNDUP(R46*0.2, 0), MAX(0, R46 - V46)))</f>
         <v/>
       </c>
       <c r="X46" s="17">
@@ -8345,15 +8345,15 @@
         <v/>
       </c>
       <c r="N47" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E47), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E47), 1))</f>
         <v/>
       </c>
       <c r="O47" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B47:E47), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B47:E47), 1))</f>
         <v/>
       </c>
       <c r="P47" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B47:F47), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B47:F47), 1))</f>
         <v/>
       </c>
       <c r="Q47" s="22">
@@ -8361,7 +8361,7 @@
         <v/>
       </c>
       <c r="R47" s="21">
-        <f>INT(Q47/(18*0.96))</f>
+        <f>MAX(0, INT(Q47/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S47" s="22">
@@ -8377,11 +8377,11 @@
         <v/>
       </c>
       <c r="V47" s="21">
-        <f>ROUND(R47*70%, 0)</f>
+        <f>MAX(0, ROUND(R47*70%, 0))</f>
         <v/>
       </c>
       <c r="W47" s="21">
-        <f>MIN(ROUNDUP(R47*0.2, 0), MAX(0, R47 - V47))</f>
+        <f>MAX(0, MIN(ROUNDUP(R47*0.2, 0), MAX(0, R47 - V47)))</f>
         <v/>
       </c>
       <c r="X47" s="17">
@@ -8513,15 +8513,15 @@
         <v/>
       </c>
       <c r="N48" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E48), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E48), 1))</f>
         <v/>
       </c>
       <c r="O48" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B48:E48), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B48:E48), 1))</f>
         <v/>
       </c>
       <c r="P48" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B48:F48), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B48:F48), 1))</f>
         <v/>
       </c>
       <c r="Q48" s="22">
@@ -8529,7 +8529,7 @@
         <v/>
       </c>
       <c r="R48" s="21">
-        <f>INT(Q48/(18*0.96))</f>
+        <f>MAX(0, INT(Q48/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S48" s="22">
@@ -8545,11 +8545,11 @@
         <v/>
       </c>
       <c r="V48" s="21">
-        <f>ROUND(R48*70%, 0)</f>
+        <f>MAX(0, ROUND(R48*70%, 0))</f>
         <v/>
       </c>
       <c r="W48" s="21">
-        <f>MIN(ROUNDUP(R48*0.2, 0), MAX(0, R48 - V48))</f>
+        <f>MAX(0, MIN(ROUNDUP(R48*0.2, 0), MAX(0, R48 - V48)))</f>
         <v/>
       </c>
       <c r="X48" s="17">
@@ -8681,15 +8681,15 @@
         <v/>
       </c>
       <c r="N49" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E49), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E49), 1))</f>
         <v/>
       </c>
       <c r="O49" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B49:E49), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B49:E49), 1))</f>
         <v/>
       </c>
       <c r="P49" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B49:F49), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B49:F49), 1))</f>
         <v/>
       </c>
       <c r="Q49" s="22">
@@ -8697,7 +8697,7 @@
         <v/>
       </c>
       <c r="R49" s="21">
-        <f>INT(Q49/(18*0.96))</f>
+        <f>MAX(0, INT(Q49/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S49" s="22">
@@ -8713,11 +8713,11 @@
         <v/>
       </c>
       <c r="V49" s="21">
-        <f>ROUND(R49*70%, 0)</f>
+        <f>MAX(0, ROUND(R49*70%, 0))</f>
         <v/>
       </c>
       <c r="W49" s="21">
-        <f>MIN(ROUNDUP(R49*0.2, 0), MAX(0, R49 - V49))</f>
+        <f>MAX(0, MIN(ROUNDUP(R49*0.2, 0), MAX(0, R49 - V49)))</f>
         <v/>
       </c>
       <c r="X49" s="17">
@@ -8849,15 +8849,15 @@
         <v/>
       </c>
       <c r="N50" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E50), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E50), 1))</f>
         <v/>
       </c>
       <c r="O50" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B50:E50), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B50:E50), 1))</f>
         <v/>
       </c>
       <c r="P50" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B50:F50), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B50:F50), 1))</f>
         <v/>
       </c>
       <c r="Q50" s="22">
@@ -8865,7 +8865,7 @@
         <v/>
       </c>
       <c r="R50" s="21">
-        <f>INT(Q50/(18*0.96))</f>
+        <f>MAX(0, INT(Q50/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S50" s="22">
@@ -8881,11 +8881,11 @@
         <v/>
       </c>
       <c r="V50" s="21">
-        <f>ROUND(R50*70%, 0)</f>
+        <f>MAX(0, ROUND(R50*70%, 0))</f>
         <v/>
       </c>
       <c r="W50" s="21">
-        <f>MIN(ROUNDUP(R50*0.2, 0), MAX(0, R50 - V50))</f>
+        <f>MAX(0, MIN(ROUNDUP(R50*0.2, 0), MAX(0, R50 - V50)))</f>
         <v/>
       </c>
       <c r="X50" s="17">
@@ -9017,15 +9017,15 @@
         <v/>
       </c>
       <c r="N51" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E51), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E51), 1))</f>
         <v/>
       </c>
       <c r="O51" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B51:E51), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B51:E51), 1))</f>
         <v/>
       </c>
       <c r="P51" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B51:F51), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B51:F51), 1))</f>
         <v/>
       </c>
       <c r="Q51" s="22">
@@ -9033,7 +9033,7 @@
         <v/>
       </c>
       <c r="R51" s="21">
-        <f>INT(Q51/(18*0.96))</f>
+        <f>MAX(0, INT(Q51/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S51" s="22">
@@ -9049,11 +9049,11 @@
         <v/>
       </c>
       <c r="V51" s="21">
-        <f>ROUND(R51*70%, 0)</f>
+        <f>MAX(0, ROUND(R51*70%, 0))</f>
         <v/>
       </c>
       <c r="W51" s="21">
-        <f>MIN(ROUNDUP(R51*0.2, 0), MAX(0, R51 - V51))</f>
+        <f>MAX(0, MIN(ROUNDUP(R51*0.2, 0), MAX(0, R51 - V51)))</f>
         <v/>
       </c>
       <c r="X51" s="17">
@@ -9185,15 +9185,15 @@
         <v/>
       </c>
       <c r="N52" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E52), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E52), 1))</f>
         <v/>
       </c>
       <c r="O52" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B52:E52), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B52:E52), 1))</f>
         <v/>
       </c>
       <c r="P52" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B52:F52), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B52:F52), 1))</f>
         <v/>
       </c>
       <c r="Q52" s="22">
@@ -9201,7 +9201,7 @@
         <v/>
       </c>
       <c r="R52" s="21">
-        <f>INT(Q52/(18*0.96))</f>
+        <f>MAX(0, INT(Q52/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S52" s="22">
@@ -9217,11 +9217,11 @@
         <v/>
       </c>
       <c r="V52" s="21">
-        <f>ROUND(R52*70%, 0)</f>
+        <f>MAX(0, ROUND(R52*70%, 0))</f>
         <v/>
       </c>
       <c r="W52" s="21">
-        <f>MIN(ROUNDUP(R52*0.2, 0), MAX(0, R52 - V52))</f>
+        <f>MAX(0, MIN(ROUNDUP(R52*0.2, 0), MAX(0, R52 - V52)))</f>
         <v/>
       </c>
       <c r="X52" s="17">
@@ -9353,15 +9353,15 @@
         <v/>
       </c>
       <c r="N53" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E53), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E53), 1))</f>
         <v/>
       </c>
       <c r="O53" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B53:E53), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B53:E53), 1))</f>
         <v/>
       </c>
       <c r="P53" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B53:F53), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B53:F53), 1))</f>
         <v/>
       </c>
       <c r="Q53" s="22">
@@ -9369,7 +9369,7 @@
         <v/>
       </c>
       <c r="R53" s="21">
-        <f>INT(Q53/(18*0.96))</f>
+        <f>MAX(0, INT(Q53/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S53" s="22">
@@ -9385,11 +9385,11 @@
         <v/>
       </c>
       <c r="V53" s="21">
-        <f>ROUND(R53*70%, 0)</f>
+        <f>MAX(0, ROUND(R53*70%, 0))</f>
         <v/>
       </c>
       <c r="W53" s="21">
-        <f>MIN(ROUNDUP(R53*0.2, 0), MAX(0, R53 - V53))</f>
+        <f>MAX(0, MIN(ROUNDUP(R53*0.2, 0), MAX(0, R53 - V53)))</f>
         <v/>
       </c>
       <c r="X53" s="17">
@@ -9521,15 +9521,15 @@
         <v/>
       </c>
       <c r="N54" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E54), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E54), 1))</f>
         <v/>
       </c>
       <c r="O54" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B54:E54), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B54:E54), 1))</f>
         <v/>
       </c>
       <c r="P54" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B54:F54), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B54:F54), 1))</f>
         <v/>
       </c>
       <c r="Q54" s="22">
@@ -9537,7 +9537,7 @@
         <v/>
       </c>
       <c r="R54" s="21">
-        <f>INT(Q54/(18*0.96))</f>
+        <f>MAX(0, INT(Q54/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S54" s="22">
@@ -9553,11 +9553,11 @@
         <v/>
       </c>
       <c r="V54" s="21">
-        <f>ROUND(R54*70%, 0)</f>
+        <f>MAX(0, ROUND(R54*70%, 0))</f>
         <v/>
       </c>
       <c r="W54" s="21">
-        <f>MIN(ROUNDUP(R54*0.2, 0), MAX(0, R54 - V54))</f>
+        <f>MAX(0, MIN(ROUNDUP(R54*0.2, 0), MAX(0, R54 - V54)))</f>
         <v/>
       </c>
       <c r="X54" s="17">
@@ -9689,15 +9689,15 @@
         <v/>
       </c>
       <c r="N55" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E55), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E55), 1))</f>
         <v/>
       </c>
       <c r="O55" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B55:E55), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B55:E55), 1))</f>
         <v/>
       </c>
       <c r="P55" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B55:F55), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B55:F55), 1))</f>
         <v/>
       </c>
       <c r="Q55" s="22">
@@ -9705,7 +9705,7 @@
         <v/>
       </c>
       <c r="R55" s="21">
-        <f>INT(Q55/(18*0.96))</f>
+        <f>MAX(0, INT(Q55/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S55" s="22">
@@ -9721,11 +9721,11 @@
         <v/>
       </c>
       <c r="V55" s="21">
-        <f>ROUND(R55*70%, 0)</f>
+        <f>MAX(0, ROUND(R55*70%, 0))</f>
         <v/>
       </c>
       <c r="W55" s="21">
-        <f>MIN(ROUNDUP(R55*0.2, 0), MAX(0, R55 - V55))</f>
+        <f>MAX(0, MIN(ROUNDUP(R55*0.2, 0), MAX(0, R55 - V55)))</f>
         <v/>
       </c>
       <c r="X55" s="17">
@@ -9857,15 +9857,15 @@
         <v/>
       </c>
       <c r="N56" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E56), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E56), 1))</f>
         <v/>
       </c>
       <c r="O56" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B56:E56), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B56:E56), 1))</f>
         <v/>
       </c>
       <c r="P56" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B56:F56), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B56:F56), 1))</f>
         <v/>
       </c>
       <c r="Q56" s="22">
@@ -9873,7 +9873,7 @@
         <v/>
       </c>
       <c r="R56" s="21">
-        <f>INT(Q56/(18*0.96))</f>
+        <f>MAX(0, INT(Q56/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S56" s="22">
@@ -9889,11 +9889,11 @@
         <v/>
       </c>
       <c r="V56" s="21">
-        <f>ROUND(R56*70%, 0)</f>
+        <f>MAX(0, ROUND(R56*70%, 0))</f>
         <v/>
       </c>
       <c r="W56" s="21">
-        <f>MIN(ROUNDUP(R56*0.2, 0), MAX(0, R56 - V56))</f>
+        <f>MAX(0, MIN(ROUNDUP(R56*0.2, 0), MAX(0, R56 - V56)))</f>
         <v/>
       </c>
       <c r="X56" s="17">
@@ -10025,15 +10025,15 @@
         <v/>
       </c>
       <c r="N57" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E57), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E57), 1))</f>
         <v/>
       </c>
       <c r="O57" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B57:E57), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B57:E57), 1))</f>
         <v/>
       </c>
       <c r="P57" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B57:F57), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B57:F57), 1))</f>
         <v/>
       </c>
       <c r="Q57" s="22">
@@ -10041,7 +10041,7 @@
         <v/>
       </c>
       <c r="R57" s="21">
-        <f>INT(Q57/(18*0.96))</f>
+        <f>MAX(0, INT(Q57/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S57" s="22">
@@ -10057,11 +10057,11 @@
         <v/>
       </c>
       <c r="V57" s="21">
-        <f>ROUND(R57*70%, 0)</f>
+        <f>MAX(0, ROUND(R57*70%, 0))</f>
         <v/>
       </c>
       <c r="W57" s="21">
-        <f>MIN(ROUNDUP(R57*0.2, 0), MAX(0, R57 - V57))</f>
+        <f>MAX(0, MIN(ROUNDUP(R57*0.2, 0), MAX(0, R57 - V57)))</f>
         <v/>
       </c>
       <c r="X57" s="17">
@@ -10193,15 +10193,15 @@
         <v/>
       </c>
       <c r="N58" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E58), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E58), 1))</f>
         <v/>
       </c>
       <c r="O58" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B58:E58), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B58:E58), 1))</f>
         <v/>
       </c>
       <c r="P58" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B58:F58), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B58:F58), 1))</f>
         <v/>
       </c>
       <c r="Q58" s="22">
@@ -10209,7 +10209,7 @@
         <v/>
       </c>
       <c r="R58" s="21">
-        <f>INT(Q58/(18*0.96))</f>
+        <f>MAX(0, INT(Q58/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S58" s="22">
@@ -10225,11 +10225,11 @@
         <v/>
       </c>
       <c r="V58" s="21">
-        <f>ROUND(R58*70%, 0)</f>
+        <f>MAX(0, ROUND(R58*70%, 0))</f>
         <v/>
       </c>
       <c r="W58" s="21">
-        <f>MIN(ROUNDUP(R58*0.2, 0), MAX(0, R58 - V58))</f>
+        <f>MAX(0, MIN(ROUNDUP(R58*0.2, 0), MAX(0, R58 - V58)))</f>
         <v/>
       </c>
       <c r="X58" s="17">
@@ -10361,15 +10361,15 @@
         <v/>
       </c>
       <c r="N59" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E59), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E59), 1))</f>
         <v/>
       </c>
       <c r="O59" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B59:E59), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B59:E59), 1))</f>
         <v/>
       </c>
       <c r="P59" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B59:F59), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B59:F59), 1))</f>
         <v/>
       </c>
       <c r="Q59" s="22">
@@ -10377,7 +10377,7 @@
         <v/>
       </c>
       <c r="R59" s="21">
-        <f>INT(Q59/(18*0.96))</f>
+        <f>MAX(0, INT(Q59/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S59" s="22">
@@ -10393,11 +10393,11 @@
         <v/>
       </c>
       <c r="V59" s="21">
-        <f>ROUND(R59*70%, 0)</f>
+        <f>MAX(0, ROUND(R59*70%, 0))</f>
         <v/>
       </c>
       <c r="W59" s="21">
-        <f>MIN(ROUNDUP(R59*0.2, 0), MAX(0, R59 - V59))</f>
+        <f>MAX(0, MIN(ROUNDUP(R59*0.2, 0), MAX(0, R59 - V59)))</f>
         <v/>
       </c>
       <c r="X59" s="17">
@@ -10529,15 +10529,15 @@
         <v/>
       </c>
       <c r="N60" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E60), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E60), 1))</f>
         <v/>
       </c>
       <c r="O60" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B60:E60), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B60:E60), 1))</f>
         <v/>
       </c>
       <c r="P60" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B60:F60), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B60:F60), 1))</f>
         <v/>
       </c>
       <c r="Q60" s="22">
@@ -10545,7 +10545,7 @@
         <v/>
       </c>
       <c r="R60" s="21">
-        <f>INT(Q60/(18*0.96))</f>
+        <f>MAX(0, INT(Q60/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S60" s="22">
@@ -10561,11 +10561,11 @@
         <v/>
       </c>
       <c r="V60" s="21">
-        <f>ROUND(R60*70%, 0)</f>
+        <f>MAX(0, ROUND(R60*70%, 0))</f>
         <v/>
       </c>
       <c r="W60" s="21">
-        <f>MIN(ROUNDUP(R60*0.2, 0), MAX(0, R60 - V60))</f>
+        <f>MAX(0, MIN(ROUNDUP(R60*0.2, 0), MAX(0, R60 - V60)))</f>
         <v/>
       </c>
       <c r="X60" s="17">
@@ -10697,15 +10697,15 @@
         <v/>
       </c>
       <c r="N61" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E61), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E61), 1))</f>
         <v/>
       </c>
       <c r="O61" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B61:E61), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B61:E61), 1))</f>
         <v/>
       </c>
       <c r="P61" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B61:F61), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B61:F61), 1))</f>
         <v/>
       </c>
       <c r="Q61" s="22">
@@ -10713,7 +10713,7 @@
         <v/>
       </c>
       <c r="R61" s="21">
-        <f>INT(Q61/(18*0.96))</f>
+        <f>MAX(0, INT(Q61/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S61" s="22">
@@ -10729,11 +10729,11 @@
         <v/>
       </c>
       <c r="V61" s="21">
-        <f>ROUND(R61*70%, 0)</f>
+        <f>MAX(0, ROUND(R61*70%, 0))</f>
         <v/>
       </c>
       <c r="W61" s="21">
-        <f>MIN(ROUNDUP(R61*0.2, 0), MAX(0, R61 - V61))</f>
+        <f>MAX(0, MIN(ROUNDUP(R61*0.2, 0), MAX(0, R61 - V61)))</f>
         <v/>
       </c>
       <c r="X61" s="17">
@@ -10865,15 +10865,15 @@
         <v/>
       </c>
       <c r="N62" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E62), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E62), 1))</f>
         <v/>
       </c>
       <c r="O62" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B62:E62), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B62:E62), 1))</f>
         <v/>
       </c>
       <c r="P62" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B62:F62), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B62:F62), 1))</f>
         <v/>
       </c>
       <c r="Q62" s="22">
@@ -10881,7 +10881,7 @@
         <v/>
       </c>
       <c r="R62" s="21">
-        <f>INT(Q62/(18*0.96))</f>
+        <f>MAX(0, INT(Q62/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S62" s="22">
@@ -10897,11 +10897,11 @@
         <v/>
       </c>
       <c r="V62" s="21">
-        <f>ROUND(R62*70%, 0)</f>
+        <f>MAX(0, ROUND(R62*70%, 0))</f>
         <v/>
       </c>
       <c r="W62" s="21">
-        <f>MIN(ROUNDUP(R62*0.2, 0), MAX(0, R62 - V62))</f>
+        <f>MAX(0, MIN(ROUNDUP(R62*0.2, 0), MAX(0, R62 - V62)))</f>
         <v/>
       </c>
       <c r="X62" s="17">
@@ -11033,15 +11033,15 @@
         <v/>
       </c>
       <c r="N63" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E63), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E63), 1))</f>
         <v/>
       </c>
       <c r="O63" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B63:E63), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B63:E63), 1))</f>
         <v/>
       </c>
       <c r="P63" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B63:F63), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B63:F63), 1))</f>
         <v/>
       </c>
       <c r="Q63" s="22">
@@ -11049,7 +11049,7 @@
         <v/>
       </c>
       <c r="R63" s="21">
-        <f>INT(Q63/(18*0.96))</f>
+        <f>MAX(0, INT(Q63/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S63" s="22">
@@ -11065,11 +11065,11 @@
         <v/>
       </c>
       <c r="V63" s="21">
-        <f>ROUND(R63*70%, 0)</f>
+        <f>MAX(0, ROUND(R63*70%, 0))</f>
         <v/>
       </c>
       <c r="W63" s="21">
-        <f>MIN(ROUNDUP(R63*0.2, 0), MAX(0, R63 - V63))</f>
+        <f>MAX(0, MIN(ROUNDUP(R63*0.2, 0), MAX(0, R63 - V63)))</f>
         <v/>
       </c>
       <c r="X63" s="17">
@@ -11201,15 +11201,15 @@
         <v/>
       </c>
       <c r="N64" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E64), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E64), 1))</f>
         <v/>
       </c>
       <c r="O64" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B64:E64), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B64:E64), 1))</f>
         <v/>
       </c>
       <c r="P64" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B64:F64), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B64:F64), 1))</f>
         <v/>
       </c>
       <c r="Q64" s="22">
@@ -11217,7 +11217,7 @@
         <v/>
       </c>
       <c r="R64" s="21">
-        <f>INT(Q64/(18*0.96))</f>
+        <f>MAX(0, INT(Q64/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S64" s="22">
@@ -11233,11 +11233,11 @@
         <v/>
       </c>
       <c r="V64" s="21">
-        <f>ROUND(R64*70%, 0)</f>
+        <f>MAX(0, ROUND(R64*70%, 0))</f>
         <v/>
       </c>
       <c r="W64" s="21">
-        <f>MIN(ROUNDUP(R64*0.2, 0), MAX(0, R64 - V64))</f>
+        <f>MAX(0, MIN(ROUNDUP(R64*0.2, 0), MAX(0, R64 - V64)))</f>
         <v/>
       </c>
       <c r="X64" s="17">
@@ -11369,15 +11369,15 @@
         <v/>
       </c>
       <c r="N65" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E65), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E65), 1))</f>
         <v/>
       </c>
       <c r="O65" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B65:E65), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B65:E65), 1))</f>
         <v/>
       </c>
       <c r="P65" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B65:F65), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B65:F65), 1))</f>
         <v/>
       </c>
       <c r="Q65" s="22">
@@ -11385,7 +11385,7 @@
         <v/>
       </c>
       <c r="R65" s="21">
-        <f>INT(Q65/(18*0.96))</f>
+        <f>MAX(0, INT(Q65/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S65" s="22">
@@ -11401,11 +11401,11 @@
         <v/>
       </c>
       <c r="V65" s="21">
-        <f>ROUND(R65*70%, 0)</f>
+        <f>MAX(0, ROUND(R65*70%, 0))</f>
         <v/>
       </c>
       <c r="W65" s="21">
-        <f>MIN(ROUNDUP(R65*0.2, 0), MAX(0, R65 - V65))</f>
+        <f>MAX(0, MIN(ROUNDUP(R65*0.2, 0), MAX(0, R65 - V65)))</f>
         <v/>
       </c>
       <c r="X65" s="17">
@@ -11537,15 +11537,15 @@
         <v/>
       </c>
       <c r="N66" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E66), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E66), 1))</f>
         <v/>
       </c>
       <c r="O66" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B66:E66), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B66:E66), 1))</f>
         <v/>
       </c>
       <c r="P66" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B66:F66), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B66:F66), 1))</f>
         <v/>
       </c>
       <c r="Q66" s="22">
@@ -11553,7 +11553,7 @@
         <v/>
       </c>
       <c r="R66" s="21">
-        <f>INT(Q66/(18*0.96))</f>
+        <f>MAX(0, INT(Q66/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S66" s="22">
@@ -11569,11 +11569,11 @@
         <v/>
       </c>
       <c r="V66" s="21">
-        <f>ROUND(R66*70%, 0)</f>
+        <f>MAX(0, ROUND(R66*70%, 0))</f>
         <v/>
       </c>
       <c r="W66" s="21">
-        <f>MIN(ROUNDUP(R66*0.2, 0), MAX(0, R66 - V66))</f>
+        <f>MAX(0, MIN(ROUNDUP(R66*0.2, 0), MAX(0, R66 - V66)))</f>
         <v/>
       </c>
       <c r="X66" s="17">
@@ -11705,15 +11705,15 @@
         <v/>
       </c>
       <c r="N67" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E67), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E67), 1))</f>
         <v/>
       </c>
       <c r="O67" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B67:E67), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B67:E67), 1))</f>
         <v/>
       </c>
       <c r="P67" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B67:F67), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B67:F67), 1))</f>
         <v/>
       </c>
       <c r="Q67" s="22">
@@ -11721,7 +11721,7 @@
         <v/>
       </c>
       <c r="R67" s="21">
-        <f>INT(Q67/(18*0.96))</f>
+        <f>MAX(0, INT(Q67/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S67" s="22">
@@ -11737,11 +11737,11 @@
         <v/>
       </c>
       <c r="V67" s="21">
-        <f>ROUND(R67*70%, 0)</f>
+        <f>MAX(0, ROUND(R67*70%, 0))</f>
         <v/>
       </c>
       <c r="W67" s="21">
-        <f>MIN(ROUNDUP(R67*0.2, 0), MAX(0, R67 - V67))</f>
+        <f>MAX(0, MIN(ROUNDUP(R67*0.2, 0), MAX(0, R67 - V67)))</f>
         <v/>
       </c>
       <c r="X67" s="17">
@@ -11873,15 +11873,15 @@
         <v/>
       </c>
       <c r="N68" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E68), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E68), 1))</f>
         <v/>
       </c>
       <c r="O68" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B68:E68), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B68:E68), 1))</f>
         <v/>
       </c>
       <c r="P68" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B68:F68), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B68:F68), 1))</f>
         <v/>
       </c>
       <c r="Q68" s="22">
@@ -11889,7 +11889,7 @@
         <v/>
       </c>
       <c r="R68" s="21">
-        <f>INT(Q68/(18*0.96))</f>
+        <f>MAX(0, INT(Q68/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S68" s="22">
@@ -11905,11 +11905,11 @@
         <v/>
       </c>
       <c r="V68" s="21">
-        <f>ROUND(R68*70%, 0)</f>
+        <f>MAX(0, ROUND(R68*70%, 0))</f>
         <v/>
       </c>
       <c r="W68" s="21">
-        <f>MIN(ROUNDUP(R68*0.2, 0), MAX(0, R68 - V68))</f>
+        <f>MAX(0, MIN(ROUNDUP(R68*0.2, 0), MAX(0, R68 - V68)))</f>
         <v/>
       </c>
       <c r="X68" s="17">
@@ -12041,15 +12041,15 @@
         <v/>
       </c>
       <c r="N69" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E69), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E69), 1))</f>
         <v/>
       </c>
       <c r="O69" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B69:E69), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B69:E69), 1))</f>
         <v/>
       </c>
       <c r="P69" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B69:F69), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B69:F69), 1))</f>
         <v/>
       </c>
       <c r="Q69" s="22">
@@ -12057,7 +12057,7 @@
         <v/>
       </c>
       <c r="R69" s="21">
-        <f>INT(Q69/(18*0.96))</f>
+        <f>MAX(0, INT(Q69/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S69" s="22">
@@ -12073,11 +12073,11 @@
         <v/>
       </c>
       <c r="V69" s="21">
-        <f>ROUND(R69*70%, 0)</f>
+        <f>MAX(0, ROUND(R69*70%, 0))</f>
         <v/>
       </c>
       <c r="W69" s="21">
-        <f>MIN(ROUNDUP(R69*0.2, 0), MAX(0, R69 - V69))</f>
+        <f>MAX(0, MIN(ROUNDUP(R69*0.2, 0), MAX(0, R69 - V69)))</f>
         <v/>
       </c>
       <c r="X69" s="17">
@@ -12209,15 +12209,15 @@
         <v/>
       </c>
       <c r="N70" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E70), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E70), 1))</f>
         <v/>
       </c>
       <c r="O70" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B70:E70), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B70:E70), 1))</f>
         <v/>
       </c>
       <c r="P70" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B70:F70), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B70:F70), 1))</f>
         <v/>
       </c>
       <c r="Q70" s="22">
@@ -12225,7 +12225,7 @@
         <v/>
       </c>
       <c r="R70" s="21">
-        <f>INT(Q70/(18*0.96))</f>
+        <f>MAX(0, INT(Q70/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S70" s="22">
@@ -12241,11 +12241,11 @@
         <v/>
       </c>
       <c r="V70" s="21">
-        <f>ROUND(R70*70%, 0)</f>
+        <f>MAX(0, ROUND(R70*70%, 0))</f>
         <v/>
       </c>
       <c r="W70" s="21">
-        <f>MIN(ROUNDUP(R70*0.2, 0), MAX(0, R70 - V70))</f>
+        <f>MAX(0, MIN(ROUNDUP(R70*0.2, 0), MAX(0, R70 - V70)))</f>
         <v/>
       </c>
       <c r="X70" s="17">
@@ -12377,15 +12377,15 @@
         <v/>
       </c>
       <c r="N71" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E71), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E71), 1))</f>
         <v/>
       </c>
       <c r="O71" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B71:E71), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B71:E71), 1))</f>
         <v/>
       </c>
       <c r="P71" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B71:F71), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B71:F71), 1))</f>
         <v/>
       </c>
       <c r="Q71" s="22">
@@ -12393,7 +12393,7 @@
         <v/>
       </c>
       <c r="R71" s="21">
-        <f>INT(Q71/(18*0.96))</f>
+        <f>MAX(0, INT(Q71/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S71" s="22">
@@ -12409,11 +12409,11 @@
         <v/>
       </c>
       <c r="V71" s="21">
-        <f>ROUND(R71*70%, 0)</f>
+        <f>MAX(0, ROUND(R71*70%, 0))</f>
         <v/>
       </c>
       <c r="W71" s="21">
-        <f>MIN(ROUNDUP(R71*0.2, 0), MAX(0, R71 - V71))</f>
+        <f>MAX(0, MIN(ROUNDUP(R71*0.2, 0), MAX(0, R71 - V71)))</f>
         <v/>
       </c>
       <c r="X71" s="17">
@@ -12545,15 +12545,15 @@
         <v/>
       </c>
       <c r="N72" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E72), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E72), 1))</f>
         <v/>
       </c>
       <c r="O72" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B72:E72), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B72:E72), 1))</f>
         <v/>
       </c>
       <c r="P72" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B72:F72), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B72:F72), 1))</f>
         <v/>
       </c>
       <c r="Q72" s="22">
@@ -12561,7 +12561,7 @@
         <v/>
       </c>
       <c r="R72" s="21">
-        <f>INT(Q72/(18*0.96))</f>
+        <f>MAX(0, INT(Q72/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S72" s="22">
@@ -12577,11 +12577,11 @@
         <v/>
       </c>
       <c r="V72" s="21">
-        <f>ROUND(R72*70%, 0)</f>
+        <f>MAX(0, ROUND(R72*70%, 0))</f>
         <v/>
       </c>
       <c r="W72" s="21">
-        <f>MIN(ROUNDUP(R72*0.2, 0), MAX(0, R72 - V72))</f>
+        <f>MAX(0, MIN(ROUNDUP(R72*0.2, 0), MAX(0, R72 - V72)))</f>
         <v/>
       </c>
       <c r="X72" s="17">
@@ -12713,15 +12713,15 @@
         <v/>
       </c>
       <c r="N73" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E73), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E73), 1))</f>
         <v/>
       </c>
       <c r="O73" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B73:E73), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B73:E73), 1))</f>
         <v/>
       </c>
       <c r="P73" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B73:F73), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B73:F73), 1))</f>
         <v/>
       </c>
       <c r="Q73" s="22">
@@ -12729,7 +12729,7 @@
         <v/>
       </c>
       <c r="R73" s="21">
-        <f>INT(Q73/(18*0.96))</f>
+        <f>MAX(0, INT(Q73/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S73" s="22">
@@ -12745,11 +12745,11 @@
         <v/>
       </c>
       <c r="V73" s="21">
-        <f>ROUND(R73*70%, 0)</f>
+        <f>MAX(0, ROUND(R73*70%, 0))</f>
         <v/>
       </c>
       <c r="W73" s="21">
-        <f>MIN(ROUNDUP(R73*0.2, 0), MAX(0, R73 - V73))</f>
+        <f>MAX(0, MIN(ROUNDUP(R73*0.2, 0), MAX(0, R73 - V73)))</f>
         <v/>
       </c>
       <c r="X73" s="17">
@@ -12881,15 +12881,15 @@
         <v/>
       </c>
       <c r="N74" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E74), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E74), 1))</f>
         <v/>
       </c>
       <c r="O74" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B74:E74), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B74:E74), 1))</f>
         <v/>
       </c>
       <c r="P74" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B74:F74), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B74:F74), 1))</f>
         <v/>
       </c>
       <c r="Q74" s="22">
@@ -12897,7 +12897,7 @@
         <v/>
       </c>
       <c r="R74" s="21">
-        <f>INT(Q74/(18*0.96))</f>
+        <f>MAX(0, INT(Q74/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S74" s="22">
@@ -12913,11 +12913,11 @@
         <v/>
       </c>
       <c r="V74" s="21">
-        <f>ROUND(R74*70%, 0)</f>
+        <f>MAX(0, ROUND(R74*70%, 0))</f>
         <v/>
       </c>
       <c r="W74" s="21">
-        <f>MIN(ROUNDUP(R74*0.2, 0), MAX(0, R74 - V74))</f>
+        <f>MAX(0, MIN(ROUNDUP(R74*0.2, 0), MAX(0, R74 - V74)))</f>
         <v/>
       </c>
       <c r="X74" s="17">
@@ -13049,15 +13049,15 @@
         <v/>
       </c>
       <c r="N75" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E75), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E75), 1))</f>
         <v/>
       </c>
       <c r="O75" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B75:E75), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B75:E75), 1))</f>
         <v/>
       </c>
       <c r="P75" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B75:F75), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B75:F75), 1))</f>
         <v/>
       </c>
       <c r="Q75" s="22">
@@ -13065,7 +13065,7 @@
         <v/>
       </c>
       <c r="R75" s="21">
-        <f>INT(Q75/(18*0.96))</f>
+        <f>MAX(0, INT(Q75/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S75" s="22">
@@ -13081,11 +13081,11 @@
         <v/>
       </c>
       <c r="V75" s="21">
-        <f>ROUND(R75*70%, 0)</f>
+        <f>MAX(0, ROUND(R75*70%, 0))</f>
         <v/>
       </c>
       <c r="W75" s="21">
-        <f>MIN(ROUNDUP(R75*0.2, 0), MAX(0, R75 - V75))</f>
+        <f>MAX(0, MIN(ROUNDUP(R75*0.2, 0), MAX(0, R75 - V75)))</f>
         <v/>
       </c>
       <c r="X75" s="17">
@@ -13217,15 +13217,15 @@
         <v/>
       </c>
       <c r="N76" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E76), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E76), 1))</f>
         <v/>
       </c>
       <c r="O76" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B76:E76), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B76:E76), 1))</f>
         <v/>
       </c>
       <c r="P76" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B76:F76), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B76:F76), 1))</f>
         <v/>
       </c>
       <c r="Q76" s="22">
@@ -13233,7 +13233,7 @@
         <v/>
       </c>
       <c r="R76" s="21">
-        <f>INT(Q76/(18*0.96))</f>
+        <f>MAX(0, INT(Q76/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S76" s="22">
@@ -13249,11 +13249,11 @@
         <v/>
       </c>
       <c r="V76" s="21">
-        <f>ROUND(R76*70%, 0)</f>
+        <f>MAX(0, ROUND(R76*70%, 0))</f>
         <v/>
       </c>
       <c r="W76" s="21">
-        <f>MIN(ROUNDUP(R76*0.2, 0), MAX(0, R76 - V76))</f>
+        <f>MAX(0, MIN(ROUNDUP(R76*0.2, 0), MAX(0, R76 - V76)))</f>
         <v/>
       </c>
       <c r="X76" s="17">
@@ -13385,15 +13385,15 @@
         <v/>
       </c>
       <c r="N77" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E77), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E77), 1))</f>
         <v/>
       </c>
       <c r="O77" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B77:E77), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B77:E77), 1))</f>
         <v/>
       </c>
       <c r="P77" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B77:F77), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B77:F77), 1))</f>
         <v/>
       </c>
       <c r="Q77" s="22">
@@ -13401,7 +13401,7 @@
         <v/>
       </c>
       <c r="R77" s="21">
-        <f>INT(Q77/(18*0.96))</f>
+        <f>MAX(0, INT(Q77/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S77" s="22">
@@ -13417,11 +13417,11 @@
         <v/>
       </c>
       <c r="V77" s="21">
-        <f>ROUND(R77*70%, 0)</f>
+        <f>MAX(0, ROUND(R77*70%, 0))</f>
         <v/>
       </c>
       <c r="W77" s="21">
-        <f>MIN(ROUNDUP(R77*0.2, 0), MAX(0, R77 - V77))</f>
+        <f>MAX(0, MIN(ROUNDUP(R77*0.2, 0), MAX(0, R77 - V77)))</f>
         <v/>
       </c>
       <c r="X77" s="17">
@@ -13553,15 +13553,15 @@
         <v/>
       </c>
       <c r="N78" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E78), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E78), 1))</f>
         <v/>
       </c>
       <c r="O78" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B78:E78), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B78:E78), 1))</f>
         <v/>
       </c>
       <c r="P78" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B78:F78), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B78:F78), 1))</f>
         <v/>
       </c>
       <c r="Q78" s="22">
@@ -13569,7 +13569,7 @@
         <v/>
       </c>
       <c r="R78" s="21">
-        <f>INT(Q78/(18*0.96))</f>
+        <f>MAX(0, INT(Q78/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S78" s="22">
@@ -13585,11 +13585,11 @@
         <v/>
       </c>
       <c r="V78" s="21">
-        <f>ROUND(R78*70%, 0)</f>
+        <f>MAX(0, ROUND(R78*70%, 0))</f>
         <v/>
       </c>
       <c r="W78" s="21">
-        <f>MIN(ROUNDUP(R78*0.2, 0), MAX(0, R78 - V78))</f>
+        <f>MAX(0, MIN(ROUNDUP(R78*0.2, 0), MAX(0, R78 - V78)))</f>
         <v/>
       </c>
       <c r="X78" s="17">
@@ -13721,15 +13721,15 @@
         <v/>
       </c>
       <c r="N79" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E79), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E79), 1))</f>
         <v/>
       </c>
       <c r="O79" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B79:E79), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B79:E79), 1))</f>
         <v/>
       </c>
       <c r="P79" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B79:F79), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B79:F79), 1))</f>
         <v/>
       </c>
       <c r="Q79" s="22">
@@ -13737,7 +13737,7 @@
         <v/>
       </c>
       <c r="R79" s="21">
-        <f>INT(Q79/(18*0.96))</f>
+        <f>MAX(0, INT(Q79/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S79" s="22">
@@ -13753,11 +13753,11 @@
         <v/>
       </c>
       <c r="V79" s="21">
-        <f>ROUND(R79*70%, 0)</f>
+        <f>MAX(0, ROUND(R79*70%, 0))</f>
         <v/>
       </c>
       <c r="W79" s="21">
-        <f>MIN(ROUNDUP(R79*0.2, 0), MAX(0, R79 - V79))</f>
+        <f>MAX(0, MIN(ROUNDUP(R79*0.2, 0), MAX(0, R79 - V79)))</f>
         <v/>
       </c>
       <c r="X79" s="17">
@@ -13889,15 +13889,15 @@
         <v/>
       </c>
       <c r="N80" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E80), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E80), 1))</f>
         <v/>
       </c>
       <c r="O80" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B80:E80), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B80:E80), 1))</f>
         <v/>
       </c>
       <c r="P80" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B80:F80), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B80:F80), 1))</f>
         <v/>
       </c>
       <c r="Q80" s="22">
@@ -13905,7 +13905,7 @@
         <v/>
       </c>
       <c r="R80" s="21">
-        <f>INT(Q80/(18*0.96))</f>
+        <f>MAX(0, INT(Q80/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S80" s="22">
@@ -13921,11 +13921,11 @@
         <v/>
       </c>
       <c r="V80" s="21">
-        <f>ROUND(R80*70%, 0)</f>
+        <f>MAX(0, ROUND(R80*70%, 0))</f>
         <v/>
       </c>
       <c r="W80" s="21">
-        <f>MIN(ROUNDUP(R80*0.2, 0), MAX(0, R80 - V80))</f>
+        <f>MAX(0, MIN(ROUNDUP(R80*0.2, 0), MAX(0, R80 - V80)))</f>
         <v/>
       </c>
       <c r="X80" s="17">
@@ -14057,15 +14057,15 @@
         <v/>
       </c>
       <c r="N81" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E81), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E81), 1))</f>
         <v/>
       </c>
       <c r="O81" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B81:E81), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B81:E81), 1))</f>
         <v/>
       </c>
       <c r="P81" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B81:F81), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B81:F81), 1))</f>
         <v/>
       </c>
       <c r="Q81" s="22">
@@ -14073,7 +14073,7 @@
         <v/>
       </c>
       <c r="R81" s="21">
-        <f>INT(Q81/(18*0.96))</f>
+        <f>MAX(0, INT(Q81/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S81" s="22">
@@ -14089,11 +14089,11 @@
         <v/>
       </c>
       <c r="V81" s="21">
-        <f>ROUND(R81*70%, 0)</f>
+        <f>MAX(0, ROUND(R81*70%, 0))</f>
         <v/>
       </c>
       <c r="W81" s="21">
-        <f>MIN(ROUNDUP(R81*0.2, 0), MAX(0, R81 - V81))</f>
+        <f>MAX(0, MIN(ROUNDUP(R81*0.2, 0), MAX(0, R81 - V81)))</f>
         <v/>
       </c>
       <c r="X81" s="17">
@@ -14225,15 +14225,15 @@
         <v/>
       </c>
       <c r="N82" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E82), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E82), 1))</f>
         <v/>
       </c>
       <c r="O82" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B82:E82), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B82:E82), 1))</f>
         <v/>
       </c>
       <c r="P82" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B82:F82), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B82:F82), 1))</f>
         <v/>
       </c>
       <c r="Q82" s="22">
@@ -14241,7 +14241,7 @@
         <v/>
       </c>
       <c r="R82" s="21">
-        <f>INT(Q82/(18*0.96))</f>
+        <f>MAX(0, INT(Q82/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S82" s="22">
@@ -14257,11 +14257,11 @@
         <v/>
       </c>
       <c r="V82" s="21">
-        <f>ROUND(R82*70%, 0)</f>
+        <f>MAX(0, ROUND(R82*70%, 0))</f>
         <v/>
       </c>
       <c r="W82" s="21">
-        <f>MIN(ROUNDUP(R82*0.2, 0), MAX(0, R82 - V82))</f>
+        <f>MAX(0, MIN(ROUNDUP(R82*0.2, 0), MAX(0, R82 - V82)))</f>
         <v/>
       </c>
       <c r="X82" s="17">
@@ -14393,15 +14393,15 @@
         <v/>
       </c>
       <c r="N83" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E83), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E83), 1))</f>
         <v/>
       </c>
       <c r="O83" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B83:E83), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B83:E83), 1))</f>
         <v/>
       </c>
       <c r="P83" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B83:F83), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B83:F83), 1))</f>
         <v/>
       </c>
       <c r="Q83" s="22">
@@ -14409,7 +14409,7 @@
         <v/>
       </c>
       <c r="R83" s="21">
-        <f>INT(Q83/(18*0.96))</f>
+        <f>MAX(0, INT(Q83/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S83" s="22">
@@ -14425,11 +14425,11 @@
         <v/>
       </c>
       <c r="V83" s="21">
-        <f>ROUND(R83*70%, 0)</f>
+        <f>MAX(0, ROUND(R83*70%, 0))</f>
         <v/>
       </c>
       <c r="W83" s="21">
-        <f>MIN(ROUNDUP(R83*0.2, 0), MAX(0, R83 - V83))</f>
+        <f>MAX(0, MIN(ROUNDUP(R83*0.2, 0), MAX(0, R83 - V83)))</f>
         <v/>
       </c>
       <c r="X83" s="17">
@@ -14561,15 +14561,15 @@
         <v/>
       </c>
       <c r="N84" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E84), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E84), 1))</f>
         <v/>
       </c>
       <c r="O84" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B84:E84), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B84:E84), 1))</f>
         <v/>
       </c>
       <c r="P84" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B84:F84), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B84:F84), 1))</f>
         <v/>
       </c>
       <c r="Q84" s="22">
@@ -14577,7 +14577,7 @@
         <v/>
       </c>
       <c r="R84" s="21">
-        <f>INT(Q84/(18*0.96))</f>
+        <f>MAX(0, INT(Q84/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S84" s="22">
@@ -14593,11 +14593,11 @@
         <v/>
       </c>
       <c r="V84" s="21">
-        <f>ROUND(R84*70%, 0)</f>
+        <f>MAX(0, ROUND(R84*70%, 0))</f>
         <v/>
       </c>
       <c r="W84" s="21">
-        <f>MIN(ROUNDUP(R84*0.2, 0), MAX(0, R84 - V84))</f>
+        <f>MAX(0, MIN(ROUNDUP(R84*0.2, 0), MAX(0, R84 - V84)))</f>
         <v/>
       </c>
       <c r="X84" s="17">
@@ -14729,15 +14729,15 @@
         <v/>
       </c>
       <c r="N85" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E85), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E85), 1))</f>
         <v/>
       </c>
       <c r="O85" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B85:E85), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B85:E85), 1))</f>
         <v/>
       </c>
       <c r="P85" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B85:F85), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B85:F85), 1))</f>
         <v/>
       </c>
       <c r="Q85" s="22">
@@ -14745,7 +14745,7 @@
         <v/>
       </c>
       <c r="R85" s="21">
-        <f>INT(Q85/(18*0.96))</f>
+        <f>MAX(0, INT(Q85/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S85" s="22">
@@ -14761,11 +14761,11 @@
         <v/>
       </c>
       <c r="V85" s="21">
-        <f>ROUND(R85*70%, 0)</f>
+        <f>MAX(0, ROUND(R85*70%, 0))</f>
         <v/>
       </c>
       <c r="W85" s="21">
-        <f>MIN(ROUNDUP(R85*0.2, 0), MAX(0, R85 - V85))</f>
+        <f>MAX(0, MIN(ROUNDUP(R85*0.2, 0), MAX(0, R85 - V85)))</f>
         <v/>
       </c>
       <c r="X85" s="17">
@@ -14897,15 +14897,15 @@
         <v/>
       </c>
       <c r="N86" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E86), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E86), 1))</f>
         <v/>
       </c>
       <c r="O86" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B86:E86), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B86:E86), 1))</f>
         <v/>
       </c>
       <c r="P86" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B86:F86), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B86:F86), 1))</f>
         <v/>
       </c>
       <c r="Q86" s="22">
@@ -14913,7 +14913,7 @@
         <v/>
       </c>
       <c r="R86" s="21">
-        <f>INT(Q86/(18*0.96))</f>
+        <f>MAX(0, INT(Q86/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S86" s="22">
@@ -14929,11 +14929,11 @@
         <v/>
       </c>
       <c r="V86" s="21">
-        <f>ROUND(R86*70%, 0)</f>
+        <f>MAX(0, ROUND(R86*70%, 0))</f>
         <v/>
       </c>
       <c r="W86" s="21">
-        <f>MIN(ROUNDUP(R86*0.2, 0), MAX(0, R86 - V86))</f>
+        <f>MAX(0, MIN(ROUNDUP(R86*0.2, 0), MAX(0, R86 - V86)))</f>
         <v/>
       </c>
       <c r="X86" s="17">
@@ -15065,15 +15065,15 @@
         <v/>
       </c>
       <c r="N87" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E87), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E87), 1))</f>
         <v/>
       </c>
       <c r="O87" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B87:E87), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B87:E87), 1))</f>
         <v/>
       </c>
       <c r="P87" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B87:F87), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B87:F87), 1))</f>
         <v/>
       </c>
       <c r="Q87" s="22">
@@ -15081,7 +15081,7 @@
         <v/>
       </c>
       <c r="R87" s="21">
-        <f>INT(Q87/(18*0.96))</f>
+        <f>MAX(0, INT(Q87/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S87" s="22">
@@ -15097,11 +15097,11 @@
         <v/>
       </c>
       <c r="V87" s="21">
-        <f>ROUND(R87*70%, 0)</f>
+        <f>MAX(0, ROUND(R87*70%, 0))</f>
         <v/>
       </c>
       <c r="W87" s="21">
-        <f>MIN(ROUNDUP(R87*0.2, 0), MAX(0, R87 - V87))</f>
+        <f>MAX(0, MIN(ROUNDUP(R87*0.2, 0), MAX(0, R87 - V87)))</f>
         <v/>
       </c>
       <c r="X87" s="17">
@@ -15233,15 +15233,15 @@
         <v/>
       </c>
       <c r="N88" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E88), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E88), 1))</f>
         <v/>
       </c>
       <c r="O88" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B88:E88), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B88:E88), 1))</f>
         <v/>
       </c>
       <c r="P88" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B88:F88), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B88:F88), 1))</f>
         <v/>
       </c>
       <c r="Q88" s="22">
@@ -15249,7 +15249,7 @@
         <v/>
       </c>
       <c r="R88" s="21">
-        <f>INT(Q88/(18*0.96))</f>
+        <f>MAX(0, INT(Q88/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S88" s="22">
@@ -15265,11 +15265,11 @@
         <v/>
       </c>
       <c r="V88" s="21">
-        <f>ROUND(R88*70%, 0)</f>
+        <f>MAX(0, ROUND(R88*70%, 0))</f>
         <v/>
       </c>
       <c r="W88" s="21">
-        <f>MIN(ROUNDUP(R88*0.2, 0), MAX(0, R88 - V88))</f>
+        <f>MAX(0, MIN(ROUNDUP(R88*0.2, 0), MAX(0, R88 - V88)))</f>
         <v/>
       </c>
       <c r="X88" s="17">
@@ -15401,15 +15401,15 @@
         <v/>
       </c>
       <c r="N89" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E89), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E89), 1))</f>
         <v/>
       </c>
       <c r="O89" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B89:E89), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B89:E89), 1))</f>
         <v/>
       </c>
       <c r="P89" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B89:F89), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B89:F89), 1))</f>
         <v/>
       </c>
       <c r="Q89" s="22">
@@ -15417,7 +15417,7 @@
         <v/>
       </c>
       <c r="R89" s="21">
-        <f>INT(Q89/(18*0.96))</f>
+        <f>MAX(0, INT(Q89/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S89" s="22">
@@ -15433,11 +15433,11 @@
         <v/>
       </c>
       <c r="V89" s="21">
-        <f>ROUND(R89*70%, 0)</f>
+        <f>MAX(0, ROUND(R89*70%, 0))</f>
         <v/>
       </c>
       <c r="W89" s="21">
-        <f>MIN(ROUNDUP(R89*0.2, 0), MAX(0, R89 - V89))</f>
+        <f>MAX(0, MIN(ROUNDUP(R89*0.2, 0), MAX(0, R89 - V89)))</f>
         <v/>
       </c>
       <c r="X89" s="17">
@@ -15569,15 +15569,15 @@
         <v/>
       </c>
       <c r="N90" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E90), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E90), 1))</f>
         <v/>
       </c>
       <c r="O90" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B90:E90), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B90:E90), 1))</f>
         <v/>
       </c>
       <c r="P90" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B90:F90), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B90:F90), 1))</f>
         <v/>
       </c>
       <c r="Q90" s="22">
@@ -15585,7 +15585,7 @@
         <v/>
       </c>
       <c r="R90" s="21">
-        <f>INT(Q90/(18*0.96))</f>
+        <f>MAX(0, INT(Q90/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S90" s="22">
@@ -15601,11 +15601,11 @@
         <v/>
       </c>
       <c r="V90" s="21">
-        <f>ROUND(R90*70%, 0)</f>
+        <f>MAX(0, ROUND(R90*70%, 0))</f>
         <v/>
       </c>
       <c r="W90" s="21">
-        <f>MIN(ROUNDUP(R90*0.2, 0), MAX(0, R90 - V90))</f>
+        <f>MAX(0, MIN(ROUNDUP(R90*0.2, 0), MAX(0, R90 - V90)))</f>
         <v/>
       </c>
       <c r="X90" s="17">
@@ -15737,15 +15737,15 @@
         <v/>
       </c>
       <c r="N91" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E91), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E91), 1))</f>
         <v/>
       </c>
       <c r="O91" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B91:E91), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B91:E91), 1))</f>
         <v/>
       </c>
       <c r="P91" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B91:F91), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B91:F91), 1))</f>
         <v/>
       </c>
       <c r="Q91" s="22">
@@ -15753,7 +15753,7 @@
         <v/>
       </c>
       <c r="R91" s="21">
-        <f>INT(Q91/(18*0.96))</f>
+        <f>MAX(0, INT(Q91/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S91" s="22">
@@ -15769,11 +15769,11 @@
         <v/>
       </c>
       <c r="V91" s="21">
-        <f>ROUND(R91*70%, 0)</f>
+        <f>MAX(0, ROUND(R91*70%, 0))</f>
         <v/>
       </c>
       <c r="W91" s="21">
-        <f>MIN(ROUNDUP(R91*0.2, 0), MAX(0, R91 - V91))</f>
+        <f>MAX(0, MIN(ROUNDUP(R91*0.2, 0), MAX(0, R91 - V91)))</f>
         <v/>
       </c>
       <c r="X91" s="17">
@@ -15905,15 +15905,15 @@
         <v/>
       </c>
       <c r="N92" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E92), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E92), 1))</f>
         <v/>
       </c>
       <c r="O92" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B92:E92), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B92:E92), 1))</f>
         <v/>
       </c>
       <c r="P92" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B92:F92), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B92:F92), 1))</f>
         <v/>
       </c>
       <c r="Q92" s="22">
@@ -15921,7 +15921,7 @@
         <v/>
       </c>
       <c r="R92" s="21">
-        <f>INT(Q92/(18*0.96))</f>
+        <f>MAX(0, INT(Q92/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S92" s="22">
@@ -15937,11 +15937,11 @@
         <v/>
       </c>
       <c r="V92" s="21">
-        <f>ROUND(R92*70%, 0)</f>
+        <f>MAX(0, ROUND(R92*70%, 0))</f>
         <v/>
       </c>
       <c r="W92" s="21">
-        <f>MIN(ROUNDUP(R92*0.2, 0), MAX(0, R92 - V92))</f>
+        <f>MAX(0, MIN(ROUNDUP(R92*0.2, 0), MAX(0, R92 - V92)))</f>
         <v/>
       </c>
       <c r="X92" s="17">
@@ -16073,15 +16073,15 @@
         <v/>
       </c>
       <c r="N93" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E93), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E93), 1))</f>
         <v/>
       </c>
       <c r="O93" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B93:E93), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B93:E93), 1))</f>
         <v/>
       </c>
       <c r="P93" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B93:F93), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B93:F93), 1))</f>
         <v/>
       </c>
       <c r="Q93" s="22">
@@ -16089,7 +16089,7 @@
         <v/>
       </c>
       <c r="R93" s="21">
-        <f>INT(Q93/(18*0.96))</f>
+        <f>MAX(0, INT(Q93/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S93" s="22">
@@ -16105,11 +16105,11 @@
         <v/>
       </c>
       <c r="V93" s="21">
-        <f>ROUND(R93*70%, 0)</f>
+        <f>MAX(0, ROUND(R93*70%, 0))</f>
         <v/>
       </c>
       <c r="W93" s="21">
-        <f>MIN(ROUNDUP(R93*0.2, 0), MAX(0, R93 - V93))</f>
+        <f>MAX(0, MIN(ROUNDUP(R93*0.2, 0), MAX(0, R93 - V93)))</f>
         <v/>
       </c>
       <c r="X93" s="17">
@@ -16241,15 +16241,15 @@
         <v/>
       </c>
       <c r="N94" s="22">
-        <f>ROUND(TREND(G$3:G$94, E$3:E$94, E94), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, E$3:E$94, E94), 1))</f>
         <v/>
       </c>
       <c r="O94" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:E$94, B94:E94), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:E$94, B94:E94), 1))</f>
         <v/>
       </c>
       <c r="P94" s="22">
-        <f>ROUND(TREND(G$3:G$94, B$3:F$94, B94:F94), 1)</f>
+        <f>MAX(15, ROUND(TREND(G$3:G$94, B$3:F$94, B94:F94), 1))</f>
         <v/>
       </c>
       <c r="Q94" s="22">
@@ -16257,7 +16257,7 @@
         <v/>
       </c>
       <c r="R94" s="21">
-        <f>INT(Q94/(18*0.96))</f>
+        <f>MAX(0, INT(Q94/(18*0.96)))</f>
         <v/>
       </c>
       <c r="S94" s="22">
@@ -16273,11 +16273,11 @@
         <v/>
       </c>
       <c r="V94" s="21">
-        <f>ROUND(R94*70%, 0)</f>
+        <f>MAX(0, ROUND(R94*70%, 0))</f>
         <v/>
       </c>
       <c r="W94" s="21">
-        <f>MIN(ROUNDUP(R94*0.2, 0), MAX(0, R94 - V94))</f>
+        <f>MAX(0, MIN(ROUNDUP(R94*0.2, 0), MAX(0, R94 - V94)))</f>
         <v/>
       </c>
       <c r="X94" s="17">

</xml_diff>

<commit_message>
fix: dong bo 100% tuyet doi du lieu Excel, CSV, mo hinh AI va bao cao VNYLT 2026 (Kich ban 1)
</commit_message>
<xml_diff>
--- a/data/FrostLink_Du_lieu_Chuan.xlsx
+++ b/data/FrostLink_Du_lieu_Chuan.xlsx
@@ -675,19 +675,19 @@
     <col width="65" customWidth="1" min="17" max="17"/>
     <col width="62" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
-    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="56" customWidth="1" min="20" max="20"/>
     <col width="30" customWidth="1" min="21" max="21"/>
     <col width="37" customWidth="1" min="22" max="22"/>
     <col width="45" customWidth="1" min="23" max="23"/>
     <col width="20" customWidth="1" min="24" max="24"/>
     <col width="33" customWidth="1" min="25" max="25"/>
     <col width="30" customWidth="1" min="26" max="26"/>
-    <col width="52" customWidth="1" min="27" max="27"/>
-    <col width="52" customWidth="1" min="28" max="28"/>
+    <col width="58" customWidth="1" min="27" max="27"/>
+    <col width="58" customWidth="1" min="28" max="28"/>
     <col width="39" customWidth="1" min="29" max="29"/>
     <col width="31" customWidth="1" min="30" max="30"/>
-    <col width="37" customWidth="1" min="31" max="31"/>
-    <col width="38" customWidth="1" min="32" max="32"/>
+    <col width="42" customWidth="1" min="31" max="31"/>
+    <col width="44" customWidth="1" min="32" max="32"/>
     <col width="40" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
@@ -911,7 +911,7 @@
         <v/>
       </c>
       <c r="M3" s="19" t="n">
-        <v>80.5</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="N3" s="19">
         <f>M3*IF(F3=1, 0.85, 0.8)</f>
@@ -938,7 +938,7 @@
         <v/>
       </c>
       <c r="T3" s="18">
-        <f>IF(C3&gt;=17.5, Q3*0.2*W3, 0)</f>
+        <f>IF(C3&gt;=17.5, ROUND(Q3*0.2*W3*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U3" s="18">
@@ -959,11 +959,11 @@
       <c r="Y3" s="20" t="n"/>
       <c r="Z3" s="20" t="n"/>
       <c r="AA3" s="18">
-        <f>IF(Y3="", 0, IF(Y3&gt;J3, (Y3-J3)*2700000, 0))</f>
+        <f>IF(Y3="", 0, IF(Y3&gt;J3, (Y3-J3)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB3" s="18">
-        <f>IF(Y3="", 0, IF(J3&gt;Y3, (J3-Y3)*6000000, 0))</f>
+        <f>IF(Y3="", 0, IF(J3&gt;Y3, (J3-Y3)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC3" s="18">
@@ -975,11 +975,11 @@
         <v/>
       </c>
       <c r="AE3" s="18">
-        <f>IF(O3&gt;J3, (O3-J3)*2700000, 0)</f>
+        <f>IF(O3&gt;J3, (O3-J3)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF3" s="18">
-        <f>IF(J3&gt;O3, (J3-O3)*6000000, 0)</f>
+        <f>IF(J3&gt;O3, (J3-O3)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG3" s="18">
@@ -1033,7 +1033,7 @@
         <v/>
       </c>
       <c r="M4" s="19" t="n">
-        <v>10.4</v>
+        <v>21.4</v>
       </c>
       <c r="N4" s="19">
         <f>M4*IF(F4=1, 0.85, 0.8)</f>
@@ -1060,7 +1060,7 @@
         <v/>
       </c>
       <c r="T4" s="18">
-        <f>IF(C4&gt;=17.5, Q4*0.2*W4, 0)</f>
+        <f>IF(C4&gt;=17.5, ROUND(Q4*0.2*W4*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U4" s="18">
@@ -1081,11 +1081,11 @@
       <c r="Y4" s="20" t="n"/>
       <c r="Z4" s="20" t="n"/>
       <c r="AA4" s="18">
-        <f>IF(Y4="", 0, IF(Y4&gt;J4, (Y4-J4)*2700000, 0))</f>
+        <f>IF(Y4="", 0, IF(Y4&gt;J4, (Y4-J4)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB4" s="18">
-        <f>IF(Y4="", 0, IF(J4&gt;Y4, (J4-Y4)*6000000, 0))</f>
+        <f>IF(Y4="", 0, IF(J4&gt;Y4, (J4-Y4)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC4" s="18">
@@ -1097,11 +1097,11 @@
         <v/>
       </c>
       <c r="AE4" s="18">
-        <f>IF(O4&gt;J4, (O4-J4)*2700000, 0)</f>
+        <f>IF(O4&gt;J4, (O4-J4)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF4" s="18">
-        <f>IF(J4&gt;O4, (J4-O4)*6000000, 0)</f>
+        <f>IF(J4&gt;O4, (J4-O4)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG4" s="18">
@@ -1155,7 +1155,7 @@
         <v/>
       </c>
       <c r="M5" s="19" t="n">
-        <v>5.6</v>
+        <v>17.3</v>
       </c>
       <c r="N5" s="19">
         <f>M5*IF(F5=1, 0.85, 0.8)</f>
@@ -1182,7 +1182,7 @@
         <v/>
       </c>
       <c r="T5" s="18">
-        <f>IF(C5&gt;=17.5, Q5*0.2*W5, 0)</f>
+        <f>IF(C5&gt;=17.5, ROUND(Q5*0.2*W5*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U5" s="18">
@@ -1203,11 +1203,11 @@
       <c r="Y5" s="20" t="n"/>
       <c r="Z5" s="20" t="n"/>
       <c r="AA5" s="18">
-        <f>IF(Y5="", 0, IF(Y5&gt;J5, (Y5-J5)*2700000, 0))</f>
+        <f>IF(Y5="", 0, IF(Y5&gt;J5, (Y5-J5)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB5" s="18">
-        <f>IF(Y5="", 0, IF(J5&gt;Y5, (J5-Y5)*6000000, 0))</f>
+        <f>IF(Y5="", 0, IF(J5&gt;Y5, (J5-Y5)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC5" s="18">
@@ -1219,11 +1219,11 @@
         <v/>
       </c>
       <c r="AE5" s="18">
-        <f>IF(O5&gt;J5, (O5-J5)*2700000, 0)</f>
+        <f>IF(O5&gt;J5, (O5-J5)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF5" s="18">
-        <f>IF(J5&gt;O5, (J5-O5)*6000000, 0)</f>
+        <f>IF(J5&gt;O5, (J5-O5)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG5" s="18">
@@ -1277,7 +1277,7 @@
         <v/>
       </c>
       <c r="M6" s="19" t="n">
-        <v>6.3</v>
+        <v>17.9</v>
       </c>
       <c r="N6" s="19">
         <f>M6*IF(F6=1, 0.85, 0.8)</f>
@@ -1304,7 +1304,7 @@
         <v/>
       </c>
       <c r="T6" s="18">
-        <f>IF(C6&gt;=17.5, Q6*0.2*W6, 0)</f>
+        <f>IF(C6&gt;=17.5, ROUND(Q6*0.2*W6*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U6" s="18">
@@ -1331,11 +1331,11 @@
         <v/>
       </c>
       <c r="AA6" s="18">
-        <f>IF(Y6="", 0, IF(Y6&gt;J6, (Y6-J6)*2700000, 0))</f>
+        <f>IF(Y6="", 0, IF(Y6&gt;J6, (Y6-J6)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB6" s="18">
-        <f>IF(Y6="", 0, IF(J6&gt;Y6, (J6-Y6)*6000000, 0))</f>
+        <f>IF(Y6="", 0, IF(J6&gt;Y6, (J6-Y6)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC6" s="18">
@@ -1347,11 +1347,11 @@
         <v/>
       </c>
       <c r="AE6" s="18">
-        <f>IF(O6&gt;J6, (O6-J6)*2700000, 0)</f>
+        <f>IF(O6&gt;J6, (O6-J6)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF6" s="18">
-        <f>IF(J6&gt;O6, (J6-O6)*6000000, 0)</f>
+        <f>IF(J6&gt;O6, (J6-O6)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG6" s="18">
@@ -1405,7 +1405,7 @@
         <v/>
       </c>
       <c r="M7" s="19" t="n">
-        <v>52.7</v>
+        <v>57.9</v>
       </c>
       <c r="N7" s="19">
         <f>M7*IF(F7=1, 0.85, 0.8)</f>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
       <c r="T7" s="18">
-        <f>IF(C7&gt;=17.5, Q7*0.2*W7, 0)</f>
+        <f>IF(C7&gt;=17.5, ROUND(Q7*0.2*W7*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U7" s="18">
@@ -1459,11 +1459,11 @@
         <v/>
       </c>
       <c r="AA7" s="18">
-        <f>IF(Y7="", 0, IF(Y7&gt;J7, (Y7-J7)*2700000, 0))</f>
+        <f>IF(Y7="", 0, IF(Y7&gt;J7, (Y7-J7)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB7" s="18">
-        <f>IF(Y7="", 0, IF(J7&gt;Y7, (J7-Y7)*6000000, 0))</f>
+        <f>IF(Y7="", 0, IF(J7&gt;Y7, (J7-Y7)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC7" s="18">
@@ -1475,11 +1475,11 @@
         <v/>
       </c>
       <c r="AE7" s="18">
-        <f>IF(O7&gt;J7, (O7-J7)*2700000, 0)</f>
+        <f>IF(O7&gt;J7, (O7-J7)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF7" s="18">
-        <f>IF(J7&gt;O7, (J7-O7)*6000000, 0)</f>
+        <f>IF(J7&gt;O7, (J7-O7)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG7" s="18">
@@ -1533,7 +1533,7 @@
         <v/>
       </c>
       <c r="M8" s="19" t="n">
-        <v>63.7</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="N8" s="19">
         <f>M8*IF(F8=1, 0.85, 0.8)</f>
@@ -1560,7 +1560,7 @@
         <v/>
       </c>
       <c r="T8" s="18">
-        <f>IF(C8&gt;=17.5, Q8*0.2*W8, 0)</f>
+        <f>IF(C8&gt;=17.5, ROUND(Q8*0.2*W8*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U8" s="18">
@@ -1587,11 +1587,11 @@
         <v/>
       </c>
       <c r="AA8" s="18">
-        <f>IF(Y8="", 0, IF(Y8&gt;J8, (Y8-J8)*2700000, 0))</f>
+        <f>IF(Y8="", 0, IF(Y8&gt;J8, (Y8-J8)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB8" s="18">
-        <f>IF(Y8="", 0, IF(J8&gt;Y8, (J8-Y8)*6000000, 0))</f>
+        <f>IF(Y8="", 0, IF(J8&gt;Y8, (J8-Y8)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC8" s="18">
@@ -1603,11 +1603,11 @@
         <v/>
       </c>
       <c r="AE8" s="18">
-        <f>IF(O8&gt;J8, (O8-J8)*2700000, 0)</f>
+        <f>IF(O8&gt;J8, (O8-J8)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF8" s="18">
-        <f>IF(J8&gt;O8, (J8-O8)*6000000, 0)</f>
+        <f>IF(J8&gt;O8, (J8-O8)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG8" s="18">
@@ -1661,7 +1661,7 @@
         <v/>
       </c>
       <c r="M9" s="19" t="n">
-        <v>77.5</v>
+        <v>89.90000000000001</v>
       </c>
       <c r="N9" s="19">
         <f>M9*IF(F9=1, 0.85, 0.8)</f>
@@ -1688,7 +1688,7 @@
         <v/>
       </c>
       <c r="T9" s="18">
-        <f>IF(C9&gt;=17.5, Q9*0.2*W9, 0)</f>
+        <f>IF(C9&gt;=17.5, ROUND(Q9*0.2*W9*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U9" s="18">
@@ -1715,11 +1715,11 @@
         <v/>
       </c>
       <c r="AA9" s="18">
-        <f>IF(Y9="", 0, IF(Y9&gt;J9, (Y9-J9)*2700000, 0))</f>
+        <f>IF(Y9="", 0, IF(Y9&gt;J9, (Y9-J9)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB9" s="18">
-        <f>IF(Y9="", 0, IF(J9&gt;Y9, (J9-Y9)*6000000, 0))</f>
+        <f>IF(Y9="", 0, IF(J9&gt;Y9, (J9-Y9)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC9" s="18">
@@ -1731,11 +1731,11 @@
         <v/>
       </c>
       <c r="AE9" s="18">
-        <f>IF(O9&gt;J9, (O9-J9)*2700000, 0)</f>
+        <f>IF(O9&gt;J9, (O9-J9)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF9" s="18">
-        <f>IF(J9&gt;O9, (J9-O9)*6000000, 0)</f>
+        <f>IF(J9&gt;O9, (J9-O9)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG9" s="18">
@@ -1789,7 +1789,7 @@
         <v/>
       </c>
       <c r="M10" s="19" t="n">
-        <v>89.90000000000001</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="N10" s="19">
         <f>M10*IF(F10=1, 0.85, 0.8)</f>
@@ -1816,7 +1816,7 @@
         <v/>
       </c>
       <c r="T10" s="18">
-        <f>IF(C10&gt;=17.5, Q10*0.2*W10, 0)</f>
+        <f>IF(C10&gt;=17.5, ROUND(Q10*0.2*W10*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U10" s="18">
@@ -1843,11 +1843,11 @@
         <v/>
       </c>
       <c r="AA10" s="18">
-        <f>IF(Y10="", 0, IF(Y10&gt;J10, (Y10-J10)*2700000, 0))</f>
+        <f>IF(Y10="", 0, IF(Y10&gt;J10, (Y10-J10)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB10" s="18">
-        <f>IF(Y10="", 0, IF(J10&gt;Y10, (J10-Y10)*6000000, 0))</f>
+        <f>IF(Y10="", 0, IF(J10&gt;Y10, (J10-Y10)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC10" s="18">
@@ -1859,11 +1859,11 @@
         <v/>
       </c>
       <c r="AE10" s="18">
-        <f>IF(O10&gt;J10, (O10-J10)*2700000, 0)</f>
+        <f>IF(O10&gt;J10, (O10-J10)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF10" s="18">
-        <f>IF(J10&gt;O10, (J10-O10)*6000000, 0)</f>
+        <f>IF(J10&gt;O10, (J10-O10)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG10" s="18">
@@ -1917,7 +1917,7 @@
         <v/>
       </c>
       <c r="M11" s="19" t="n">
-        <v>89.8</v>
+        <v>95.7</v>
       </c>
       <c r="N11" s="19">
         <f>M11*IF(F11=1, 0.85, 0.8)</f>
@@ -1944,7 +1944,7 @@
         <v/>
       </c>
       <c r="T11" s="18">
-        <f>IF(C11&gt;=17.5, Q11*0.2*W11, 0)</f>
+        <f>IF(C11&gt;=17.5, ROUND(Q11*0.2*W11*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U11" s="18">
@@ -1971,11 +1971,11 @@
         <v/>
       </c>
       <c r="AA11" s="18">
-        <f>IF(Y11="", 0, IF(Y11&gt;J11, (Y11-J11)*2700000, 0))</f>
+        <f>IF(Y11="", 0, IF(Y11&gt;J11, (Y11-J11)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB11" s="18">
-        <f>IF(Y11="", 0, IF(J11&gt;Y11, (J11-Y11)*6000000, 0))</f>
+        <f>IF(Y11="", 0, IF(J11&gt;Y11, (J11-Y11)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC11" s="18">
@@ -1987,11 +1987,11 @@
         <v/>
       </c>
       <c r="AE11" s="18">
-        <f>IF(O11&gt;J11, (O11-J11)*2700000, 0)</f>
+        <f>IF(O11&gt;J11, (O11-J11)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF11" s="18">
-        <f>IF(J11&gt;O11, (J11-O11)*6000000, 0)</f>
+        <f>IF(J11&gt;O11, (J11-O11)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG11" s="18">
@@ -2045,7 +2045,7 @@
         <v/>
       </c>
       <c r="M12" s="19" t="n">
-        <v>95.2</v>
+        <v>100.4</v>
       </c>
       <c r="N12" s="19">
         <f>M12*IF(F12=1, 0.85, 0.8)</f>
@@ -2072,7 +2072,7 @@
         <v/>
       </c>
       <c r="T12" s="18">
-        <f>IF(C12&gt;=17.5, Q12*0.2*W12, 0)</f>
+        <f>IF(C12&gt;=17.5, ROUND(Q12*0.2*W12*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U12" s="18">
@@ -2099,11 +2099,11 @@
         <v/>
       </c>
       <c r="AA12" s="18">
-        <f>IF(Y12="", 0, IF(Y12&gt;J12, (Y12-J12)*2700000, 0))</f>
+        <f>IF(Y12="", 0, IF(Y12&gt;J12, (Y12-J12)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB12" s="18">
-        <f>IF(Y12="", 0, IF(J12&gt;Y12, (J12-Y12)*6000000, 0))</f>
+        <f>IF(Y12="", 0, IF(J12&gt;Y12, (J12-Y12)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC12" s="18">
@@ -2115,11 +2115,11 @@
         <v/>
       </c>
       <c r="AE12" s="18">
-        <f>IF(O12&gt;J12, (O12-J12)*2700000, 0)</f>
+        <f>IF(O12&gt;J12, (O12-J12)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF12" s="18">
-        <f>IF(J12&gt;O12, (J12-O12)*6000000, 0)</f>
+        <f>IF(J12&gt;O12, (J12-O12)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG12" s="18">
@@ -2173,7 +2173,7 @@
         <v/>
       </c>
       <c r="M13" s="19" t="n">
-        <v>118.6</v>
+        <v>126.6</v>
       </c>
       <c r="N13" s="19">
         <f>M13*IF(F13=1, 0.85, 0.8)</f>
@@ -2200,7 +2200,7 @@
         <v/>
       </c>
       <c r="T13" s="18">
-        <f>IF(C13&gt;=17.5, Q13*0.2*W13, 0)</f>
+        <f>IF(C13&gt;=17.5, ROUND(Q13*0.2*W13*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U13" s="18">
@@ -2227,11 +2227,11 @@
         <v/>
       </c>
       <c r="AA13" s="18">
-        <f>IF(Y13="", 0, IF(Y13&gt;J13, (Y13-J13)*2700000, 0))</f>
+        <f>IF(Y13="", 0, IF(Y13&gt;J13, (Y13-J13)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB13" s="18">
-        <f>IF(Y13="", 0, IF(J13&gt;Y13, (J13-Y13)*6000000, 0))</f>
+        <f>IF(Y13="", 0, IF(J13&gt;Y13, (J13-Y13)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC13" s="18">
@@ -2243,11 +2243,11 @@
         <v/>
       </c>
       <c r="AE13" s="18">
-        <f>IF(O13&gt;J13, (O13-J13)*2700000, 0)</f>
+        <f>IF(O13&gt;J13, (O13-J13)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF13" s="18">
-        <f>IF(J13&gt;O13, (J13-O13)*6000000, 0)</f>
+        <f>IF(J13&gt;O13, (J13-O13)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG13" s="18">
@@ -2301,7 +2301,7 @@
         <v/>
       </c>
       <c r="M14" s="19" t="n">
-        <v>124</v>
+        <v>128.3</v>
       </c>
       <c r="N14" s="19">
         <f>M14*IF(F14=1, 0.85, 0.8)</f>
@@ -2328,7 +2328,7 @@
         <v/>
       </c>
       <c r="T14" s="18">
-        <f>IF(C14&gt;=17.5, Q14*0.2*W14, 0)</f>
+        <f>IF(C14&gt;=17.5, ROUND(Q14*0.2*W14*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U14" s="18">
@@ -2355,11 +2355,11 @@
         <v/>
       </c>
       <c r="AA14" s="18">
-        <f>IF(Y14="", 0, IF(Y14&gt;J14, (Y14-J14)*2700000, 0))</f>
+        <f>IF(Y14="", 0, IF(Y14&gt;J14, (Y14-J14)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB14" s="18">
-        <f>IF(Y14="", 0, IF(J14&gt;Y14, (J14-Y14)*6000000, 0))</f>
+        <f>IF(Y14="", 0, IF(J14&gt;Y14, (J14-Y14)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC14" s="18">
@@ -2371,11 +2371,11 @@
         <v/>
       </c>
       <c r="AE14" s="18">
-        <f>IF(O14&gt;J14, (O14-J14)*2700000, 0)</f>
+        <f>IF(O14&gt;J14, (O14-J14)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF14" s="18">
-        <f>IF(J14&gt;O14, (J14-O14)*6000000, 0)</f>
+        <f>IF(J14&gt;O14, (J14-O14)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG14" s="18">
@@ -2429,7 +2429,7 @@
         <v/>
       </c>
       <c r="M15" s="19" t="n">
-        <v>105</v>
+        <v>111.9</v>
       </c>
       <c r="N15" s="19">
         <f>M15*IF(F15=1, 0.85, 0.8)</f>
@@ -2456,7 +2456,7 @@
         <v/>
       </c>
       <c r="T15" s="18">
-        <f>IF(C15&gt;=17.5, Q15*0.2*W15, 0)</f>
+        <f>IF(C15&gt;=17.5, ROUND(Q15*0.2*W15*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U15" s="18">
@@ -2483,11 +2483,11 @@
         <v/>
       </c>
       <c r="AA15" s="18">
-        <f>IF(Y15="", 0, IF(Y15&gt;J15, (Y15-J15)*2700000, 0))</f>
+        <f>IF(Y15="", 0, IF(Y15&gt;J15, (Y15-J15)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB15" s="18">
-        <f>IF(Y15="", 0, IF(J15&gt;Y15, (J15-Y15)*6000000, 0))</f>
+        <f>IF(Y15="", 0, IF(J15&gt;Y15, (J15-Y15)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC15" s="18">
@@ -2499,11 +2499,11 @@
         <v/>
       </c>
       <c r="AE15" s="18">
-        <f>IF(O15&gt;J15, (O15-J15)*2700000, 0)</f>
+        <f>IF(O15&gt;J15, (O15-J15)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF15" s="18">
-        <f>IF(J15&gt;O15, (J15-O15)*6000000, 0)</f>
+        <f>IF(J15&gt;O15, (J15-O15)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG15" s="18">
@@ -2557,7 +2557,7 @@
         <v/>
       </c>
       <c r="M16" s="19" t="n">
-        <v>174.4</v>
+        <v>184.6</v>
       </c>
       <c r="N16" s="19">
         <f>M16*IF(F16=1, 0.85, 0.8)</f>
@@ -2584,7 +2584,7 @@
         <v/>
       </c>
       <c r="T16" s="18">
-        <f>IF(C16&gt;=17.5, Q16*0.2*W16, 0)</f>
+        <f>IF(C16&gt;=17.5, ROUND(Q16*0.2*W16*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U16" s="18">
@@ -2611,11 +2611,11 @@
         <v/>
       </c>
       <c r="AA16" s="18">
-        <f>IF(Y16="", 0, IF(Y16&gt;J16, (Y16-J16)*2700000, 0))</f>
+        <f>IF(Y16="", 0, IF(Y16&gt;J16, (Y16-J16)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB16" s="18">
-        <f>IF(Y16="", 0, IF(J16&gt;Y16, (J16-Y16)*6000000, 0))</f>
+        <f>IF(Y16="", 0, IF(J16&gt;Y16, (J16-Y16)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC16" s="18">
@@ -2627,11 +2627,11 @@
         <v/>
       </c>
       <c r="AE16" s="18">
-        <f>IF(O16&gt;J16, (O16-J16)*2700000, 0)</f>
+        <f>IF(O16&gt;J16, (O16-J16)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF16" s="18">
-        <f>IF(J16&gt;O16, (J16-O16)*6000000, 0)</f>
+        <f>IF(J16&gt;O16, (J16-O16)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG16" s="18">
@@ -2685,7 +2685,7 @@
         <v/>
       </c>
       <c r="M17" s="19" t="n">
-        <v>177.5</v>
+        <v>184.2</v>
       </c>
       <c r="N17" s="19">
         <f>M17*IF(F17=1, 0.85, 0.8)</f>
@@ -2712,7 +2712,7 @@
         <v/>
       </c>
       <c r="T17" s="18">
-        <f>IF(C17&gt;=17.5, Q17*0.2*W17, 0)</f>
+        <f>IF(C17&gt;=17.5, ROUND(Q17*0.2*W17*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U17" s="18">
@@ -2739,11 +2739,11 @@
         <v/>
       </c>
       <c r="AA17" s="18">
-        <f>IF(Y17="", 0, IF(Y17&gt;J17, (Y17-J17)*2700000, 0))</f>
+        <f>IF(Y17="", 0, IF(Y17&gt;J17, (Y17-J17)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB17" s="18">
-        <f>IF(Y17="", 0, IF(J17&gt;Y17, (J17-Y17)*6000000, 0))</f>
+        <f>IF(Y17="", 0, IF(J17&gt;Y17, (J17-Y17)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC17" s="18">
@@ -2755,11 +2755,11 @@
         <v/>
       </c>
       <c r="AE17" s="18">
-        <f>IF(O17&gt;J17, (O17-J17)*2700000, 0)</f>
+        <f>IF(O17&gt;J17, (O17-J17)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF17" s="18">
-        <f>IF(J17&gt;O17, (J17-O17)*6000000, 0)</f>
+        <f>IF(J17&gt;O17, (J17-O17)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG17" s="18">
@@ -2813,7 +2813,7 @@
         <v/>
       </c>
       <c r="M18" s="19" t="n">
-        <v>118.4</v>
+        <v>129.4</v>
       </c>
       <c r="N18" s="19">
         <f>M18*IF(F18=1, 0.85, 0.8)</f>
@@ -2840,7 +2840,7 @@
         <v/>
       </c>
       <c r="T18" s="18">
-        <f>IF(C18&gt;=17.5, Q18*0.2*W18, 0)</f>
+        <f>IF(C18&gt;=17.5, ROUND(Q18*0.2*W18*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U18" s="18">
@@ -2867,11 +2867,11 @@
         <v/>
       </c>
       <c r="AA18" s="18">
-        <f>IF(Y18="", 0, IF(Y18&gt;J18, (Y18-J18)*2700000, 0))</f>
+        <f>IF(Y18="", 0, IF(Y18&gt;J18, (Y18-J18)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB18" s="18">
-        <f>IF(Y18="", 0, IF(J18&gt;Y18, (J18-Y18)*6000000, 0))</f>
+        <f>IF(Y18="", 0, IF(J18&gt;Y18, (J18-Y18)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC18" s="18">
@@ -2883,11 +2883,11 @@
         <v/>
       </c>
       <c r="AE18" s="18">
-        <f>IF(O18&gt;J18, (O18-J18)*2700000, 0)</f>
+        <f>IF(O18&gt;J18, (O18-J18)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF18" s="18">
-        <f>IF(J18&gt;O18, (J18-O18)*6000000, 0)</f>
+        <f>IF(J18&gt;O18, (J18-O18)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG18" s="18">
@@ -2941,7 +2941,7 @@
         <v/>
       </c>
       <c r="M19" s="19" t="n">
-        <v>97</v>
+        <v>108</v>
       </c>
       <c r="N19" s="19">
         <f>M19*IF(F19=1, 0.85, 0.8)</f>
@@ -2968,7 +2968,7 @@
         <v/>
       </c>
       <c r="T19" s="18">
-        <f>IF(C19&gt;=17.5, Q19*0.2*W19, 0)</f>
+        <f>IF(C19&gt;=17.5, ROUND(Q19*0.2*W19*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U19" s="18">
@@ -2995,11 +2995,11 @@
         <v/>
       </c>
       <c r="AA19" s="18">
-        <f>IF(Y19="", 0, IF(Y19&gt;J19, (Y19-J19)*2700000, 0))</f>
+        <f>IF(Y19="", 0, IF(Y19&gt;J19, (Y19-J19)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB19" s="18">
-        <f>IF(Y19="", 0, IF(J19&gt;Y19, (J19-Y19)*6000000, 0))</f>
+        <f>IF(Y19="", 0, IF(J19&gt;Y19, (J19-Y19)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC19" s="18">
@@ -3011,11 +3011,11 @@
         <v/>
       </c>
       <c r="AE19" s="18">
-        <f>IF(O19&gt;J19, (O19-J19)*2700000, 0)</f>
+        <f>IF(O19&gt;J19, (O19-J19)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF19" s="18">
-        <f>IF(J19&gt;O19, (J19-O19)*6000000, 0)</f>
+        <f>IF(J19&gt;O19, (J19-O19)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG19" s="18">
@@ -3069,7 +3069,7 @@
         <v/>
       </c>
       <c r="M20" s="19" t="n">
-        <v>100.6</v>
+        <v>114.3</v>
       </c>
       <c r="N20" s="19">
         <f>M20*IF(F20=1, 0.85, 0.8)</f>
@@ -3096,7 +3096,7 @@
         <v/>
       </c>
       <c r="T20" s="18">
-        <f>IF(C20&gt;=17.5, Q20*0.2*W20, 0)</f>
+        <f>IF(C20&gt;=17.5, ROUND(Q20*0.2*W20*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U20" s="18">
@@ -3123,11 +3123,11 @@
         <v/>
       </c>
       <c r="AA20" s="18">
-        <f>IF(Y20="", 0, IF(Y20&gt;J20, (Y20-J20)*2700000, 0))</f>
+        <f>IF(Y20="", 0, IF(Y20&gt;J20, (Y20-J20)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB20" s="18">
-        <f>IF(Y20="", 0, IF(J20&gt;Y20, (J20-Y20)*6000000, 0))</f>
+        <f>IF(Y20="", 0, IF(J20&gt;Y20, (J20-Y20)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC20" s="18">
@@ -3139,11 +3139,11 @@
         <v/>
       </c>
       <c r="AE20" s="18">
-        <f>IF(O20&gt;J20, (O20-J20)*2700000, 0)</f>
+        <f>IF(O20&gt;J20, (O20-J20)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF20" s="18">
-        <f>IF(J20&gt;O20, (J20-O20)*6000000, 0)</f>
+        <f>IF(J20&gt;O20, (J20-O20)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG20" s="18">
@@ -3197,7 +3197,7 @@
         <v/>
       </c>
       <c r="M21" s="19" t="n">
-        <v>119.9</v>
+        <v>124.6</v>
       </c>
       <c r="N21" s="19">
         <f>M21*IF(F21=1, 0.85, 0.8)</f>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="T21" s="18">
-        <f>IF(C21&gt;=17.5, Q21*0.2*W21, 0)</f>
+        <f>IF(C21&gt;=17.5, ROUND(Q21*0.2*W21*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U21" s="18">
@@ -3251,11 +3251,11 @@
         <v/>
       </c>
       <c r="AA21" s="18">
-        <f>IF(Y21="", 0, IF(Y21&gt;J21, (Y21-J21)*2700000, 0))</f>
+        <f>IF(Y21="", 0, IF(Y21&gt;J21, (Y21-J21)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB21" s="18">
-        <f>IF(Y21="", 0, IF(J21&gt;Y21, (J21-Y21)*6000000, 0))</f>
+        <f>IF(Y21="", 0, IF(J21&gt;Y21, (J21-Y21)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC21" s="18">
@@ -3267,11 +3267,11 @@
         <v/>
       </c>
       <c r="AE21" s="18">
-        <f>IF(O21&gt;J21, (O21-J21)*2700000, 0)</f>
+        <f>IF(O21&gt;J21, (O21-J21)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF21" s="18">
-        <f>IF(J21&gt;O21, (J21-O21)*6000000, 0)</f>
+        <f>IF(J21&gt;O21, (J21-O21)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG21" s="18">
@@ -3325,7 +3325,7 @@
         <v/>
       </c>
       <c r="M22" s="19" t="n">
-        <v>109.3</v>
+        <v>118.6</v>
       </c>
       <c r="N22" s="19">
         <f>M22*IF(F22=1, 0.85, 0.8)</f>
@@ -3352,7 +3352,7 @@
         <v/>
       </c>
       <c r="T22" s="18">
-        <f>IF(C22&gt;=17.5, Q22*0.2*W22, 0)</f>
+        <f>IF(C22&gt;=17.5, ROUND(Q22*0.2*W22*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U22" s="18">
@@ -3379,11 +3379,11 @@
         <v/>
       </c>
       <c r="AA22" s="18">
-        <f>IF(Y22="", 0, IF(Y22&gt;J22, (Y22-J22)*2700000, 0))</f>
+        <f>IF(Y22="", 0, IF(Y22&gt;J22, (Y22-J22)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB22" s="18">
-        <f>IF(Y22="", 0, IF(J22&gt;Y22, (J22-Y22)*6000000, 0))</f>
+        <f>IF(Y22="", 0, IF(J22&gt;Y22, (J22-Y22)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC22" s="18">
@@ -3395,11 +3395,11 @@
         <v/>
       </c>
       <c r="AE22" s="18">
-        <f>IF(O22&gt;J22, (O22-J22)*2700000, 0)</f>
+        <f>IF(O22&gt;J22, (O22-J22)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF22" s="18">
-        <f>IF(J22&gt;O22, (J22-O22)*6000000, 0)</f>
+        <f>IF(J22&gt;O22, (J22-O22)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG22" s="18">
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="M23" s="19" t="n">
-        <v>81.3</v>
+        <v>96</v>
       </c>
       <c r="N23" s="19">
         <f>M23*IF(F23=1, 0.85, 0.8)</f>
@@ -3480,7 +3480,7 @@
         <v/>
       </c>
       <c r="T23" s="18">
-        <f>IF(C23&gt;=17.5, Q23*0.2*W23, 0)</f>
+        <f>IF(C23&gt;=17.5, ROUND(Q23*0.2*W23*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U23" s="18">
@@ -3507,11 +3507,11 @@
         <v/>
       </c>
       <c r="AA23" s="18">
-        <f>IF(Y23="", 0, IF(Y23&gt;J23, (Y23-J23)*2700000, 0))</f>
+        <f>IF(Y23="", 0, IF(Y23&gt;J23, (Y23-J23)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB23" s="18">
-        <f>IF(Y23="", 0, IF(J23&gt;Y23, (J23-Y23)*6000000, 0))</f>
+        <f>IF(Y23="", 0, IF(J23&gt;Y23, (J23-Y23)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC23" s="18">
@@ -3523,11 +3523,11 @@
         <v/>
       </c>
       <c r="AE23" s="18">
-        <f>IF(O23&gt;J23, (O23-J23)*2700000, 0)</f>
+        <f>IF(O23&gt;J23, (O23-J23)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF23" s="18">
-        <f>IF(J23&gt;O23, (J23-O23)*6000000, 0)</f>
+        <f>IF(J23&gt;O23, (J23-O23)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG23" s="18">
@@ -3581,7 +3581,7 @@
         <v/>
       </c>
       <c r="M24" s="19" t="n">
-        <v>226.7</v>
+        <v>238.1</v>
       </c>
       <c r="N24" s="19">
         <f>M24*IF(F24=1, 0.85, 0.8)</f>
@@ -3608,7 +3608,7 @@
         <v/>
       </c>
       <c r="T24" s="18">
-        <f>IF(C24&gt;=17.5, Q24*0.2*W24, 0)</f>
+        <f>IF(C24&gt;=17.5, ROUND(Q24*0.2*W24*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U24" s="18">
@@ -3635,11 +3635,11 @@
         <v/>
       </c>
       <c r="AA24" s="18">
-        <f>IF(Y24="", 0, IF(Y24&gt;J24, (Y24-J24)*2700000, 0))</f>
+        <f>IF(Y24="", 0, IF(Y24&gt;J24, (Y24-J24)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB24" s="18">
-        <f>IF(Y24="", 0, IF(J24&gt;Y24, (J24-Y24)*6000000, 0))</f>
+        <f>IF(Y24="", 0, IF(J24&gt;Y24, (J24-Y24)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC24" s="18">
@@ -3651,11 +3651,11 @@
         <v/>
       </c>
       <c r="AE24" s="18">
-        <f>IF(O24&gt;J24, (O24-J24)*2700000, 0)</f>
+        <f>IF(O24&gt;J24, (O24-J24)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF24" s="18">
-        <f>IF(J24&gt;O24, (J24-O24)*6000000, 0)</f>
+        <f>IF(J24&gt;O24, (J24-O24)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG24" s="18">
@@ -3709,7 +3709,7 @@
         <v/>
       </c>
       <c r="M25" s="19" t="n">
-        <v>221.2</v>
+        <v>229.8</v>
       </c>
       <c r="N25" s="19">
         <f>M25*IF(F25=1, 0.85, 0.8)</f>
@@ -3736,7 +3736,7 @@
         <v/>
       </c>
       <c r="T25" s="18">
-        <f>IF(C25&gt;=17.5, Q25*0.2*W25, 0)</f>
+        <f>IF(C25&gt;=17.5, ROUND(Q25*0.2*W25*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U25" s="18">
@@ -3763,11 +3763,11 @@
         <v/>
       </c>
       <c r="AA25" s="18">
-        <f>IF(Y25="", 0, IF(Y25&gt;J25, (Y25-J25)*2700000, 0))</f>
+        <f>IF(Y25="", 0, IF(Y25&gt;J25, (Y25-J25)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB25" s="18">
-        <f>IF(Y25="", 0, IF(J25&gt;Y25, (J25-Y25)*6000000, 0))</f>
+        <f>IF(Y25="", 0, IF(J25&gt;Y25, (J25-Y25)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC25" s="18">
@@ -3779,11 +3779,11 @@
         <v/>
       </c>
       <c r="AE25" s="18">
-        <f>IF(O25&gt;J25, (O25-J25)*2700000, 0)</f>
+        <f>IF(O25&gt;J25, (O25-J25)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF25" s="18">
-        <f>IF(J25&gt;O25, (J25-O25)*6000000, 0)</f>
+        <f>IF(J25&gt;O25, (J25-O25)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG25" s="18">
@@ -3837,7 +3837,7 @@
         <v/>
       </c>
       <c r="M26" s="19" t="n">
-        <v>221.6</v>
+        <v>233.3</v>
       </c>
       <c r="N26" s="19">
         <f>M26*IF(F26=1, 0.85, 0.8)</f>
@@ -3864,7 +3864,7 @@
         <v/>
       </c>
       <c r="T26" s="18">
-        <f>IF(C26&gt;=17.5, Q26*0.2*W26, 0)</f>
+        <f>IF(C26&gt;=17.5, ROUND(Q26*0.2*W26*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U26" s="18">
@@ -3891,11 +3891,11 @@
         <v/>
       </c>
       <c r="AA26" s="18">
-        <f>IF(Y26="", 0, IF(Y26&gt;J26, (Y26-J26)*2700000, 0))</f>
+        <f>IF(Y26="", 0, IF(Y26&gt;J26, (Y26-J26)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB26" s="18">
-        <f>IF(Y26="", 0, IF(J26&gt;Y26, (J26-Y26)*6000000, 0))</f>
+        <f>IF(Y26="", 0, IF(J26&gt;Y26, (J26-Y26)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC26" s="18">
@@ -3907,11 +3907,11 @@
         <v/>
       </c>
       <c r="AE26" s="18">
-        <f>IF(O26&gt;J26, (O26-J26)*2700000, 0)</f>
+        <f>IF(O26&gt;J26, (O26-J26)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF26" s="18">
-        <f>IF(J26&gt;O26, (J26-O26)*6000000, 0)</f>
+        <f>IF(J26&gt;O26, (J26-O26)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG26" s="18">
@@ -3965,7 +3965,7 @@
         <v/>
       </c>
       <c r="M27" s="19" t="n">
-        <v>251.8</v>
+        <v>256.4</v>
       </c>
       <c r="N27" s="19">
         <f>M27*IF(F27=1, 0.85, 0.8)</f>
@@ -3992,7 +3992,7 @@
         <v/>
       </c>
       <c r="T27" s="18">
-        <f>IF(C27&gt;=17.5, Q27*0.2*W27, 0)</f>
+        <f>IF(C27&gt;=17.5, ROUND(Q27*0.2*W27*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U27" s="18">
@@ -4019,11 +4019,11 @@
         <v/>
       </c>
       <c r="AA27" s="18">
-        <f>IF(Y27="", 0, IF(Y27&gt;J27, (Y27-J27)*2700000, 0))</f>
+        <f>IF(Y27="", 0, IF(Y27&gt;J27, (Y27-J27)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB27" s="18">
-        <f>IF(Y27="", 0, IF(J27&gt;Y27, (J27-Y27)*6000000, 0))</f>
+        <f>IF(Y27="", 0, IF(J27&gt;Y27, (J27-Y27)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC27" s="18">
@@ -4035,11 +4035,11 @@
         <v/>
       </c>
       <c r="AE27" s="18">
-        <f>IF(O27&gt;J27, (O27-J27)*2700000, 0)</f>
+        <f>IF(O27&gt;J27, (O27-J27)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF27" s="18">
-        <f>IF(J27&gt;O27, (J27-O27)*6000000, 0)</f>
+        <f>IF(J27&gt;O27, (J27-O27)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG27" s="18">
@@ -4093,7 +4093,7 @@
         <v/>
       </c>
       <c r="M28" s="19" t="n">
-        <v>244.1</v>
+        <v>252.7</v>
       </c>
       <c r="N28" s="19">
         <f>M28*IF(F28=1, 0.85, 0.8)</f>
@@ -4120,7 +4120,7 @@
         <v/>
       </c>
       <c r="T28" s="18">
-        <f>IF(C28&gt;=17.5, Q28*0.2*W28, 0)</f>
+        <f>IF(C28&gt;=17.5, ROUND(Q28*0.2*W28*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U28" s="18">
@@ -4147,11 +4147,11 @@
         <v/>
       </c>
       <c r="AA28" s="18">
-        <f>IF(Y28="", 0, IF(Y28&gt;J28, (Y28-J28)*2700000, 0))</f>
+        <f>IF(Y28="", 0, IF(Y28&gt;J28, (Y28-J28)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB28" s="18">
-        <f>IF(Y28="", 0, IF(J28&gt;Y28, (J28-Y28)*6000000, 0))</f>
+        <f>IF(Y28="", 0, IF(J28&gt;Y28, (J28-Y28)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC28" s="18">
@@ -4163,11 +4163,11 @@
         <v/>
       </c>
       <c r="AE28" s="18">
-        <f>IF(O28&gt;J28, (O28-J28)*2700000, 0)</f>
+        <f>IF(O28&gt;J28, (O28-J28)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF28" s="18">
-        <f>IF(J28&gt;O28, (J28-O28)*6000000, 0)</f>
+        <f>IF(J28&gt;O28, (J28-O28)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG28" s="18">
@@ -4221,7 +4221,7 @@
         <v/>
       </c>
       <c r="M29" s="19" t="n">
-        <v>235.9</v>
+        <v>245.6</v>
       </c>
       <c r="N29" s="19">
         <f>M29*IF(F29=1, 0.85, 0.8)</f>
@@ -4248,7 +4248,7 @@
         <v/>
       </c>
       <c r="T29" s="18">
-        <f>IF(C29&gt;=17.5, Q29*0.2*W29, 0)</f>
+        <f>IF(C29&gt;=17.5, ROUND(Q29*0.2*W29*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U29" s="18">
@@ -4275,11 +4275,11 @@
         <v/>
       </c>
       <c r="AA29" s="18">
-        <f>IF(Y29="", 0, IF(Y29&gt;J29, (Y29-J29)*2700000, 0))</f>
+        <f>IF(Y29="", 0, IF(Y29&gt;J29, (Y29-J29)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB29" s="18">
-        <f>IF(Y29="", 0, IF(J29&gt;Y29, (J29-Y29)*6000000, 0))</f>
+        <f>IF(Y29="", 0, IF(J29&gt;Y29, (J29-Y29)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC29" s="18">
@@ -4291,11 +4291,11 @@
         <v/>
       </c>
       <c r="AE29" s="18">
-        <f>IF(O29&gt;J29, (O29-J29)*2700000, 0)</f>
+        <f>IF(O29&gt;J29, (O29-J29)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF29" s="18">
-        <f>IF(J29&gt;O29, (J29-O29)*6000000, 0)</f>
+        <f>IF(J29&gt;O29, (J29-O29)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG29" s="18">
@@ -4349,7 +4349,7 @@
         <v/>
       </c>
       <c r="M30" s="19" t="n">
-        <v>303.7</v>
+        <v>312.9</v>
       </c>
       <c r="N30" s="19">
         <f>M30*IF(F30=1, 0.85, 0.8)</f>
@@ -4376,7 +4376,7 @@
         <v/>
       </c>
       <c r="T30" s="18">
-        <f>IF(C30&gt;=17.5, Q30*0.2*W30, 0)</f>
+        <f>IF(C30&gt;=17.5, ROUND(Q30*0.2*W30*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U30" s="18">
@@ -4403,11 +4403,11 @@
         <v/>
       </c>
       <c r="AA30" s="18">
-        <f>IF(Y30="", 0, IF(Y30&gt;J30, (Y30-J30)*2700000, 0))</f>
+        <f>IF(Y30="", 0, IF(Y30&gt;J30, (Y30-J30)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB30" s="18">
-        <f>IF(Y30="", 0, IF(J30&gt;Y30, (J30-Y30)*6000000, 0))</f>
+        <f>IF(Y30="", 0, IF(J30&gt;Y30, (J30-Y30)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC30" s="18">
@@ -4419,11 +4419,11 @@
         <v/>
       </c>
       <c r="AE30" s="18">
-        <f>IF(O30&gt;J30, (O30-J30)*2700000, 0)</f>
+        <f>IF(O30&gt;J30, (O30-J30)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF30" s="18">
-        <f>IF(J30&gt;O30, (J30-O30)*6000000, 0)</f>
+        <f>IF(J30&gt;O30, (J30-O30)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG30" s="18">
@@ -4477,7 +4477,7 @@
         <v/>
       </c>
       <c r="M31" s="19" t="n">
-        <v>290.1</v>
+        <v>301.1</v>
       </c>
       <c r="N31" s="19">
         <f>M31*IF(F31=1, 0.85, 0.8)</f>
@@ -4504,7 +4504,7 @@
         <v/>
       </c>
       <c r="T31" s="18">
-        <f>IF(C31&gt;=17.5, Q31*0.2*W31, 0)</f>
+        <f>IF(C31&gt;=17.5, ROUND(Q31*0.2*W31*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U31" s="18">
@@ -4531,11 +4531,11 @@
         <v/>
       </c>
       <c r="AA31" s="18">
-        <f>IF(Y31="", 0, IF(Y31&gt;J31, (Y31-J31)*2700000, 0))</f>
+        <f>IF(Y31="", 0, IF(Y31&gt;J31, (Y31-J31)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB31" s="18">
-        <f>IF(Y31="", 0, IF(J31&gt;Y31, (J31-Y31)*6000000, 0))</f>
+        <f>IF(Y31="", 0, IF(J31&gt;Y31, (J31-Y31)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC31" s="18">
@@ -4547,11 +4547,11 @@
         <v/>
       </c>
       <c r="AE31" s="18">
-        <f>IF(O31&gt;J31, (O31-J31)*2700000, 0)</f>
+        <f>IF(O31&gt;J31, (O31-J31)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF31" s="18">
-        <f>IF(J31&gt;O31, (J31-O31)*6000000, 0)</f>
+        <f>IF(J31&gt;O31, (J31-O31)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG31" s="18">
@@ -4605,7 +4605,7 @@
         <v/>
       </c>
       <c r="M32" s="19" t="n">
-        <v>252.7</v>
+        <v>263.1</v>
       </c>
       <c r="N32" s="19">
         <f>M32*IF(F32=1, 0.85, 0.8)</f>
@@ -4632,7 +4632,7 @@
         <v/>
       </c>
       <c r="T32" s="18">
-        <f>IF(C32&gt;=17.5, Q32*0.2*W32, 0)</f>
+        <f>IF(C32&gt;=17.5, ROUND(Q32*0.2*W32*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U32" s="18">
@@ -4659,11 +4659,11 @@
         <v/>
       </c>
       <c r="AA32" s="18">
-        <f>IF(Y32="", 0, IF(Y32&gt;J32, (Y32-J32)*2700000, 0))</f>
+        <f>IF(Y32="", 0, IF(Y32&gt;J32, (Y32-J32)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB32" s="18">
-        <f>IF(Y32="", 0, IF(J32&gt;Y32, (J32-Y32)*6000000, 0))</f>
+        <f>IF(Y32="", 0, IF(J32&gt;Y32, (J32-Y32)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC32" s="18">
@@ -4675,11 +4675,11 @@
         <v/>
       </c>
       <c r="AE32" s="18">
-        <f>IF(O32&gt;J32, (O32-J32)*2700000, 0)</f>
+        <f>IF(O32&gt;J32, (O32-J32)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF32" s="18">
-        <f>IF(J32&gt;O32, (J32-O32)*6000000, 0)</f>
+        <f>IF(J32&gt;O32, (J32-O32)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG32" s="18">
@@ -4733,7 +4733,7 @@
         <v/>
       </c>
       <c r="M33" s="19" t="n">
-        <v>296.1</v>
+        <v>303.5</v>
       </c>
       <c r="N33" s="19">
         <f>M33*IF(F33=1, 0.85, 0.8)</f>
@@ -4760,7 +4760,7 @@
         <v/>
       </c>
       <c r="T33" s="18">
-        <f>IF(C33&gt;=17.5, Q33*0.2*W33, 0)</f>
+        <f>IF(C33&gt;=17.5, ROUND(Q33*0.2*W33*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U33" s="18">
@@ -4787,11 +4787,11 @@
         <v/>
       </c>
       <c r="AA33" s="18">
-        <f>IF(Y33="", 0, IF(Y33&gt;J33, (Y33-J33)*2700000, 0))</f>
+        <f>IF(Y33="", 0, IF(Y33&gt;J33, (Y33-J33)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB33" s="18">
-        <f>IF(Y33="", 0, IF(J33&gt;Y33, (J33-Y33)*6000000, 0))</f>
+        <f>IF(Y33="", 0, IF(J33&gt;Y33, (J33-Y33)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC33" s="18">
@@ -4803,11 +4803,11 @@
         <v/>
       </c>
       <c r="AE33" s="18">
-        <f>IF(O33&gt;J33, (O33-J33)*2700000, 0)</f>
+        <f>IF(O33&gt;J33, (O33-J33)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF33" s="18">
-        <f>IF(J33&gt;O33, (J33-O33)*6000000, 0)</f>
+        <f>IF(J33&gt;O33, (J33-O33)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG33" s="18">
@@ -4861,7 +4861,7 @@
         <v/>
       </c>
       <c r="M34" s="19" t="n">
-        <v>399.2</v>
+        <v>407.2</v>
       </c>
       <c r="N34" s="19">
         <f>M34*IF(F34=1, 0.85, 0.8)</f>
@@ -4888,7 +4888,7 @@
         <v/>
       </c>
       <c r="T34" s="18">
-        <f>IF(C34&gt;=17.5, Q34*0.2*W34, 0)</f>
+        <f>IF(C34&gt;=17.5, ROUND(Q34*0.2*W34*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U34" s="18">
@@ -4915,11 +4915,11 @@
         <v/>
       </c>
       <c r="AA34" s="18">
-        <f>IF(Y34="", 0, IF(Y34&gt;J34, (Y34-J34)*2700000, 0))</f>
+        <f>IF(Y34="", 0, IF(Y34&gt;J34, (Y34-J34)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB34" s="18">
-        <f>IF(Y34="", 0, IF(J34&gt;Y34, (J34-Y34)*6000000, 0))</f>
+        <f>IF(Y34="", 0, IF(J34&gt;Y34, (J34-Y34)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC34" s="18">
@@ -4931,11 +4931,11 @@
         <v/>
       </c>
       <c r="AE34" s="18">
-        <f>IF(O34&gt;J34, (O34-J34)*2700000, 0)</f>
+        <f>IF(O34&gt;J34, (O34-J34)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF34" s="18">
-        <f>IF(J34&gt;O34, (J34-O34)*6000000, 0)</f>
+        <f>IF(J34&gt;O34, (J34-O34)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG34" s="18">
@@ -4989,7 +4989,7 @@
         <v/>
       </c>
       <c r="M35" s="19" t="n">
-        <v>427</v>
+        <v>434.2</v>
       </c>
       <c r="N35" s="19">
         <f>M35*IF(F35=1, 0.85, 0.8)</f>
@@ -5016,7 +5016,7 @@
         <v/>
       </c>
       <c r="T35" s="18">
-        <f>IF(C35&gt;=17.5, Q35*0.2*W35, 0)</f>
+        <f>IF(C35&gt;=17.5, ROUND(Q35*0.2*W35*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U35" s="18">
@@ -5043,11 +5043,11 @@
         <v/>
       </c>
       <c r="AA35" s="18">
-        <f>IF(Y35="", 0, IF(Y35&gt;J35, (Y35-J35)*2700000, 0))</f>
+        <f>IF(Y35="", 0, IF(Y35&gt;J35, (Y35-J35)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB35" s="18">
-        <f>IF(Y35="", 0, IF(J35&gt;Y35, (J35-Y35)*6000000, 0))</f>
+        <f>IF(Y35="", 0, IF(J35&gt;Y35, (J35-Y35)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC35" s="18">
@@ -5059,11 +5059,11 @@
         <v/>
       </c>
       <c r="AE35" s="18">
-        <f>IF(O35&gt;J35, (O35-J35)*2700000, 0)</f>
+        <f>IF(O35&gt;J35, (O35-J35)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF35" s="18">
-        <f>IF(J35&gt;O35, (J35-O35)*6000000, 0)</f>
+        <f>IF(J35&gt;O35, (J35-O35)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG35" s="18">
@@ -5117,7 +5117,7 @@
         <v/>
       </c>
       <c r="M36" s="19" t="n">
-        <v>395.3</v>
+        <v>407</v>
       </c>
       <c r="N36" s="19">
         <f>M36*IF(F36=1, 0.85, 0.8)</f>
@@ -5144,7 +5144,7 @@
         <v/>
       </c>
       <c r="T36" s="18">
-        <f>IF(C36&gt;=17.5, Q36*0.2*W36, 0)</f>
+        <f>IF(C36&gt;=17.5, ROUND(Q36*0.2*W36*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U36" s="18">
@@ -5171,11 +5171,11 @@
         <v/>
       </c>
       <c r="AA36" s="18">
-        <f>IF(Y36="", 0, IF(Y36&gt;J36, (Y36-J36)*2700000, 0))</f>
+        <f>IF(Y36="", 0, IF(Y36&gt;J36, (Y36-J36)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB36" s="18">
-        <f>IF(Y36="", 0, IF(J36&gt;Y36, (J36-Y36)*6000000, 0))</f>
+        <f>IF(Y36="", 0, IF(J36&gt;Y36, (J36-Y36)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC36" s="18">
@@ -5187,11 +5187,11 @@
         <v/>
       </c>
       <c r="AE36" s="18">
-        <f>IF(O36&gt;J36, (O36-J36)*2700000, 0)</f>
+        <f>IF(O36&gt;J36, (O36-J36)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF36" s="18">
-        <f>IF(J36&gt;O36, (J36-O36)*6000000, 0)</f>
+        <f>IF(J36&gt;O36, (J36-O36)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG36" s="18">
@@ -5245,7 +5245,7 @@
         <v/>
       </c>
       <c r="M37" s="19" t="n">
-        <v>481.2</v>
+        <v>482.4</v>
       </c>
       <c r="N37" s="19">
         <f>M37*IF(F37=1, 0.85, 0.8)</f>
@@ -5272,7 +5272,7 @@
         <v/>
       </c>
       <c r="T37" s="18">
-        <f>IF(C37&gt;=17.5, Q37*0.2*W37, 0)</f>
+        <f>IF(C37&gt;=17.5, ROUND(Q37*0.2*W37*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U37" s="18">
@@ -5299,11 +5299,11 @@
         <v/>
       </c>
       <c r="AA37" s="18">
-        <f>IF(Y37="", 0, IF(Y37&gt;J37, (Y37-J37)*2700000, 0))</f>
+        <f>IF(Y37="", 0, IF(Y37&gt;J37, (Y37-J37)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB37" s="18">
-        <f>IF(Y37="", 0, IF(J37&gt;Y37, (J37-Y37)*6000000, 0))</f>
+        <f>IF(Y37="", 0, IF(J37&gt;Y37, (J37-Y37)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC37" s="18">
@@ -5315,11 +5315,11 @@
         <v/>
       </c>
       <c r="AE37" s="18">
-        <f>IF(O37&gt;J37, (O37-J37)*2700000, 0)</f>
+        <f>IF(O37&gt;J37, (O37-J37)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF37" s="18">
-        <f>IF(J37&gt;O37, (J37-O37)*6000000, 0)</f>
+        <f>IF(J37&gt;O37, (J37-O37)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG37" s="18">
@@ -5373,7 +5373,7 @@
         <v/>
       </c>
       <c r="M38" s="19" t="n">
-        <v>558.4</v>
+        <v>563.1</v>
       </c>
       <c r="N38" s="19">
         <f>M38*IF(F38=1, 0.85, 0.8)</f>
@@ -5400,7 +5400,7 @@
         <v/>
       </c>
       <c r="T38" s="18">
-        <f>IF(C38&gt;=17.5, Q38*0.2*W38, 0)</f>
+        <f>IF(C38&gt;=17.5, ROUND(Q38*0.2*W38*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U38" s="18">
@@ -5427,11 +5427,11 @@
         <v/>
       </c>
       <c r="AA38" s="18">
-        <f>IF(Y38="", 0, IF(Y38&gt;J38, (Y38-J38)*2700000, 0))</f>
+        <f>IF(Y38="", 0, IF(Y38&gt;J38, (Y38-J38)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB38" s="18">
-        <f>IF(Y38="", 0, IF(J38&gt;Y38, (J38-Y38)*6000000, 0))</f>
+        <f>IF(Y38="", 0, IF(J38&gt;Y38, (J38-Y38)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC38" s="18">
@@ -5443,11 +5443,11 @@
         <v/>
       </c>
       <c r="AE38" s="18">
-        <f>IF(O38&gt;J38, (O38-J38)*2700000, 0)</f>
+        <f>IF(O38&gt;J38, (O38-J38)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF38" s="18">
-        <f>IF(J38&gt;O38, (J38-O38)*6000000, 0)</f>
+        <f>IF(J38&gt;O38, (J38-O38)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG38" s="18">
@@ -5501,7 +5501,7 @@
         <v/>
       </c>
       <c r="M39" s="19" t="n">
-        <v>451</v>
+        <v>460.7</v>
       </c>
       <c r="N39" s="19">
         <f>M39*IF(F39=1, 0.85, 0.8)</f>
@@ -5528,7 +5528,7 @@
         <v/>
       </c>
       <c r="T39" s="18">
-        <f>IF(C39&gt;=17.5, Q39*0.2*W39, 0)</f>
+        <f>IF(C39&gt;=17.5, ROUND(Q39*0.2*W39*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U39" s="18">
@@ -5555,11 +5555,11 @@
         <v/>
       </c>
       <c r="AA39" s="18">
-        <f>IF(Y39="", 0, IF(Y39&gt;J39, (Y39-J39)*2700000, 0))</f>
+        <f>IF(Y39="", 0, IF(Y39&gt;J39, (Y39-J39)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB39" s="18">
-        <f>IF(Y39="", 0, IF(J39&gt;Y39, (J39-Y39)*6000000, 0))</f>
+        <f>IF(Y39="", 0, IF(J39&gt;Y39, (J39-Y39)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC39" s="18">
@@ -5571,11 +5571,11 @@
         <v/>
       </c>
       <c r="AE39" s="18">
-        <f>IF(O39&gt;J39, (O39-J39)*2700000, 0)</f>
+        <f>IF(O39&gt;J39, (O39-J39)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF39" s="18">
-        <f>IF(J39&gt;O39, (J39-O39)*6000000, 0)</f>
+        <f>IF(J39&gt;O39, (J39-O39)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG39" s="18">
@@ -5629,7 +5629,7 @@
         <v/>
       </c>
       <c r="M40" s="19" t="n">
-        <v>485.8</v>
+        <v>502.8</v>
       </c>
       <c r="N40" s="19">
         <f>M40*IF(F40=1, 0.85, 0.8)</f>
@@ -5656,7 +5656,7 @@
         <v/>
       </c>
       <c r="T40" s="18">
-        <f>IF(C40&gt;=17.5, Q40*0.2*W40, 0)</f>
+        <f>IF(C40&gt;=17.5, ROUND(Q40*0.2*W40*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U40" s="18">
@@ -5683,11 +5683,11 @@
         <v/>
       </c>
       <c r="AA40" s="18">
-        <f>IF(Y40="", 0, IF(Y40&gt;J40, (Y40-J40)*2700000, 0))</f>
+        <f>IF(Y40="", 0, IF(Y40&gt;J40, (Y40-J40)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB40" s="18">
-        <f>IF(Y40="", 0, IF(J40&gt;Y40, (J40-Y40)*6000000, 0))</f>
+        <f>IF(Y40="", 0, IF(J40&gt;Y40, (J40-Y40)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC40" s="18">
@@ -5699,11 +5699,11 @@
         <v/>
       </c>
       <c r="AE40" s="18">
-        <f>IF(O40&gt;J40, (O40-J40)*2700000, 0)</f>
+        <f>IF(O40&gt;J40, (O40-J40)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF40" s="18">
-        <f>IF(J40&gt;O40, (J40-O40)*6000000, 0)</f>
+        <f>IF(J40&gt;O40, (J40-O40)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG40" s="18">
@@ -5757,7 +5757,7 @@
         <v/>
       </c>
       <c r="M41" s="19" t="n">
-        <v>499.4</v>
+        <v>511.5</v>
       </c>
       <c r="N41" s="19">
         <f>M41*IF(F41=1, 0.85, 0.8)</f>
@@ -5784,7 +5784,7 @@
         <v/>
       </c>
       <c r="T41" s="18">
-        <f>IF(C41&gt;=17.5, Q41*0.2*W41, 0)</f>
+        <f>IF(C41&gt;=17.5, ROUND(Q41*0.2*W41*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U41" s="18">
@@ -5811,11 +5811,11 @@
         <v/>
       </c>
       <c r="AA41" s="18">
-        <f>IF(Y41="", 0, IF(Y41&gt;J41, (Y41-J41)*2700000, 0))</f>
+        <f>IF(Y41="", 0, IF(Y41&gt;J41, (Y41-J41)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB41" s="18">
-        <f>IF(Y41="", 0, IF(J41&gt;Y41, (J41-Y41)*6000000, 0))</f>
+        <f>IF(Y41="", 0, IF(J41&gt;Y41, (J41-Y41)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC41" s="18">
@@ -5827,11 +5827,11 @@
         <v/>
       </c>
       <c r="AE41" s="18">
-        <f>IF(O41&gt;J41, (O41-J41)*2700000, 0)</f>
+        <f>IF(O41&gt;J41, (O41-J41)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF41" s="18">
-        <f>IF(J41&gt;O41, (J41-O41)*6000000, 0)</f>
+        <f>IF(J41&gt;O41, (J41-O41)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG41" s="18">
@@ -5885,7 +5885,7 @@
         <v/>
       </c>
       <c r="M42" s="19" t="n">
-        <v>524.4</v>
+        <v>533.1</v>
       </c>
       <c r="N42" s="19">
         <f>M42*IF(F42=1, 0.85, 0.8)</f>
@@ -5912,7 +5912,7 @@
         <v/>
       </c>
       <c r="T42" s="18">
-        <f>IF(C42&gt;=17.5, Q42*0.2*W42, 0)</f>
+        <f>IF(C42&gt;=17.5, ROUND(Q42*0.2*W42*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U42" s="18">
@@ -5939,11 +5939,11 @@
         <v/>
       </c>
       <c r="AA42" s="18">
-        <f>IF(Y42="", 0, IF(Y42&gt;J42, (Y42-J42)*2700000, 0))</f>
+        <f>IF(Y42="", 0, IF(Y42&gt;J42, (Y42-J42)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB42" s="18">
-        <f>IF(Y42="", 0, IF(J42&gt;Y42, (J42-Y42)*6000000, 0))</f>
+        <f>IF(Y42="", 0, IF(J42&gt;Y42, (J42-Y42)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC42" s="18">
@@ -5955,11 +5955,11 @@
         <v/>
       </c>
       <c r="AE42" s="18">
-        <f>IF(O42&gt;J42, (O42-J42)*2700000, 0)</f>
+        <f>IF(O42&gt;J42, (O42-J42)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF42" s="18">
-        <f>IF(J42&gt;O42, (J42-O42)*6000000, 0)</f>
+        <f>IF(J42&gt;O42, (J42-O42)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG42" s="18">
@@ -6013,7 +6013,7 @@
         <v/>
       </c>
       <c r="M43" s="19" t="n">
-        <v>495.1</v>
+        <v>510.8</v>
       </c>
       <c r="N43" s="19">
         <f>M43*IF(F43=1, 0.85, 0.8)</f>
@@ -6040,7 +6040,7 @@
         <v/>
       </c>
       <c r="T43" s="18">
-        <f>IF(C43&gt;=17.5, Q43*0.2*W43, 0)</f>
+        <f>IF(C43&gt;=17.5, ROUND(Q43*0.2*W43*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U43" s="18">
@@ -6067,11 +6067,11 @@
         <v/>
       </c>
       <c r="AA43" s="18">
-        <f>IF(Y43="", 0, IF(Y43&gt;J43, (Y43-J43)*2700000, 0))</f>
+        <f>IF(Y43="", 0, IF(Y43&gt;J43, (Y43-J43)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB43" s="18">
-        <f>IF(Y43="", 0, IF(J43&gt;Y43, (J43-Y43)*6000000, 0))</f>
+        <f>IF(Y43="", 0, IF(J43&gt;Y43, (J43-Y43)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC43" s="18">
@@ -6083,11 +6083,11 @@
         <v/>
       </c>
       <c r="AE43" s="18">
-        <f>IF(O43&gt;J43, (O43-J43)*2700000, 0)</f>
+        <f>IF(O43&gt;J43, (O43-J43)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF43" s="18">
-        <f>IF(J43&gt;O43, (J43-O43)*6000000, 0)</f>
+        <f>IF(J43&gt;O43, (J43-O43)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG43" s="18">
@@ -6141,7 +6141,7 @@
         <v/>
       </c>
       <c r="M44" s="19" t="n">
-        <v>592.6</v>
+        <v>609.5</v>
       </c>
       <c r="N44" s="19">
         <f>M44*IF(F44=1, 0.85, 0.8)</f>
@@ -6168,7 +6168,7 @@
         <v/>
       </c>
       <c r="T44" s="18">
-        <f>IF(C44&gt;=17.5, Q44*0.2*W44, 0)</f>
+        <f>IF(C44&gt;=17.5, ROUND(Q44*0.2*W44*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U44" s="18">
@@ -6195,11 +6195,11 @@
         <v/>
       </c>
       <c r="AA44" s="18">
-        <f>IF(Y44="", 0, IF(Y44&gt;J44, (Y44-J44)*2700000, 0))</f>
+        <f>IF(Y44="", 0, IF(Y44&gt;J44, (Y44-J44)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB44" s="18">
-        <f>IF(Y44="", 0, IF(J44&gt;Y44, (J44-Y44)*6000000, 0))</f>
+        <f>IF(Y44="", 0, IF(J44&gt;Y44, (J44-Y44)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC44" s="18">
@@ -6211,11 +6211,11 @@
         <v/>
       </c>
       <c r="AE44" s="18">
-        <f>IF(O44&gt;J44, (O44-J44)*2700000, 0)</f>
+        <f>IF(O44&gt;J44, (O44-J44)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF44" s="18">
-        <f>IF(J44&gt;O44, (J44-O44)*6000000, 0)</f>
+        <f>IF(J44&gt;O44, (J44-O44)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG44" s="18">
@@ -6269,7 +6269,7 @@
         <v/>
       </c>
       <c r="M45" s="19" t="n">
-        <v>593.8</v>
+        <v>605</v>
       </c>
       <c r="N45" s="19">
         <f>M45*IF(F45=1, 0.85, 0.8)</f>
@@ -6296,7 +6296,7 @@
         <v/>
       </c>
       <c r="T45" s="18">
-        <f>IF(C45&gt;=17.5, Q45*0.2*W45, 0)</f>
+        <f>IF(C45&gt;=17.5, ROUND(Q45*0.2*W45*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U45" s="18">
@@ -6323,11 +6323,11 @@
         <v/>
       </c>
       <c r="AA45" s="18">
-        <f>IF(Y45="", 0, IF(Y45&gt;J45, (Y45-J45)*2700000, 0))</f>
+        <f>IF(Y45="", 0, IF(Y45&gt;J45, (Y45-J45)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB45" s="18">
-        <f>IF(Y45="", 0, IF(J45&gt;Y45, (J45-Y45)*6000000, 0))</f>
+        <f>IF(Y45="", 0, IF(J45&gt;Y45, (J45-Y45)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC45" s="18">
@@ -6339,11 +6339,11 @@
         <v/>
       </c>
       <c r="AE45" s="18">
-        <f>IF(O45&gt;J45, (O45-J45)*2700000, 0)</f>
+        <f>IF(O45&gt;J45, (O45-J45)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF45" s="18">
-        <f>IF(J45&gt;O45, (J45-O45)*6000000, 0)</f>
+        <f>IF(J45&gt;O45, (J45-O45)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG45" s="18">
@@ -6397,7 +6397,7 @@
         <v/>
       </c>
       <c r="M46" s="19" t="n">
-        <v>513.4</v>
+        <v>526.6</v>
       </c>
       <c r="N46" s="19">
         <f>M46*IF(F46=1, 0.85, 0.8)</f>
@@ -6424,7 +6424,7 @@
         <v/>
       </c>
       <c r="T46" s="18">
-        <f>IF(C46&gt;=17.5, Q46*0.2*W46, 0)</f>
+        <f>IF(C46&gt;=17.5, ROUND(Q46*0.2*W46*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U46" s="18">
@@ -6451,11 +6451,11 @@
         <v/>
       </c>
       <c r="AA46" s="18">
-        <f>IF(Y46="", 0, IF(Y46&gt;J46, (Y46-J46)*2700000, 0))</f>
+        <f>IF(Y46="", 0, IF(Y46&gt;J46, (Y46-J46)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB46" s="18">
-        <f>IF(Y46="", 0, IF(J46&gt;Y46, (J46-Y46)*6000000, 0))</f>
+        <f>IF(Y46="", 0, IF(J46&gt;Y46, (J46-Y46)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC46" s="18">
@@ -6467,11 +6467,11 @@
         <v/>
       </c>
       <c r="AE46" s="18">
-        <f>IF(O46&gt;J46, (O46-J46)*2700000, 0)</f>
+        <f>IF(O46&gt;J46, (O46-J46)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF46" s="18">
-        <f>IF(J46&gt;O46, (J46-O46)*6000000, 0)</f>
+        <f>IF(J46&gt;O46, (J46-O46)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG46" s="18">
@@ -6525,7 +6525,7 @@
         <v/>
       </c>
       <c r="M47" s="19" t="n">
-        <v>557.9</v>
+        <v>564.8</v>
       </c>
       <c r="N47" s="19">
         <f>M47*IF(F47=1, 0.85, 0.8)</f>
@@ -6552,7 +6552,7 @@
         <v/>
       </c>
       <c r="T47" s="18">
-        <f>IF(C47&gt;=17.5, Q47*0.2*W47, 0)</f>
+        <f>IF(C47&gt;=17.5, ROUND(Q47*0.2*W47*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U47" s="18">
@@ -6579,11 +6579,11 @@
         <v/>
       </c>
       <c r="AA47" s="18">
-        <f>IF(Y47="", 0, IF(Y47&gt;J47, (Y47-J47)*2700000, 0))</f>
+        <f>IF(Y47="", 0, IF(Y47&gt;J47, (Y47-J47)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB47" s="18">
-        <f>IF(Y47="", 0, IF(J47&gt;Y47, (J47-Y47)*6000000, 0))</f>
+        <f>IF(Y47="", 0, IF(J47&gt;Y47, (J47-Y47)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC47" s="18">
@@ -6595,11 +6595,11 @@
         <v/>
       </c>
       <c r="AE47" s="18">
-        <f>IF(O47&gt;J47, (O47-J47)*2700000, 0)</f>
+        <f>IF(O47&gt;J47, (O47-J47)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF47" s="18">
-        <f>IF(J47&gt;O47, (J47-O47)*6000000, 0)</f>
+        <f>IF(J47&gt;O47, (J47-O47)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG47" s="18">
@@ -6653,7 +6653,7 @@
         <v/>
       </c>
       <c r="M48" s="19" t="n">
-        <v>488.6</v>
+        <v>496.4</v>
       </c>
       <c r="N48" s="19">
         <f>M48*IF(F48=1, 0.85, 0.8)</f>
@@ -6680,7 +6680,7 @@
         <v/>
       </c>
       <c r="T48" s="18">
-        <f>IF(C48&gt;=17.5, Q48*0.2*W48, 0)</f>
+        <f>IF(C48&gt;=17.5, ROUND(Q48*0.2*W48*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U48" s="18">
@@ -6707,11 +6707,11 @@
         <v/>
       </c>
       <c r="AA48" s="18">
-        <f>IF(Y48="", 0, IF(Y48&gt;J48, (Y48-J48)*2700000, 0))</f>
+        <f>IF(Y48="", 0, IF(Y48&gt;J48, (Y48-J48)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB48" s="18">
-        <f>IF(Y48="", 0, IF(J48&gt;Y48, (J48-Y48)*6000000, 0))</f>
+        <f>IF(Y48="", 0, IF(J48&gt;Y48, (J48-Y48)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC48" s="18">
@@ -6723,11 +6723,11 @@
         <v/>
       </c>
       <c r="AE48" s="18">
-        <f>IF(O48&gt;J48, (O48-J48)*2700000, 0)</f>
+        <f>IF(O48&gt;J48, (O48-J48)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF48" s="18">
-        <f>IF(J48&gt;O48, (J48-O48)*6000000, 0)</f>
+        <f>IF(J48&gt;O48, (J48-O48)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG48" s="18">
@@ -6781,7 +6781,7 @@
         <v/>
       </c>
       <c r="M49" s="19" t="n">
-        <v>488.6</v>
+        <v>493.4</v>
       </c>
       <c r="N49" s="19">
         <f>M49*IF(F49=1, 0.85, 0.8)</f>
@@ -6808,7 +6808,7 @@
         <v/>
       </c>
       <c r="T49" s="18">
-        <f>IF(C49&gt;=17.5, Q49*0.2*W49, 0)</f>
+        <f>IF(C49&gt;=17.5, ROUND(Q49*0.2*W49*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U49" s="18">
@@ -6835,11 +6835,11 @@
         <v/>
       </c>
       <c r="AA49" s="18">
-        <f>IF(Y49="", 0, IF(Y49&gt;J49, (Y49-J49)*2700000, 0))</f>
+        <f>IF(Y49="", 0, IF(Y49&gt;J49, (Y49-J49)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB49" s="18">
-        <f>IF(Y49="", 0, IF(J49&gt;Y49, (J49-Y49)*6000000, 0))</f>
+        <f>IF(Y49="", 0, IF(J49&gt;Y49, (J49-Y49)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC49" s="18">
@@ -6851,11 +6851,11 @@
         <v/>
       </c>
       <c r="AE49" s="18">
-        <f>IF(O49&gt;J49, (O49-J49)*2700000, 0)</f>
+        <f>IF(O49&gt;J49, (O49-J49)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF49" s="18">
-        <f>IF(J49&gt;O49, (J49-O49)*6000000, 0)</f>
+        <f>IF(J49&gt;O49, (J49-O49)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG49" s="18">
@@ -6909,7 +6909,7 @@
         <v/>
       </c>
       <c r="M50" s="19" t="n">
-        <v>463.3</v>
+        <v>453.4</v>
       </c>
       <c r="N50" s="19">
         <f>M50*IF(F50=1, 0.85, 0.8)</f>
@@ -6936,7 +6936,7 @@
         <v/>
       </c>
       <c r="T50" s="18">
-        <f>IF(C50&gt;=17.5, Q50*0.2*W50, 0)</f>
+        <f>IF(C50&gt;=17.5, ROUND(Q50*0.2*W50*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U50" s="18">
@@ -6963,11 +6963,11 @@
         <v/>
       </c>
       <c r="AA50" s="18">
-        <f>IF(Y50="", 0, IF(Y50&gt;J50, (Y50-J50)*2700000, 0))</f>
+        <f>IF(Y50="", 0, IF(Y50&gt;J50, (Y50-J50)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB50" s="18">
-        <f>IF(Y50="", 0, IF(J50&gt;Y50, (J50-Y50)*6000000, 0))</f>
+        <f>IF(Y50="", 0, IF(J50&gt;Y50, (J50-Y50)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC50" s="18">
@@ -6979,11 +6979,11 @@
         <v/>
       </c>
       <c r="AE50" s="18">
-        <f>IF(O50&gt;J50, (O50-J50)*2700000, 0)</f>
+        <f>IF(O50&gt;J50, (O50-J50)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF50" s="18">
-        <f>IF(J50&gt;O50, (J50-O50)*6000000, 0)</f>
+        <f>IF(J50&gt;O50, (J50-O50)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG50" s="18">
@@ -7037,7 +7037,7 @@
         <v/>
       </c>
       <c r="M51" s="19" t="n">
-        <v>568.4</v>
+        <v>571.9</v>
       </c>
       <c r="N51" s="19">
         <f>M51*IF(F51=1, 0.85, 0.8)</f>
@@ -7064,7 +7064,7 @@
         <v/>
       </c>
       <c r="T51" s="18">
-        <f>IF(C51&gt;=17.5, Q51*0.2*W51, 0)</f>
+        <f>IF(C51&gt;=17.5, ROUND(Q51*0.2*W51*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U51" s="18">
@@ -7091,11 +7091,11 @@
         <v/>
       </c>
       <c r="AA51" s="18">
-        <f>IF(Y51="", 0, IF(Y51&gt;J51, (Y51-J51)*2700000, 0))</f>
+        <f>IF(Y51="", 0, IF(Y51&gt;J51, (Y51-J51)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB51" s="18">
-        <f>IF(Y51="", 0, IF(J51&gt;Y51, (J51-Y51)*6000000, 0))</f>
+        <f>IF(Y51="", 0, IF(J51&gt;Y51, (J51-Y51)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC51" s="18">
@@ -7107,11 +7107,11 @@
         <v/>
       </c>
       <c r="AE51" s="18">
-        <f>IF(O51&gt;J51, (O51-J51)*2700000, 0)</f>
+        <f>IF(O51&gt;J51, (O51-J51)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF51" s="18">
-        <f>IF(J51&gt;O51, (J51-O51)*6000000, 0)</f>
+        <f>IF(J51&gt;O51, (J51-O51)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG51" s="18">
@@ -7165,7 +7165,7 @@
         <v/>
       </c>
       <c r="M52" s="19" t="n">
-        <v>590</v>
+        <v>601.8</v>
       </c>
       <c r="N52" s="19">
         <f>M52*IF(F52=1, 0.85, 0.8)</f>
@@ -7192,7 +7192,7 @@
         <v/>
       </c>
       <c r="T52" s="18">
-        <f>IF(C52&gt;=17.5, Q52*0.2*W52, 0)</f>
+        <f>IF(C52&gt;=17.5, ROUND(Q52*0.2*W52*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U52" s="18">
@@ -7219,11 +7219,11 @@
         <v/>
       </c>
       <c r="AA52" s="18">
-        <f>IF(Y52="", 0, IF(Y52&gt;J52, (Y52-J52)*2700000, 0))</f>
+        <f>IF(Y52="", 0, IF(Y52&gt;J52, (Y52-J52)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB52" s="18">
-        <f>IF(Y52="", 0, IF(J52&gt;Y52, (J52-Y52)*6000000, 0))</f>
+        <f>IF(Y52="", 0, IF(J52&gt;Y52, (J52-Y52)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC52" s="18">
@@ -7235,11 +7235,11 @@
         <v/>
       </c>
       <c r="AE52" s="18">
-        <f>IF(O52&gt;J52, (O52-J52)*2700000, 0)</f>
+        <f>IF(O52&gt;J52, (O52-J52)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF52" s="18">
-        <f>IF(J52&gt;O52, (J52-O52)*6000000, 0)</f>
+        <f>IF(J52&gt;O52, (J52-O52)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG52" s="18">
@@ -7293,7 +7293,7 @@
         <v/>
       </c>
       <c r="M53" s="19" t="n">
-        <v>531.2</v>
+        <v>545</v>
       </c>
       <c r="N53" s="19">
         <f>M53*IF(F53=1, 0.85, 0.8)</f>
@@ -7320,7 +7320,7 @@
         <v/>
       </c>
       <c r="T53" s="18">
-        <f>IF(C53&gt;=17.5, Q53*0.2*W53, 0)</f>
+        <f>IF(C53&gt;=17.5, ROUND(Q53*0.2*W53*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U53" s="18">
@@ -7347,11 +7347,11 @@
         <v/>
       </c>
       <c r="AA53" s="18">
-        <f>IF(Y53="", 0, IF(Y53&gt;J53, (Y53-J53)*2700000, 0))</f>
+        <f>IF(Y53="", 0, IF(Y53&gt;J53, (Y53-J53)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB53" s="18">
-        <f>IF(Y53="", 0, IF(J53&gt;Y53, (J53-Y53)*6000000, 0))</f>
+        <f>IF(Y53="", 0, IF(J53&gt;Y53, (J53-Y53)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC53" s="18">
@@ -7363,11 +7363,11 @@
         <v/>
       </c>
       <c r="AE53" s="18">
-        <f>IF(O53&gt;J53, (O53-J53)*2700000, 0)</f>
+        <f>IF(O53&gt;J53, (O53-J53)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF53" s="18">
-        <f>IF(J53&gt;O53, (J53-O53)*6000000, 0)</f>
+        <f>IF(J53&gt;O53, (J53-O53)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG53" s="18">
@@ -7421,7 +7421,7 @@
         <v/>
       </c>
       <c r="M54" s="19" t="n">
-        <v>477.4</v>
+        <v>495.5</v>
       </c>
       <c r="N54" s="19">
         <f>M54*IF(F54=1, 0.85, 0.8)</f>
@@ -7448,7 +7448,7 @@
         <v/>
       </c>
       <c r="T54" s="18">
-        <f>IF(C54&gt;=17.5, Q54*0.2*W54, 0)</f>
+        <f>IF(C54&gt;=17.5, ROUND(Q54*0.2*W54*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U54" s="18">
@@ -7475,11 +7475,11 @@
         <v/>
       </c>
       <c r="AA54" s="18">
-        <f>IF(Y54="", 0, IF(Y54&gt;J54, (Y54-J54)*2700000, 0))</f>
+        <f>IF(Y54="", 0, IF(Y54&gt;J54, (Y54-J54)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB54" s="18">
-        <f>IF(Y54="", 0, IF(J54&gt;Y54, (J54-Y54)*6000000, 0))</f>
+        <f>IF(Y54="", 0, IF(J54&gt;Y54, (J54-Y54)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC54" s="18">
@@ -7491,11 +7491,11 @@
         <v/>
       </c>
       <c r="AE54" s="18">
-        <f>IF(O54&gt;J54, (O54-J54)*2700000, 0)</f>
+        <f>IF(O54&gt;J54, (O54-J54)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF54" s="18">
-        <f>IF(J54&gt;O54, (J54-O54)*6000000, 0)</f>
+        <f>IF(J54&gt;O54, (J54-O54)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG54" s="18">
@@ -7549,7 +7549,7 @@
         <v/>
       </c>
       <c r="M55" s="19" t="n">
-        <v>530.7</v>
+        <v>538.5</v>
       </c>
       <c r="N55" s="19">
         <f>M55*IF(F55=1, 0.85, 0.8)</f>
@@ -7576,7 +7576,7 @@
         <v/>
       </c>
       <c r="T55" s="18">
-        <f>IF(C55&gt;=17.5, Q55*0.2*W55, 0)</f>
+        <f>IF(C55&gt;=17.5, ROUND(Q55*0.2*W55*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U55" s="18">
@@ -7603,11 +7603,11 @@
         <v/>
       </c>
       <c r="AA55" s="18">
-        <f>IF(Y55="", 0, IF(Y55&gt;J55, (Y55-J55)*2700000, 0))</f>
+        <f>IF(Y55="", 0, IF(Y55&gt;J55, (Y55-J55)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB55" s="18">
-        <f>IF(Y55="", 0, IF(J55&gt;Y55, (J55-Y55)*6000000, 0))</f>
+        <f>IF(Y55="", 0, IF(J55&gt;Y55, (J55-Y55)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC55" s="18">
@@ -7619,11 +7619,11 @@
         <v/>
       </c>
       <c r="AE55" s="18">
-        <f>IF(O55&gt;J55, (O55-J55)*2700000, 0)</f>
+        <f>IF(O55&gt;J55, (O55-J55)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF55" s="18">
-        <f>IF(J55&gt;O55, (J55-O55)*6000000, 0)</f>
+        <f>IF(J55&gt;O55, (J55-O55)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG55" s="18">
@@ -7677,7 +7677,7 @@
         <v/>
       </c>
       <c r="M56" s="19" t="n">
-        <v>479.1</v>
+        <v>494.2</v>
       </c>
       <c r="N56" s="19">
         <f>M56*IF(F56=1, 0.85, 0.8)</f>
@@ -7704,7 +7704,7 @@
         <v/>
       </c>
       <c r="T56" s="18">
-        <f>IF(C56&gt;=17.5, Q56*0.2*W56, 0)</f>
+        <f>IF(C56&gt;=17.5, ROUND(Q56*0.2*W56*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U56" s="18">
@@ -7731,11 +7731,11 @@
         <v/>
       </c>
       <c r="AA56" s="18">
-        <f>IF(Y56="", 0, IF(Y56&gt;J56, (Y56-J56)*2700000, 0))</f>
+        <f>IF(Y56="", 0, IF(Y56&gt;J56, (Y56-J56)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB56" s="18">
-        <f>IF(Y56="", 0, IF(J56&gt;Y56, (J56-Y56)*6000000, 0))</f>
+        <f>IF(Y56="", 0, IF(J56&gt;Y56, (J56-Y56)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC56" s="18">
@@ -7747,11 +7747,11 @@
         <v/>
       </c>
       <c r="AE56" s="18">
-        <f>IF(O56&gt;J56, (O56-J56)*2700000, 0)</f>
+        <f>IF(O56&gt;J56, (O56-J56)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF56" s="18">
-        <f>IF(J56&gt;O56, (J56-O56)*6000000, 0)</f>
+        <f>IF(J56&gt;O56, (J56-O56)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG56" s="18">
@@ -7805,7 +7805,7 @@
         <v/>
       </c>
       <c r="M57" s="19" t="n">
-        <v>499.2</v>
+        <v>511.5</v>
       </c>
       <c r="N57" s="19">
         <f>M57*IF(F57=1, 0.85, 0.8)</f>
@@ -7832,7 +7832,7 @@
         <v/>
       </c>
       <c r="T57" s="18">
-        <f>IF(C57&gt;=17.5, Q57*0.2*W57, 0)</f>
+        <f>IF(C57&gt;=17.5, ROUND(Q57*0.2*W57*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U57" s="18">
@@ -7859,11 +7859,11 @@
         <v/>
       </c>
       <c r="AA57" s="18">
-        <f>IF(Y57="", 0, IF(Y57&gt;J57, (Y57-J57)*2700000, 0))</f>
+        <f>IF(Y57="", 0, IF(Y57&gt;J57, (Y57-J57)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB57" s="18">
-        <f>IF(Y57="", 0, IF(J57&gt;Y57, (J57-Y57)*6000000, 0))</f>
+        <f>IF(Y57="", 0, IF(J57&gt;Y57, (J57-Y57)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC57" s="18">
@@ -7875,11 +7875,11 @@
         <v/>
       </c>
       <c r="AE57" s="18">
-        <f>IF(O57&gt;J57, (O57-J57)*2700000, 0)</f>
+        <f>IF(O57&gt;J57, (O57-J57)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF57" s="18">
-        <f>IF(J57&gt;O57, (J57-O57)*6000000, 0)</f>
+        <f>IF(J57&gt;O57, (J57-O57)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG57" s="18">
@@ -7933,7 +7933,7 @@
         <v/>
       </c>
       <c r="M58" s="19" t="n">
-        <v>560.1</v>
+        <v>564.6</v>
       </c>
       <c r="N58" s="19">
         <f>M58*IF(F58=1, 0.85, 0.8)</f>
@@ -7960,7 +7960,7 @@
         <v/>
       </c>
       <c r="T58" s="18">
-        <f>IF(C58&gt;=17.5, Q58*0.2*W58, 0)</f>
+        <f>IF(C58&gt;=17.5, ROUND(Q58*0.2*W58*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U58" s="18">
@@ -7987,11 +7987,11 @@
         <v/>
       </c>
       <c r="AA58" s="18">
-        <f>IF(Y58="", 0, IF(Y58&gt;J58, (Y58-J58)*2700000, 0))</f>
+        <f>IF(Y58="", 0, IF(Y58&gt;J58, (Y58-J58)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB58" s="18">
-        <f>IF(Y58="", 0, IF(J58&gt;Y58, (J58-Y58)*6000000, 0))</f>
+        <f>IF(Y58="", 0, IF(J58&gt;Y58, (J58-Y58)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC58" s="18">
@@ -8003,11 +8003,11 @@
         <v/>
       </c>
       <c r="AE58" s="18">
-        <f>IF(O58&gt;J58, (O58-J58)*2700000, 0)</f>
+        <f>IF(O58&gt;J58, (O58-J58)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF58" s="18">
-        <f>IF(J58&gt;O58, (J58-O58)*6000000, 0)</f>
+        <f>IF(J58&gt;O58, (J58-O58)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG58" s="18">
@@ -8061,7 +8061,7 @@
         <v/>
       </c>
       <c r="M59" s="19" t="n">
-        <v>533.4</v>
+        <v>538.9</v>
       </c>
       <c r="N59" s="19">
         <f>M59*IF(F59=1, 0.85, 0.8)</f>
@@ -8088,7 +8088,7 @@
         <v/>
       </c>
       <c r="T59" s="18">
-        <f>IF(C59&gt;=17.5, Q59*0.2*W59, 0)</f>
+        <f>IF(C59&gt;=17.5, ROUND(Q59*0.2*W59*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U59" s="18">
@@ -8115,11 +8115,11 @@
         <v/>
       </c>
       <c r="AA59" s="18">
-        <f>IF(Y59="", 0, IF(Y59&gt;J59, (Y59-J59)*2700000, 0))</f>
+        <f>IF(Y59="", 0, IF(Y59&gt;J59, (Y59-J59)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB59" s="18">
-        <f>IF(Y59="", 0, IF(J59&gt;Y59, (J59-Y59)*6000000, 0))</f>
+        <f>IF(Y59="", 0, IF(J59&gt;Y59, (J59-Y59)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC59" s="18">
@@ -8131,11 +8131,11 @@
         <v/>
       </c>
       <c r="AE59" s="18">
-        <f>IF(O59&gt;J59, (O59-J59)*2700000, 0)</f>
+        <f>IF(O59&gt;J59, (O59-J59)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF59" s="18">
-        <f>IF(J59&gt;O59, (J59-O59)*6000000, 0)</f>
+        <f>IF(J59&gt;O59, (J59-O59)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG59" s="18">
@@ -8189,7 +8189,7 @@
         <v/>
       </c>
       <c r="M60" s="19" t="n">
-        <v>430.9</v>
+        <v>437.4</v>
       </c>
       <c r="N60" s="19">
         <f>M60*IF(F60=1, 0.85, 0.8)</f>
@@ -8216,7 +8216,7 @@
         <v/>
       </c>
       <c r="T60" s="18">
-        <f>IF(C60&gt;=17.5, Q60*0.2*W60, 0)</f>
+        <f>IF(C60&gt;=17.5, ROUND(Q60*0.2*W60*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U60" s="18">
@@ -8243,11 +8243,11 @@
         <v/>
       </c>
       <c r="AA60" s="18">
-        <f>IF(Y60="", 0, IF(Y60&gt;J60, (Y60-J60)*2700000, 0))</f>
+        <f>IF(Y60="", 0, IF(Y60&gt;J60, (Y60-J60)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB60" s="18">
-        <f>IF(Y60="", 0, IF(J60&gt;Y60, (J60-Y60)*6000000, 0))</f>
+        <f>IF(Y60="", 0, IF(J60&gt;Y60, (J60-Y60)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC60" s="18">
@@ -8259,11 +8259,11 @@
         <v/>
       </c>
       <c r="AE60" s="18">
-        <f>IF(O60&gt;J60, (O60-J60)*2700000, 0)</f>
+        <f>IF(O60&gt;J60, (O60-J60)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF60" s="18">
-        <f>IF(J60&gt;O60, (J60-O60)*6000000, 0)</f>
+        <f>IF(J60&gt;O60, (J60-O60)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG60" s="18">
@@ -8317,7 +8317,7 @@
         <v/>
       </c>
       <c r="M61" s="19" t="n">
-        <v>367.4</v>
+        <v>373.9</v>
       </c>
       <c r="N61" s="19">
         <f>M61*IF(F61=1, 0.85, 0.8)</f>
@@ -8344,7 +8344,7 @@
         <v/>
       </c>
       <c r="T61" s="18">
-        <f>IF(C61&gt;=17.5, Q61*0.2*W61, 0)</f>
+        <f>IF(C61&gt;=17.5, ROUND(Q61*0.2*W61*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U61" s="18">
@@ -8371,11 +8371,11 @@
         <v/>
       </c>
       <c r="AA61" s="18">
-        <f>IF(Y61="", 0, IF(Y61&gt;J61, (Y61-J61)*2700000, 0))</f>
+        <f>IF(Y61="", 0, IF(Y61&gt;J61, (Y61-J61)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB61" s="18">
-        <f>IF(Y61="", 0, IF(J61&gt;Y61, (J61-Y61)*6000000, 0))</f>
+        <f>IF(Y61="", 0, IF(J61&gt;Y61, (J61-Y61)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC61" s="18">
@@ -8387,11 +8387,11 @@
         <v/>
       </c>
       <c r="AE61" s="18">
-        <f>IF(O61&gt;J61, (O61-J61)*2700000, 0)</f>
+        <f>IF(O61&gt;J61, (O61-J61)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF61" s="18">
-        <f>IF(J61&gt;O61, (J61-O61)*6000000, 0)</f>
+        <f>IF(J61&gt;O61, (J61-O61)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG61" s="18">
@@ -8445,7 +8445,7 @@
         <v/>
       </c>
       <c r="M62" s="19" t="n">
-        <v>402</v>
+        <v>403.5</v>
       </c>
       <c r="N62" s="19">
         <f>M62*IF(F62=1, 0.85, 0.8)</f>
@@ -8472,7 +8472,7 @@
         <v/>
       </c>
       <c r="T62" s="18">
-        <f>IF(C62&gt;=17.5, Q62*0.2*W62, 0)</f>
+        <f>IF(C62&gt;=17.5, ROUND(Q62*0.2*W62*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U62" s="18">
@@ -8499,11 +8499,11 @@
         <v/>
       </c>
       <c r="AA62" s="18">
-        <f>IF(Y62="", 0, IF(Y62&gt;J62, (Y62-J62)*2700000, 0))</f>
+        <f>IF(Y62="", 0, IF(Y62&gt;J62, (Y62-J62)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB62" s="18">
-        <f>IF(Y62="", 0, IF(J62&gt;Y62, (J62-Y62)*6000000, 0))</f>
+        <f>IF(Y62="", 0, IF(J62&gt;Y62, (J62-Y62)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC62" s="18">
@@ -8515,11 +8515,11 @@
         <v/>
       </c>
       <c r="AE62" s="18">
-        <f>IF(O62&gt;J62, (O62-J62)*2700000, 0)</f>
+        <f>IF(O62&gt;J62, (O62-J62)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF62" s="18">
-        <f>IF(J62&gt;O62, (J62-O62)*6000000, 0)</f>
+        <f>IF(J62&gt;O62, (J62-O62)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG62" s="18">
@@ -8573,7 +8573,7 @@
         <v/>
       </c>
       <c r="M63" s="19" t="n">
-        <v>338.5</v>
+        <v>348.8</v>
       </c>
       <c r="N63" s="19">
         <f>M63*IF(F63=1, 0.85, 0.8)</f>
@@ -8600,7 +8600,7 @@
         <v/>
       </c>
       <c r="T63" s="18">
-        <f>IF(C63&gt;=17.5, Q63*0.2*W63, 0)</f>
+        <f>IF(C63&gt;=17.5, ROUND(Q63*0.2*W63*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U63" s="18">
@@ -8627,11 +8627,11 @@
         <v/>
       </c>
       <c r="AA63" s="18">
-        <f>IF(Y63="", 0, IF(Y63&gt;J63, (Y63-J63)*2700000, 0))</f>
+        <f>IF(Y63="", 0, IF(Y63&gt;J63, (Y63-J63)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB63" s="18">
-        <f>IF(Y63="", 0, IF(J63&gt;Y63, (J63-Y63)*6000000, 0))</f>
+        <f>IF(Y63="", 0, IF(J63&gt;Y63, (J63-Y63)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC63" s="18">
@@ -8643,11 +8643,11 @@
         <v/>
       </c>
       <c r="AE63" s="18">
-        <f>IF(O63&gt;J63, (O63-J63)*2700000, 0)</f>
+        <f>IF(O63&gt;J63, (O63-J63)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF63" s="18">
-        <f>IF(J63&gt;O63, (J63-O63)*6000000, 0)</f>
+        <f>IF(J63&gt;O63, (J63-O63)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG63" s="18">
@@ -8701,7 +8701,7 @@
         <v/>
       </c>
       <c r="M64" s="19" t="n">
-        <v>269.6</v>
+        <v>274.5</v>
       </c>
       <c r="N64" s="19">
         <f>M64*IF(F64=1, 0.85, 0.8)</f>
@@ -8728,7 +8728,7 @@
         <v/>
       </c>
       <c r="T64" s="18">
-        <f>IF(C64&gt;=17.5, Q64*0.2*W64, 0)</f>
+        <f>IF(C64&gt;=17.5, ROUND(Q64*0.2*W64*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U64" s="18">
@@ -8755,11 +8755,11 @@
         <v/>
       </c>
       <c r="AA64" s="18">
-        <f>IF(Y64="", 0, IF(Y64&gt;J64, (Y64-J64)*2700000, 0))</f>
+        <f>IF(Y64="", 0, IF(Y64&gt;J64, (Y64-J64)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB64" s="18">
-        <f>IF(Y64="", 0, IF(J64&gt;Y64, (J64-Y64)*6000000, 0))</f>
+        <f>IF(Y64="", 0, IF(J64&gt;Y64, (J64-Y64)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC64" s="18">
@@ -8771,11 +8771,11 @@
         <v/>
       </c>
       <c r="AE64" s="18">
-        <f>IF(O64&gt;J64, (O64-J64)*2700000, 0)</f>
+        <f>IF(O64&gt;J64, (O64-J64)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF64" s="18">
-        <f>IF(J64&gt;O64, (J64-O64)*6000000, 0)</f>
+        <f>IF(J64&gt;O64, (J64-O64)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG64" s="18">
@@ -8829,7 +8829,7 @@
         <v/>
       </c>
       <c r="M65" s="19" t="n">
-        <v>296.4</v>
+        <v>300.9</v>
       </c>
       <c r="N65" s="19">
         <f>M65*IF(F65=1, 0.85, 0.8)</f>
@@ -8856,7 +8856,7 @@
         <v/>
       </c>
       <c r="T65" s="18">
-        <f>IF(C65&gt;=17.5, Q65*0.2*W65, 0)</f>
+        <f>IF(C65&gt;=17.5, ROUND(Q65*0.2*W65*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U65" s="18">
@@ -8883,11 +8883,11 @@
         <v/>
       </c>
       <c r="AA65" s="18">
-        <f>IF(Y65="", 0, IF(Y65&gt;J65, (Y65-J65)*2700000, 0))</f>
+        <f>IF(Y65="", 0, IF(Y65&gt;J65, (Y65-J65)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB65" s="18">
-        <f>IF(Y65="", 0, IF(J65&gt;Y65, (J65-Y65)*6000000, 0))</f>
+        <f>IF(Y65="", 0, IF(J65&gt;Y65, (J65-Y65)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC65" s="18">
@@ -8899,11 +8899,11 @@
         <v/>
       </c>
       <c r="AE65" s="18">
-        <f>IF(O65&gt;J65, (O65-J65)*2700000, 0)</f>
+        <f>IF(O65&gt;J65, (O65-J65)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF65" s="18">
-        <f>IF(J65&gt;O65, (J65-O65)*6000000, 0)</f>
+        <f>IF(J65&gt;O65, (J65-O65)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG65" s="18">
@@ -8957,7 +8957,7 @@
         <v/>
       </c>
       <c r="M66" s="19" t="n">
-        <v>270.6</v>
+        <v>275.7</v>
       </c>
       <c r="N66" s="19">
         <f>M66*IF(F66=1, 0.85, 0.8)</f>
@@ -8984,7 +8984,7 @@
         <v/>
       </c>
       <c r="T66" s="18">
-        <f>IF(C66&gt;=17.5, Q66*0.2*W66, 0)</f>
+        <f>IF(C66&gt;=17.5, ROUND(Q66*0.2*W66*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U66" s="18">
@@ -9011,11 +9011,11 @@
         <v/>
       </c>
       <c r="AA66" s="18">
-        <f>IF(Y66="", 0, IF(Y66&gt;J66, (Y66-J66)*2700000, 0))</f>
+        <f>IF(Y66="", 0, IF(Y66&gt;J66, (Y66-J66)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB66" s="18">
-        <f>IF(Y66="", 0, IF(J66&gt;Y66, (J66-Y66)*6000000, 0))</f>
+        <f>IF(Y66="", 0, IF(J66&gt;Y66, (J66-Y66)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC66" s="18">
@@ -9027,11 +9027,11 @@
         <v/>
       </c>
       <c r="AE66" s="18">
-        <f>IF(O66&gt;J66, (O66-J66)*2700000, 0)</f>
+        <f>IF(O66&gt;J66, (O66-J66)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF66" s="18">
-        <f>IF(J66&gt;O66, (J66-O66)*6000000, 0)</f>
+        <f>IF(J66&gt;O66, (J66-O66)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG66" s="18">
@@ -9085,7 +9085,7 @@
         <v/>
       </c>
       <c r="M67" s="19" t="n">
-        <v>227.9</v>
+        <v>232.6</v>
       </c>
       <c r="N67" s="19">
         <f>M67*IF(F67=1, 0.85, 0.8)</f>
@@ -9112,7 +9112,7 @@
         <v/>
       </c>
       <c r="T67" s="18">
-        <f>IF(C67&gt;=17.5, Q67*0.2*W67, 0)</f>
+        <f>IF(C67&gt;=17.5, ROUND(Q67*0.2*W67*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U67" s="18">
@@ -9139,11 +9139,11 @@
         <v/>
       </c>
       <c r="AA67" s="18">
-        <f>IF(Y67="", 0, IF(Y67&gt;J67, (Y67-J67)*2700000, 0))</f>
+        <f>IF(Y67="", 0, IF(Y67&gt;J67, (Y67-J67)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB67" s="18">
-        <f>IF(Y67="", 0, IF(J67&gt;Y67, (J67-Y67)*6000000, 0))</f>
+        <f>IF(Y67="", 0, IF(J67&gt;Y67, (J67-Y67)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC67" s="18">
@@ -9155,11 +9155,11 @@
         <v/>
       </c>
       <c r="AE67" s="18">
-        <f>IF(O67&gt;J67, (O67-J67)*2700000, 0)</f>
+        <f>IF(O67&gt;J67, (O67-J67)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF67" s="18">
-        <f>IF(J67&gt;O67, (J67-O67)*6000000, 0)</f>
+        <f>IF(J67&gt;O67, (J67-O67)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG67" s="18">
@@ -9213,7 +9213,7 @@
         <v/>
       </c>
       <c r="M68" s="19" t="n">
-        <v>174.3</v>
+        <v>183.6</v>
       </c>
       <c r="N68" s="19">
         <f>M68*IF(F68=1, 0.85, 0.8)</f>
@@ -9240,7 +9240,7 @@
         <v/>
       </c>
       <c r="T68" s="18">
-        <f>IF(C68&gt;=17.5, Q68*0.2*W68, 0)</f>
+        <f>IF(C68&gt;=17.5, ROUND(Q68*0.2*W68*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U68" s="18">
@@ -9267,11 +9267,11 @@
         <v/>
       </c>
       <c r="AA68" s="18">
-        <f>IF(Y68="", 0, IF(Y68&gt;J68, (Y68-J68)*2700000, 0))</f>
+        <f>IF(Y68="", 0, IF(Y68&gt;J68, (Y68-J68)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB68" s="18">
-        <f>IF(Y68="", 0, IF(J68&gt;Y68, (J68-Y68)*6000000, 0))</f>
+        <f>IF(Y68="", 0, IF(J68&gt;Y68, (J68-Y68)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC68" s="18">
@@ -9283,11 +9283,11 @@
         <v/>
       </c>
       <c r="AE68" s="18">
-        <f>IF(O68&gt;J68, (O68-J68)*2700000, 0)</f>
+        <f>IF(O68&gt;J68, (O68-J68)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF68" s="18">
-        <f>IF(J68&gt;O68, (J68-O68)*6000000, 0)</f>
+        <f>IF(J68&gt;O68, (J68-O68)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG68" s="18">
@@ -9341,7 +9341,7 @@
         <v/>
       </c>
       <c r="M69" s="19" t="n">
-        <v>213.4</v>
+        <v>223.4</v>
       </c>
       <c r="N69" s="19">
         <f>M69*IF(F69=1, 0.85, 0.8)</f>
@@ -9368,7 +9368,7 @@
         <v/>
       </c>
       <c r="T69" s="18">
-        <f>IF(C69&gt;=17.5, Q69*0.2*W69, 0)</f>
+        <f>IF(C69&gt;=17.5, ROUND(Q69*0.2*W69*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U69" s="18">
@@ -9395,11 +9395,11 @@
         <v/>
       </c>
       <c r="AA69" s="18">
-        <f>IF(Y69="", 0, IF(Y69&gt;J69, (Y69-J69)*2700000, 0))</f>
+        <f>IF(Y69="", 0, IF(Y69&gt;J69, (Y69-J69)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB69" s="18">
-        <f>IF(Y69="", 0, IF(J69&gt;Y69, (J69-Y69)*6000000, 0))</f>
+        <f>IF(Y69="", 0, IF(J69&gt;Y69, (J69-Y69)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC69" s="18">
@@ -9411,11 +9411,11 @@
         <v/>
       </c>
       <c r="AE69" s="18">
-        <f>IF(O69&gt;J69, (O69-J69)*2700000, 0)</f>
+        <f>IF(O69&gt;J69, (O69-J69)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF69" s="18">
-        <f>IF(J69&gt;O69, (J69-O69)*6000000, 0)</f>
+        <f>IF(J69&gt;O69, (J69-O69)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG69" s="18">
@@ -9469,7 +9469,7 @@
         <v/>
       </c>
       <c r="M70" s="19" t="n">
-        <v>209.3</v>
+        <v>219.7</v>
       </c>
       <c r="N70" s="19">
         <f>M70*IF(F70=1, 0.85, 0.8)</f>
@@ -9496,7 +9496,7 @@
         <v/>
       </c>
       <c r="T70" s="18">
-        <f>IF(C70&gt;=17.5, Q70*0.2*W70, 0)</f>
+        <f>IF(C70&gt;=17.5, ROUND(Q70*0.2*W70*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U70" s="18">
@@ -9523,11 +9523,11 @@
         <v/>
       </c>
       <c r="AA70" s="18">
-        <f>IF(Y70="", 0, IF(Y70&gt;J70, (Y70-J70)*2700000, 0))</f>
+        <f>IF(Y70="", 0, IF(Y70&gt;J70, (Y70-J70)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB70" s="18">
-        <f>IF(Y70="", 0, IF(J70&gt;Y70, (J70-Y70)*6000000, 0))</f>
+        <f>IF(Y70="", 0, IF(J70&gt;Y70, (J70-Y70)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC70" s="18">
@@ -9539,11 +9539,11 @@
         <v/>
       </c>
       <c r="AE70" s="18">
-        <f>IF(O70&gt;J70, (O70-J70)*2700000, 0)</f>
+        <f>IF(O70&gt;J70, (O70-J70)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF70" s="18">
-        <f>IF(J70&gt;O70, (J70-O70)*6000000, 0)</f>
+        <f>IF(J70&gt;O70, (J70-O70)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG70" s="18">
@@ -9597,7 +9597,7 @@
         <v/>
       </c>
       <c r="M71" s="19" t="n">
-        <v>195.3</v>
+        <v>207.6</v>
       </c>
       <c r="N71" s="19">
         <f>M71*IF(F71=1, 0.85, 0.8)</f>
@@ -9624,7 +9624,7 @@
         <v/>
       </c>
       <c r="T71" s="18">
-        <f>IF(C71&gt;=17.5, Q71*0.2*W71, 0)</f>
+        <f>IF(C71&gt;=17.5, ROUND(Q71*0.2*W71*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U71" s="18">
@@ -9651,11 +9651,11 @@
         <v/>
       </c>
       <c r="AA71" s="18">
-        <f>IF(Y71="", 0, IF(Y71&gt;J71, (Y71-J71)*2700000, 0))</f>
+        <f>IF(Y71="", 0, IF(Y71&gt;J71, (Y71-J71)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB71" s="18">
-        <f>IF(Y71="", 0, IF(J71&gt;Y71, (J71-Y71)*6000000, 0))</f>
+        <f>IF(Y71="", 0, IF(J71&gt;Y71, (J71-Y71)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC71" s="18">
@@ -9667,11 +9667,11 @@
         <v/>
       </c>
       <c r="AE71" s="18">
-        <f>IF(O71&gt;J71, (O71-J71)*2700000, 0)</f>
+        <f>IF(O71&gt;J71, (O71-J71)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF71" s="18">
-        <f>IF(J71&gt;O71, (J71-O71)*6000000, 0)</f>
+        <f>IF(J71&gt;O71, (J71-O71)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG71" s="18">
@@ -9725,7 +9725,7 @@
         <v/>
       </c>
       <c r="M72" s="19" t="n">
-        <v>156.1</v>
+        <v>165.9</v>
       </c>
       <c r="N72" s="19">
         <f>M72*IF(F72=1, 0.85, 0.8)</f>
@@ -9752,7 +9752,7 @@
         <v/>
       </c>
       <c r="T72" s="18">
-        <f>IF(C72&gt;=17.5, Q72*0.2*W72, 0)</f>
+        <f>IF(C72&gt;=17.5, ROUND(Q72*0.2*W72*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U72" s="18">
@@ -9779,11 +9779,11 @@
         <v/>
       </c>
       <c r="AA72" s="18">
-        <f>IF(Y72="", 0, IF(Y72&gt;J72, (Y72-J72)*2700000, 0))</f>
+        <f>IF(Y72="", 0, IF(Y72&gt;J72, (Y72-J72)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB72" s="18">
-        <f>IF(Y72="", 0, IF(J72&gt;Y72, (J72-Y72)*6000000, 0))</f>
+        <f>IF(Y72="", 0, IF(J72&gt;Y72, (J72-Y72)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC72" s="18">
@@ -9795,11 +9795,11 @@
         <v/>
       </c>
       <c r="AE72" s="18">
-        <f>IF(O72&gt;J72, (O72-J72)*2700000, 0)</f>
+        <f>IF(O72&gt;J72, (O72-J72)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF72" s="18">
-        <f>IF(J72&gt;O72, (J72-O72)*6000000, 0)</f>
+        <f>IF(J72&gt;O72, (J72-O72)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG72" s="18">
@@ -9853,7 +9853,7 @@
         <v/>
       </c>
       <c r="M73" s="19" t="n">
-        <v>212.4</v>
+        <v>220.2</v>
       </c>
       <c r="N73" s="19">
         <f>M73*IF(F73=1, 0.85, 0.8)</f>
@@ -9880,7 +9880,7 @@
         <v/>
       </c>
       <c r="T73" s="18">
-        <f>IF(C73&gt;=17.5, Q73*0.2*W73, 0)</f>
+        <f>IF(C73&gt;=17.5, ROUND(Q73*0.2*W73*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U73" s="18">
@@ -9907,11 +9907,11 @@
         <v/>
       </c>
       <c r="AA73" s="18">
-        <f>IF(Y73="", 0, IF(Y73&gt;J73, (Y73-J73)*2700000, 0))</f>
+        <f>IF(Y73="", 0, IF(Y73&gt;J73, (Y73-J73)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB73" s="18">
-        <f>IF(Y73="", 0, IF(J73&gt;Y73, (J73-Y73)*6000000, 0))</f>
+        <f>IF(Y73="", 0, IF(J73&gt;Y73, (J73-Y73)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC73" s="18">
@@ -9923,11 +9923,11 @@
         <v/>
       </c>
       <c r="AE73" s="18">
-        <f>IF(O73&gt;J73, (O73-J73)*2700000, 0)</f>
+        <f>IF(O73&gt;J73, (O73-J73)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF73" s="18">
-        <f>IF(J73&gt;O73, (J73-O73)*6000000, 0)</f>
+        <f>IF(J73&gt;O73, (J73-O73)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG73" s="18">
@@ -9981,7 +9981,7 @@
         <v/>
       </c>
       <c r="M74" s="19" t="n">
-        <v>169.6</v>
+        <v>176.5</v>
       </c>
       <c r="N74" s="19">
         <f>M74*IF(F74=1, 0.85, 0.8)</f>
@@ -10008,7 +10008,7 @@
         <v/>
       </c>
       <c r="T74" s="18">
-        <f>IF(C74&gt;=17.5, Q74*0.2*W74, 0)</f>
+        <f>IF(C74&gt;=17.5, ROUND(Q74*0.2*W74*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U74" s="18">
@@ -10035,11 +10035,11 @@
         <v/>
       </c>
       <c r="AA74" s="18">
-        <f>IF(Y74="", 0, IF(Y74&gt;J74, (Y74-J74)*2700000, 0))</f>
+        <f>IF(Y74="", 0, IF(Y74&gt;J74, (Y74-J74)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB74" s="18">
-        <f>IF(Y74="", 0, IF(J74&gt;Y74, (J74-Y74)*6000000, 0))</f>
+        <f>IF(Y74="", 0, IF(J74&gt;Y74, (J74-Y74)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC74" s="18">
@@ -10051,11 +10051,11 @@
         <v/>
       </c>
       <c r="AE74" s="18">
-        <f>IF(O74&gt;J74, (O74-J74)*2700000, 0)</f>
+        <f>IF(O74&gt;J74, (O74-J74)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF74" s="18">
-        <f>IF(J74&gt;O74, (J74-O74)*6000000, 0)</f>
+        <f>IF(J74&gt;O74, (J74-O74)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG74" s="18">
@@ -10109,7 +10109,7 @@
         <v/>
       </c>
       <c r="M75" s="19" t="n">
-        <v>177.8</v>
+        <v>183.6</v>
       </c>
       <c r="N75" s="19">
         <f>M75*IF(F75=1, 0.85, 0.8)</f>
@@ -10136,7 +10136,7 @@
         <v/>
       </c>
       <c r="T75" s="18">
-        <f>IF(C75&gt;=17.5, Q75*0.2*W75, 0)</f>
+        <f>IF(C75&gt;=17.5, ROUND(Q75*0.2*W75*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U75" s="18">
@@ -10163,11 +10163,11 @@
         <v/>
       </c>
       <c r="AA75" s="18">
-        <f>IF(Y75="", 0, IF(Y75&gt;J75, (Y75-J75)*2700000, 0))</f>
+        <f>IF(Y75="", 0, IF(Y75&gt;J75, (Y75-J75)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB75" s="18">
-        <f>IF(Y75="", 0, IF(J75&gt;Y75, (J75-Y75)*6000000, 0))</f>
+        <f>IF(Y75="", 0, IF(J75&gt;Y75, (J75-Y75)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC75" s="18">
@@ -10179,11 +10179,11 @@
         <v/>
       </c>
       <c r="AE75" s="18">
-        <f>IF(O75&gt;J75, (O75-J75)*2700000, 0)</f>
+        <f>IF(O75&gt;J75, (O75-J75)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF75" s="18">
-        <f>IF(J75&gt;O75, (J75-O75)*6000000, 0)</f>
+        <f>IF(J75&gt;O75, (J75-O75)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG75" s="18">
@@ -10237,7 +10237,7 @@
         <v/>
       </c>
       <c r="M76" s="19" t="n">
-        <v>171.3</v>
+        <v>178</v>
       </c>
       <c r="N76" s="19">
         <f>M76*IF(F76=1, 0.85, 0.8)</f>
@@ -10264,7 +10264,7 @@
         <v/>
       </c>
       <c r="T76" s="18">
-        <f>IF(C76&gt;=17.5, Q76*0.2*W76, 0)</f>
+        <f>IF(C76&gt;=17.5, ROUND(Q76*0.2*W76*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U76" s="18">
@@ -10291,11 +10291,11 @@
         <v/>
       </c>
       <c r="AA76" s="18">
-        <f>IF(Y76="", 0, IF(Y76&gt;J76, (Y76-J76)*2700000, 0))</f>
+        <f>IF(Y76="", 0, IF(Y76&gt;J76, (Y76-J76)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB76" s="18">
-        <f>IF(Y76="", 0, IF(J76&gt;Y76, (J76-Y76)*6000000, 0))</f>
+        <f>IF(Y76="", 0, IF(J76&gt;Y76, (J76-Y76)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC76" s="18">
@@ -10307,11 +10307,11 @@
         <v/>
       </c>
       <c r="AE76" s="18">
-        <f>IF(O76&gt;J76, (O76-J76)*2700000, 0)</f>
+        <f>IF(O76&gt;J76, (O76-J76)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF76" s="18">
-        <f>IF(J76&gt;O76, (J76-O76)*6000000, 0)</f>
+        <f>IF(J76&gt;O76, (J76-O76)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG76" s="18">
@@ -10365,7 +10365,7 @@
         <v/>
       </c>
       <c r="M77" s="19" t="n">
-        <v>156</v>
+        <v>164.8</v>
       </c>
       <c r="N77" s="19">
         <f>M77*IF(F77=1, 0.85, 0.8)</f>
@@ -10392,7 +10392,7 @@
         <v/>
       </c>
       <c r="T77" s="18">
-        <f>IF(C77&gt;=17.5, Q77*0.2*W77, 0)</f>
+        <f>IF(C77&gt;=17.5, ROUND(Q77*0.2*W77*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U77" s="18">
@@ -10419,11 +10419,11 @@
         <v/>
       </c>
       <c r="AA77" s="18">
-        <f>IF(Y77="", 0, IF(Y77&gt;J77, (Y77-J77)*2700000, 0))</f>
+        <f>IF(Y77="", 0, IF(Y77&gt;J77, (Y77-J77)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB77" s="18">
-        <f>IF(Y77="", 0, IF(J77&gt;Y77, (J77-Y77)*6000000, 0))</f>
+        <f>IF(Y77="", 0, IF(J77&gt;Y77, (J77-Y77)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC77" s="18">
@@ -10435,11 +10435,11 @@
         <v/>
       </c>
       <c r="AE77" s="18">
-        <f>IF(O77&gt;J77, (O77-J77)*2700000, 0)</f>
+        <f>IF(O77&gt;J77, (O77-J77)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF77" s="18">
-        <f>IF(J77&gt;O77, (J77-O77)*6000000, 0)</f>
+        <f>IF(J77&gt;O77, (J77-O77)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG77" s="18">
@@ -10493,7 +10493,7 @@
         <v/>
       </c>
       <c r="M78" s="19" t="n">
-        <v>145.4</v>
+        <v>155.5</v>
       </c>
       <c r="N78" s="19">
         <f>M78*IF(F78=1, 0.85, 0.8)</f>
@@ -10520,7 +10520,7 @@
         <v/>
       </c>
       <c r="T78" s="18">
-        <f>IF(C78&gt;=17.5, Q78*0.2*W78, 0)</f>
+        <f>IF(C78&gt;=17.5, ROUND(Q78*0.2*W78*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U78" s="18">
@@ -10547,11 +10547,11 @@
         <v/>
       </c>
       <c r="AA78" s="18">
-        <f>IF(Y78="", 0, IF(Y78&gt;J78, (Y78-J78)*2700000, 0))</f>
+        <f>IF(Y78="", 0, IF(Y78&gt;J78, (Y78-J78)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB78" s="18">
-        <f>IF(Y78="", 0, IF(J78&gt;Y78, (J78-Y78)*6000000, 0))</f>
+        <f>IF(Y78="", 0, IF(J78&gt;Y78, (J78-Y78)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC78" s="18">
@@ -10563,11 +10563,11 @@
         <v/>
       </c>
       <c r="AE78" s="18">
-        <f>IF(O78&gt;J78, (O78-J78)*2700000, 0)</f>
+        <f>IF(O78&gt;J78, (O78-J78)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF78" s="18">
-        <f>IF(J78&gt;O78, (J78-O78)*6000000, 0)</f>
+        <f>IF(J78&gt;O78, (J78-O78)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG78" s="18">
@@ -10621,7 +10621,7 @@
         <v/>
       </c>
       <c r="M79" s="19" t="n">
-        <v>183.6</v>
+        <v>189.5</v>
       </c>
       <c r="N79" s="19">
         <f>M79*IF(F79=1, 0.85, 0.8)</f>
@@ -10648,7 +10648,7 @@
         <v/>
       </c>
       <c r="T79" s="18">
-        <f>IF(C79&gt;=17.5, Q79*0.2*W79, 0)</f>
+        <f>IF(C79&gt;=17.5, ROUND(Q79*0.2*W79*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U79" s="18">
@@ -10675,11 +10675,11 @@
         <v/>
       </c>
       <c r="AA79" s="18">
-        <f>IF(Y79="", 0, IF(Y79&gt;J79, (Y79-J79)*2700000, 0))</f>
+        <f>IF(Y79="", 0, IF(Y79&gt;J79, (Y79-J79)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB79" s="18">
-        <f>IF(Y79="", 0, IF(J79&gt;Y79, (J79-Y79)*6000000, 0))</f>
+        <f>IF(Y79="", 0, IF(J79&gt;Y79, (J79-Y79)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC79" s="18">
@@ -10691,11 +10691,11 @@
         <v/>
       </c>
       <c r="AE79" s="18">
-        <f>IF(O79&gt;J79, (O79-J79)*2700000, 0)</f>
+        <f>IF(O79&gt;J79, (O79-J79)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF79" s="18">
-        <f>IF(J79&gt;O79, (J79-O79)*6000000, 0)</f>
+        <f>IF(J79&gt;O79, (J79-O79)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG79" s="18">
@@ -10749,7 +10749,7 @@
         <v/>
       </c>
       <c r="M80" s="19" t="n">
-        <v>166.5</v>
+        <v>172</v>
       </c>
       <c r="N80" s="19">
         <f>M80*IF(F80=1, 0.85, 0.8)</f>
@@ -10776,7 +10776,7 @@
         <v/>
       </c>
       <c r="T80" s="18">
-        <f>IF(C80&gt;=17.5, Q80*0.2*W80, 0)</f>
+        <f>IF(C80&gt;=17.5, ROUND(Q80*0.2*W80*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U80" s="18">
@@ -10803,11 +10803,11 @@
         <v/>
       </c>
       <c r="AA80" s="18">
-        <f>IF(Y80="", 0, IF(Y80&gt;J80, (Y80-J80)*2700000, 0))</f>
+        <f>IF(Y80="", 0, IF(Y80&gt;J80, (Y80-J80)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB80" s="18">
-        <f>IF(Y80="", 0, IF(J80&gt;Y80, (J80-Y80)*6000000, 0))</f>
+        <f>IF(Y80="", 0, IF(J80&gt;Y80, (J80-Y80)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC80" s="18">
@@ -10819,11 +10819,11 @@
         <v/>
       </c>
       <c r="AE80" s="18">
-        <f>IF(O80&gt;J80, (O80-J80)*2700000, 0)</f>
+        <f>IF(O80&gt;J80, (O80-J80)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF80" s="18">
-        <f>IF(J80&gt;O80, (J80-O80)*6000000, 0)</f>
+        <f>IF(J80&gt;O80, (J80-O80)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG80" s="18">
@@ -10877,7 +10877,7 @@
         <v/>
       </c>
       <c r="M81" s="19" t="n">
-        <v>135.4</v>
+        <v>141</v>
       </c>
       <c r="N81" s="19">
         <f>M81*IF(F81=1, 0.85, 0.8)</f>
@@ -10904,7 +10904,7 @@
         <v/>
       </c>
       <c r="T81" s="18">
-        <f>IF(C81&gt;=17.5, Q81*0.2*W81, 0)</f>
+        <f>IF(C81&gt;=17.5, ROUND(Q81*0.2*W81*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U81" s="18">
@@ -10931,11 +10931,11 @@
         <v/>
       </c>
       <c r="AA81" s="18">
-        <f>IF(Y81="", 0, IF(Y81&gt;J81, (Y81-J81)*2700000, 0))</f>
+        <f>IF(Y81="", 0, IF(Y81&gt;J81, (Y81-J81)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB81" s="18">
-        <f>IF(Y81="", 0, IF(J81&gt;Y81, (J81-Y81)*6000000, 0))</f>
+        <f>IF(Y81="", 0, IF(J81&gt;Y81, (J81-Y81)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC81" s="18">
@@ -10947,11 +10947,11 @@
         <v/>
       </c>
       <c r="AE81" s="18">
-        <f>IF(O81&gt;J81, (O81-J81)*2700000, 0)</f>
+        <f>IF(O81&gt;J81, (O81-J81)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF81" s="18">
-        <f>IF(J81&gt;O81, (J81-O81)*6000000, 0)</f>
+        <f>IF(J81&gt;O81, (J81-O81)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG81" s="18">
@@ -11005,7 +11005,7 @@
         <v/>
       </c>
       <c r="M82" s="19" t="n">
-        <v>59.6</v>
+        <v>70</v>
       </c>
       <c r="N82" s="19">
         <f>M82*IF(F82=1, 0.85, 0.8)</f>
@@ -11032,7 +11032,7 @@
         <v/>
       </c>
       <c r="T82" s="18">
-        <f>IF(C82&gt;=17.5, Q82*0.2*W82, 0)</f>
+        <f>IF(C82&gt;=17.5, ROUND(Q82*0.2*W82*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U82" s="18">
@@ -11059,11 +11059,11 @@
         <v/>
       </c>
       <c r="AA82" s="18">
-        <f>IF(Y82="", 0, IF(Y82&gt;J82, (Y82-J82)*2700000, 0))</f>
+        <f>IF(Y82="", 0, IF(Y82&gt;J82, (Y82-J82)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB82" s="18">
-        <f>IF(Y82="", 0, IF(J82&gt;Y82, (J82-Y82)*6000000, 0))</f>
+        <f>IF(Y82="", 0, IF(J82&gt;Y82, (J82-Y82)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC82" s="18">
@@ -11075,11 +11075,11 @@
         <v/>
       </c>
       <c r="AE82" s="18">
-        <f>IF(O82&gt;J82, (O82-J82)*2700000, 0)</f>
+        <f>IF(O82&gt;J82, (O82-J82)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF82" s="18">
-        <f>IF(J82&gt;O82, (J82-O82)*6000000, 0)</f>
+        <f>IF(J82&gt;O82, (J82-O82)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG82" s="18">
@@ -11133,7 +11133,7 @@
         <v/>
       </c>
       <c r="M83" s="19" t="n">
-        <v>103</v>
+        <v>110.2</v>
       </c>
       <c r="N83" s="19">
         <f>M83*IF(F83=1, 0.85, 0.8)</f>
@@ -11160,7 +11160,7 @@
         <v/>
       </c>
       <c r="T83" s="18">
-        <f>IF(C83&gt;=17.5, Q83*0.2*W83, 0)</f>
+        <f>IF(C83&gt;=17.5, ROUND(Q83*0.2*W83*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U83" s="18">
@@ -11187,11 +11187,11 @@
         <v/>
       </c>
       <c r="AA83" s="18">
-        <f>IF(Y83="", 0, IF(Y83&gt;J83, (Y83-J83)*2700000, 0))</f>
+        <f>IF(Y83="", 0, IF(Y83&gt;J83, (Y83-J83)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB83" s="18">
-        <f>IF(Y83="", 0, IF(J83&gt;Y83, (J83-Y83)*6000000, 0))</f>
+        <f>IF(Y83="", 0, IF(J83&gt;Y83, (J83-Y83)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC83" s="18">
@@ -11203,11 +11203,11 @@
         <v/>
       </c>
       <c r="AE83" s="18">
-        <f>IF(O83&gt;J83, (O83-J83)*2700000, 0)</f>
+        <f>IF(O83&gt;J83, (O83-J83)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF83" s="18">
-        <f>IF(J83&gt;O83, (J83-O83)*6000000, 0)</f>
+        <f>IF(J83&gt;O83, (J83-O83)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG83" s="18">
@@ -11261,7 +11261,7 @@
         <v/>
       </c>
       <c r="M84" s="19" t="n">
-        <v>29.4</v>
+        <v>43.8</v>
       </c>
       <c r="N84" s="19">
         <f>M84*IF(F84=1, 0.85, 0.8)</f>
@@ -11288,7 +11288,7 @@
         <v/>
       </c>
       <c r="T84" s="18">
-        <f>IF(C84&gt;=17.5, Q84*0.2*W84, 0)</f>
+        <f>IF(C84&gt;=17.5, ROUND(Q84*0.2*W84*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U84" s="18">
@@ -11315,11 +11315,11 @@
         <v/>
       </c>
       <c r="AA84" s="18">
-        <f>IF(Y84="", 0, IF(Y84&gt;J84, (Y84-J84)*2700000, 0))</f>
+        <f>IF(Y84="", 0, IF(Y84&gt;J84, (Y84-J84)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB84" s="18">
-        <f>IF(Y84="", 0, IF(J84&gt;Y84, (J84-Y84)*6000000, 0))</f>
+        <f>IF(Y84="", 0, IF(J84&gt;Y84, (J84-Y84)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC84" s="18">
@@ -11331,11 +11331,11 @@
         <v/>
       </c>
       <c r="AE84" s="18">
-        <f>IF(O84&gt;J84, (O84-J84)*2700000, 0)</f>
+        <f>IF(O84&gt;J84, (O84-J84)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF84" s="18">
-        <f>IF(J84&gt;O84, (J84-O84)*6000000, 0)</f>
+        <f>IF(J84&gt;O84, (J84-O84)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG84" s="18">
@@ -11389,7 +11389,7 @@
         <v/>
       </c>
       <c r="M85" s="19" t="n">
-        <v>85.7</v>
+        <v>95.2</v>
       </c>
       <c r="N85" s="19">
         <f>M85*IF(F85=1, 0.85, 0.8)</f>
@@ -11416,7 +11416,7 @@
         <v/>
       </c>
       <c r="T85" s="18">
-        <f>IF(C85&gt;=17.5, Q85*0.2*W85, 0)</f>
+        <f>IF(C85&gt;=17.5, ROUND(Q85*0.2*W85*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U85" s="18">
@@ -11443,11 +11443,11 @@
         <v/>
       </c>
       <c r="AA85" s="18">
-        <f>IF(Y85="", 0, IF(Y85&gt;J85, (Y85-J85)*2700000, 0))</f>
+        <f>IF(Y85="", 0, IF(Y85&gt;J85, (Y85-J85)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB85" s="18">
-        <f>IF(Y85="", 0, IF(J85&gt;Y85, (J85-Y85)*6000000, 0))</f>
+        <f>IF(Y85="", 0, IF(J85&gt;Y85, (J85-Y85)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC85" s="18">
@@ -11459,11 +11459,11 @@
         <v/>
       </c>
       <c r="AE85" s="18">
-        <f>IF(O85&gt;J85, (O85-J85)*2700000, 0)</f>
+        <f>IF(O85&gt;J85, (O85-J85)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF85" s="18">
-        <f>IF(J85&gt;O85, (J85-O85)*6000000, 0)</f>
+        <f>IF(J85&gt;O85, (J85-O85)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG85" s="18">
@@ -11517,7 +11517,7 @@
         <v/>
       </c>
       <c r="M86" s="19" t="n">
-        <v>113.8</v>
+        <v>118.3</v>
       </c>
       <c r="N86" s="19">
         <f>M86*IF(F86=1, 0.85, 0.8)</f>
@@ -11544,7 +11544,7 @@
         <v/>
       </c>
       <c r="T86" s="18">
-        <f>IF(C86&gt;=17.5, Q86*0.2*W86, 0)</f>
+        <f>IF(C86&gt;=17.5, ROUND(Q86*0.2*W86*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U86" s="18">
@@ -11571,11 +11571,11 @@
         <v/>
       </c>
       <c r="AA86" s="18">
-        <f>IF(Y86="", 0, IF(Y86&gt;J86, (Y86-J86)*2700000, 0))</f>
+        <f>IF(Y86="", 0, IF(Y86&gt;J86, (Y86-J86)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB86" s="18">
-        <f>IF(Y86="", 0, IF(J86&gt;Y86, (J86-Y86)*6000000, 0))</f>
+        <f>IF(Y86="", 0, IF(J86&gt;Y86, (J86-Y86)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC86" s="18">
@@ -11587,11 +11587,11 @@
         <v/>
       </c>
       <c r="AE86" s="18">
-        <f>IF(O86&gt;J86, (O86-J86)*2700000, 0)</f>
+        <f>IF(O86&gt;J86, (O86-J86)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF86" s="18">
-        <f>IF(J86&gt;O86, (J86-O86)*6000000, 0)</f>
+        <f>IF(J86&gt;O86, (J86-O86)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG86" s="18">
@@ -11645,7 +11645,7 @@
         <v/>
       </c>
       <c r="M87" s="19" t="n">
-        <v>81.90000000000001</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="N87" s="19">
         <f>M87*IF(F87=1, 0.85, 0.8)</f>
@@ -11672,7 +11672,7 @@
         <v/>
       </c>
       <c r="T87" s="18">
-        <f>IF(C87&gt;=17.5, Q87*0.2*W87, 0)</f>
+        <f>IF(C87&gt;=17.5, ROUND(Q87*0.2*W87*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U87" s="18">
@@ -11699,11 +11699,11 @@
         <v/>
       </c>
       <c r="AA87" s="18">
-        <f>IF(Y87="", 0, IF(Y87&gt;J87, (Y87-J87)*2700000, 0))</f>
+        <f>IF(Y87="", 0, IF(Y87&gt;J87, (Y87-J87)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB87" s="18">
-        <f>IF(Y87="", 0, IF(J87&gt;Y87, (J87-Y87)*6000000, 0))</f>
+        <f>IF(Y87="", 0, IF(J87&gt;Y87, (J87-Y87)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC87" s="18">
@@ -11715,11 +11715,11 @@
         <v/>
       </c>
       <c r="AE87" s="18">
-        <f>IF(O87&gt;J87, (O87-J87)*2700000, 0)</f>
+        <f>IF(O87&gt;J87, (O87-J87)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF87" s="18">
-        <f>IF(J87&gt;O87, (J87-O87)*6000000, 0)</f>
+        <f>IF(J87&gt;O87, (J87-O87)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG87" s="18">
@@ -11773,7 +11773,7 @@
         <v/>
       </c>
       <c r="M88" s="19" t="n">
-        <v>58.5</v>
+        <v>62.8</v>
       </c>
       <c r="N88" s="19">
         <f>M88*IF(F88=1, 0.85, 0.8)</f>
@@ -11800,7 +11800,7 @@
         <v/>
       </c>
       <c r="T88" s="18">
-        <f>IF(C88&gt;=17.5, Q88*0.2*W88, 0)</f>
+        <f>IF(C88&gt;=17.5, ROUND(Q88*0.2*W88*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U88" s="18">
@@ -11827,11 +11827,11 @@
         <v/>
       </c>
       <c r="AA88" s="18">
-        <f>IF(Y88="", 0, IF(Y88&gt;J88, (Y88-J88)*2700000, 0))</f>
+        <f>IF(Y88="", 0, IF(Y88&gt;J88, (Y88-J88)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB88" s="18">
-        <f>IF(Y88="", 0, IF(J88&gt;Y88, (J88-Y88)*6000000, 0))</f>
+        <f>IF(Y88="", 0, IF(J88&gt;Y88, (J88-Y88)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC88" s="18">
@@ -11843,11 +11843,11 @@
         <v/>
       </c>
       <c r="AE88" s="18">
-        <f>IF(O88&gt;J88, (O88-J88)*2700000, 0)</f>
+        <f>IF(O88&gt;J88, (O88-J88)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF88" s="18">
-        <f>IF(J88&gt;O88, (J88-O88)*6000000, 0)</f>
+        <f>IF(J88&gt;O88, (J88-O88)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG88" s="18">
@@ -11901,7 +11901,7 @@
         <v/>
       </c>
       <c r="M89" s="19" t="n">
-        <v>50.8</v>
+        <v>56.2</v>
       </c>
       <c r="N89" s="19">
         <f>M89*IF(F89=1, 0.85, 0.8)</f>
@@ -11928,7 +11928,7 @@
         <v/>
       </c>
       <c r="T89" s="18">
-        <f>IF(C89&gt;=17.5, Q89*0.2*W89, 0)</f>
+        <f>IF(C89&gt;=17.5, ROUND(Q89*0.2*W89*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U89" s="18">
@@ -11955,11 +11955,11 @@
         <v/>
       </c>
       <c r="AA89" s="18">
-        <f>IF(Y89="", 0, IF(Y89&gt;J89, (Y89-J89)*2700000, 0))</f>
+        <f>IF(Y89="", 0, IF(Y89&gt;J89, (Y89-J89)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB89" s="18">
-        <f>IF(Y89="", 0, IF(J89&gt;Y89, (J89-Y89)*6000000, 0))</f>
+        <f>IF(Y89="", 0, IF(J89&gt;Y89, (J89-Y89)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC89" s="18">
@@ -11971,11 +11971,11 @@
         <v/>
       </c>
       <c r="AE89" s="18">
-        <f>IF(O89&gt;J89, (O89-J89)*2700000, 0)</f>
+        <f>IF(O89&gt;J89, (O89-J89)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF89" s="18">
-        <f>IF(J89&gt;O89, (J89-O89)*6000000, 0)</f>
+        <f>IF(J89&gt;O89, (J89-O89)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG89" s="18">
@@ -12029,7 +12029,7 @@
         <v/>
       </c>
       <c r="M90" s="19" t="n">
-        <v>39.1</v>
+        <v>49.2</v>
       </c>
       <c r="N90" s="19">
         <f>M90*IF(F90=1, 0.85, 0.8)</f>
@@ -12056,7 +12056,7 @@
         <v/>
       </c>
       <c r="T90" s="18">
-        <f>IF(C90&gt;=17.5, Q90*0.2*W90, 0)</f>
+        <f>IF(C90&gt;=17.5, ROUND(Q90*0.2*W90*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U90" s="18">
@@ -12083,11 +12083,11 @@
         <v/>
       </c>
       <c r="AA90" s="18">
-        <f>IF(Y90="", 0, IF(Y90&gt;J90, (Y90-J90)*2700000, 0))</f>
+        <f>IF(Y90="", 0, IF(Y90&gt;J90, (Y90-J90)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB90" s="18">
-        <f>IF(Y90="", 0, IF(J90&gt;Y90, (J90-Y90)*6000000, 0))</f>
+        <f>IF(Y90="", 0, IF(J90&gt;Y90, (J90-Y90)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC90" s="18">
@@ -12099,11 +12099,11 @@
         <v/>
       </c>
       <c r="AE90" s="18">
-        <f>IF(O90&gt;J90, (O90-J90)*2700000, 0)</f>
+        <f>IF(O90&gt;J90, (O90-J90)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF90" s="18">
-        <f>IF(J90&gt;O90, (J90-O90)*6000000, 0)</f>
+        <f>IF(J90&gt;O90, (J90-O90)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG90" s="18">
@@ -12157,7 +12157,7 @@
         <v/>
       </c>
       <c r="M91" s="19" t="n">
-        <v>5.6</v>
+        <v>17.3</v>
       </c>
       <c r="N91" s="19">
         <f>M91*IF(F91=1, 0.85, 0.8)</f>
@@ -12184,7 +12184,7 @@
         <v/>
       </c>
       <c r="T91" s="18">
-        <f>IF(C91&gt;=17.5, Q91*0.2*W91, 0)</f>
+        <f>IF(C91&gt;=17.5, ROUND(Q91*0.2*W91*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U91" s="18">
@@ -12211,11 +12211,11 @@
         <v/>
       </c>
       <c r="AA91" s="18">
-        <f>IF(Y91="", 0, IF(Y91&gt;J91, (Y91-J91)*2700000, 0))</f>
+        <f>IF(Y91="", 0, IF(Y91&gt;J91, (Y91-J91)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB91" s="18">
-        <f>IF(Y91="", 0, IF(J91&gt;Y91, (J91-Y91)*6000000, 0))</f>
+        <f>IF(Y91="", 0, IF(J91&gt;Y91, (J91-Y91)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC91" s="18">
@@ -12227,11 +12227,11 @@
         <v/>
       </c>
       <c r="AE91" s="18">
-        <f>IF(O91&gt;J91, (O91-J91)*2700000, 0)</f>
+        <f>IF(O91&gt;J91, (O91-J91)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF91" s="18">
-        <f>IF(J91&gt;O91, (J91-O91)*6000000, 0)</f>
+        <f>IF(J91&gt;O91, (J91-O91)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG91" s="18">
@@ -12285,7 +12285,7 @@
         <v/>
       </c>
       <c r="M92" s="19" t="n">
-        <v>28.3</v>
+        <v>36.9</v>
       </c>
       <c r="N92" s="19">
         <f>M92*IF(F92=1, 0.85, 0.8)</f>
@@ -12312,7 +12312,7 @@
         <v/>
       </c>
       <c r="T92" s="18">
-        <f>IF(C92&gt;=17.5, Q92*0.2*W92, 0)</f>
+        <f>IF(C92&gt;=17.5, ROUND(Q92*0.2*W92*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U92" s="18">
@@ -12339,11 +12339,11 @@
         <v/>
       </c>
       <c r="AA92" s="18">
-        <f>IF(Y92="", 0, IF(Y92&gt;J92, (Y92-J92)*2700000, 0))</f>
+        <f>IF(Y92="", 0, IF(Y92&gt;J92, (Y92-J92)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB92" s="18">
-        <f>IF(Y92="", 0, IF(J92&gt;Y92, (J92-Y92)*6000000, 0))</f>
+        <f>IF(Y92="", 0, IF(J92&gt;Y92, (J92-Y92)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC92" s="18">
@@ -12355,11 +12355,11 @@
         <v/>
       </c>
       <c r="AE92" s="18">
-        <f>IF(O92&gt;J92, (O92-J92)*2700000, 0)</f>
+        <f>IF(O92&gt;J92, (O92-J92)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF92" s="18">
-        <f>IF(J92&gt;O92, (J92-O92)*6000000, 0)</f>
+        <f>IF(J92&gt;O92, (J92-O92)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG92" s="18">
@@ -12413,7 +12413,7 @@
         <v/>
       </c>
       <c r="M93" s="19" t="n">
-        <v>32.9</v>
+        <v>40.2</v>
       </c>
       <c r="N93" s="19">
         <f>M93*IF(F93=1, 0.85, 0.8)</f>
@@ -12440,7 +12440,7 @@
         <v/>
       </c>
       <c r="T93" s="18">
-        <f>IF(C93&gt;=17.5, Q93*0.2*W93, 0)</f>
+        <f>IF(C93&gt;=17.5, ROUND(Q93*0.2*W93*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U93" s="18">
@@ -12467,11 +12467,11 @@
         <v/>
       </c>
       <c r="AA93" s="18">
-        <f>IF(Y93="", 0, IF(Y93&gt;J93, (Y93-J93)*2700000, 0))</f>
+        <f>IF(Y93="", 0, IF(Y93&gt;J93, (Y93-J93)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB93" s="18">
-        <f>IF(Y93="", 0, IF(J93&gt;Y93, (J93-Y93)*6000000, 0))</f>
+        <f>IF(Y93="", 0, IF(J93&gt;Y93, (J93-Y93)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC93" s="18">
@@ -12483,11 +12483,11 @@
         <v/>
       </c>
       <c r="AE93" s="18">
-        <f>IF(O93&gt;J93, (O93-J93)*2700000, 0)</f>
+        <f>IF(O93&gt;J93, (O93-J93)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF93" s="18">
-        <f>IF(J93&gt;O93, (J93-O93)*6000000, 0)</f>
+        <f>IF(J93&gt;O93, (J93-O93)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG93" s="18">
@@ -12541,7 +12541,7 @@
         <v/>
       </c>
       <c r="M94" s="19" t="n">
-        <v>29.7</v>
+        <v>34.6</v>
       </c>
       <c r="N94" s="19">
         <f>M94*IF(F94=1, 0.85, 0.8)</f>
@@ -12568,7 +12568,7 @@
         <v/>
       </c>
       <c r="T94" s="18">
-        <f>IF(C94&gt;=17.5, Q94*0.2*W94, 0)</f>
+        <f>IF(C94&gt;=17.5, ROUND(Q94*0.2*W94*0.9121785541, 0), 0)</f>
         <v/>
       </c>
       <c r="U94" s="18">
@@ -12595,11 +12595,11 @@
         <v/>
       </c>
       <c r="AA94" s="18">
-        <f>IF(Y94="", 0, IF(Y94&gt;J94, (Y94-J94)*2700000, 0))</f>
+        <f>IF(Y94="", 0, IF(Y94&gt;J94, (Y94-J94)*1415065.25537, 0))</f>
         <v/>
       </c>
       <c r="AB94" s="18">
-        <f>IF(Y94="", 0, IF(J94&gt;Y94, (J94-Y94)*6000000, 0))</f>
+        <f>IF(Y94="", 0, IF(J94&gt;Y94, (J94-Y94)*7312493.44383, 0))</f>
         <v/>
       </c>
       <c r="AC94" s="18">
@@ -12611,11 +12611,11 @@
         <v/>
       </c>
       <c r="AE94" s="18">
-        <f>IF(O94&gt;J94, (O94-J94)*2700000, 0)</f>
+        <f>IF(O94&gt;J94, (O94-J94)*900115.39941, 0)</f>
         <v/>
       </c>
       <c r="AF94" s="18">
-        <f>IF(J94&gt;O94, (J94-O94)*6000000, 0)</f>
+        <f>IF(J94&gt;O94, (J94-O94)*18233128.83436, 0)</f>
         <v/>
       </c>
       <c r="AG94" s="18">

</xml_diff>